<commit_message>
Add LSEG trading comps and model-vs-consensus check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SS5TWs33kf5v4j8orcJC9a
</commit_message>
<xml_diff>
--- a/projects/01-equity-pitch-kit/models/LSEG_Model.xlsx
+++ b/projects/01-equity-pitch-kit/models/LSEG_Model.xlsx
@@ -12,8 +12,10 @@
     <sheet name="Inputs" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Model" sheetId="3" state="visible" r:id="rId5"/>
     <sheet name="DCF" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Scenarios" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Sources" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Comps" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="vs Consensus" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Scenarios" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Sources" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="304" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="398" uniqueCount="290">
   <si>
     <t xml:space="preserve">London Stock Exchange Group plc (LSEG.L)</t>
   </si>
@@ -60,6 +62,12 @@
     <t xml:space="preserve">Net debt / EBITDA 2027E</t>
   </si>
   <si>
+    <t xml:space="preserve">Peer median fwd P/E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied value at peer median (p)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Balance sheet checks (sum, should be 0)</t>
   </si>
   <si>
@@ -604,6 +612,213 @@
   </si>
   <si>
     <t xml:space="preserve">Implied 2027E P/E at current price</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LSEG – Trading comparables</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prices 20–23 Oct 2026; stockanalysis.com, accessed 25 Oct 2026. Forward P/E is the primary metric (consistent consensus basis); EV/EBITDA is trailing, provider-defined.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Company</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ticker</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peer group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ccy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mkt cap (bn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV (bn)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fwd P/E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EV/EBITDA TTM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EBITDA margin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S&amp;P Global</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SPGI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data &amp; analytics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">USD</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moody's</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MCO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MSCI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FactSet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FDS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RELX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REL.L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GBP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Experian</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXPN.L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Intercontinental Exchange</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ICE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exchanges &amp; infrastructure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nasdaq</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NDAQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CME Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deutsche Börse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DB1.DE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Euronext</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ENX.PA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median – all peers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mean – all peers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Max</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Min</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median – Data &amp; analytics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Median – Exchanges &amp; infrastructure</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LSEG (same source)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LSEG discount to peer median (fwd P/E)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied LSEG value per share (p)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  LSEG price on same source (p)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  at all-peer median fwd P/E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  at data &amp; analytics median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  at exchanges median</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  at peer minimum (bear cross-check)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read: LSEG trades at a discount to both data and exchange peers, closest to FactSet – the market is pricing it as an AI-exposed terminal business, although c.half of income is Markets, FTSE Russell and Risk Intelligence.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LSEG – Model vs company-compiled consensus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Consensus: LSEG IR, compiled 13 Oct 2026 (12 analysts) – before the Octus deal and Q3 guidance upgrade. Model figures are live links.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Line</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model 2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cons 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cons 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cons 2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diff 2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diff 2027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diff 2028</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data &amp; Analytics</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FTSE Russell</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk Intelligence</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Markets</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Read: model sits close to consensus on income and EBITDA; EPS a little above (lower NCI drag, buyback timing). The variant view is in the multiple, not the numbers.</t>
   </si>
   <si>
     <t xml:space="preserve">LSEG – Scenario outputs</t>
@@ -1274,7 +1489,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -1372,7 +1587,25 @@
       <c r="A13" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="7" t="n">
+      <c r="B13" s="6" t="n">
+        <f aca="false">Comps!G17</f>
+        <v>22.45</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <f aca="false">Comps!B29</f>
+        <v>11585.1277868407</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" s="7" t="n">
         <f aca="false">SUM(Model!D68:I68)</f>
         <v>0</v>
       </c>
@@ -1404,29 +1637,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="E4" s="9" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="F4" s="9" t="n">
         <v>2026</v>
@@ -1446,7 +1679,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
@@ -1460,37 +1693,37 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>2</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E7" s="0" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C8" s="13" t="n">
         <f aca="false">CHOOSE(Inputs!$C$7,F8,G8,H8)</f>
         <v>0</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E8" s="0" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F8" s="14" t="n">
         <v>-0.025</v>
@@ -1504,20 +1737,20 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="B9" s="0" t="s">
         <v>26</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>24</v>
       </c>
       <c r="C9" s="13" t="n">
         <f aca="false">CHOOSE(Inputs!$C$7,F9,G9,H9)</f>
         <v>0</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E9" s="0" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F9" s="14" t="n">
         <v>-0.01</v>
@@ -1531,20 +1764,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C10" s="13" t="n">
         <f aca="false">CHOOSE(Inputs!$C$7,F10,G10,H10)</f>
         <v>0.03</v>
       </c>
       <c r="D10" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E10" s="0" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F10" s="14" t="n">
         <v>0.025</v>
@@ -1558,7 +1791,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -1572,58 +1805,58 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C13" s="15" t="n">
         <v>9510</v>
       </c>
       <c r="D13" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E13" s="0" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C14" s="16" t="n">
         <v>1.32</v>
       </c>
       <c r="D14" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E14" s="0" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B15" s="0" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C15" s="17" t="n">
         <v>510</v>
       </c>
       <c r="D15" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E15" s="0" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -1637,16 +1870,16 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="0" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B18" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D18" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E18" s="0" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F18" s="14" t="n">
         <v>0.04</v>
@@ -1666,16 +1899,16 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="B19" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D19" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E19" s="0" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F19" s="14" t="n">
         <v>0.085</v>
@@ -1695,16 +1928,16 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="B20" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="D20" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="E20" s="0" t="s">
         <v>43</v>
-      </c>
-      <c r="B20" s="0" t="s">
-        <v>24</v>
-      </c>
-      <c r="D20" s="0" t="s">
-        <v>21</v>
-      </c>
-      <c r="E20" s="0" t="s">
-        <v>41</v>
       </c>
       <c r="F20" s="14" t="n">
         <v>0.09</v>
@@ -1724,16 +1957,16 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="0" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B21" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D21" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E21" s="0" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F21" s="14" t="n">
         <v>0.11</v>
@@ -1753,16 +1986,16 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B22" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D22" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E22" s="0" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F22" s="14" t="n">
         <v>0</v>
@@ -1782,21 +2015,21 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="B23" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C23" s="14" t="n">
         <v>0.03</v>
       </c>
       <c r="D23" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -1810,16 +2043,16 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B26" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D26" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E26" s="0" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="F26" s="14" t="n">
         <v>0.515</v>
@@ -1839,16 +2072,16 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B27" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D27" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E27" s="0" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F27" s="14" t="n">
         <v>0.11</v>
@@ -1868,16 +2101,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B28" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D28" s="0" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="E28" s="0" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="F28" s="14" t="n">
         <v>0.095</v>
@@ -1897,38 +2130,38 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B29" s="0" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C29" s="18" t="n">
         <v>1150</v>
       </c>
       <c r="D29" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E29" s="0" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="0" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B30" s="0" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C30" s="14" t="n">
         <v>0.05</v>
       </c>
       <c r="D30" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="B32" s="11"/>
       <c r="C32" s="11"/>
@@ -1942,89 +2175,89 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="0" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B33" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C33" s="14" t="n">
         <v>0.245</v>
       </c>
       <c r="D33" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E33" s="0" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="0" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="B34" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C34" s="14" t="n">
         <v>0.129</v>
       </c>
       <c r="D34" s="0" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E34" s="0" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B35" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C35" s="14" t="n">
         <v>0.6</v>
       </c>
       <c r="D35" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="B36" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C36" s="19" t="n">
         <v>0.0255</v>
       </c>
       <c r="D36" s="0" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E36" s="0" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="B37" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C37" s="14" t="n">
         <v>0.03</v>
       </c>
       <c r="D37" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E37" s="0" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="B39" s="11"/>
       <c r="C39" s="11"/>
@@ -2038,33 +2271,33 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="0" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B40" s="0" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C40" s="14" t="n">
         <v>0.36</v>
       </c>
       <c r="D40" s="0" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E40" s="0" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="0" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="B41" s="0" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D41" s="0" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="E41" s="0" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F41" s="18" t="n">
         <v>3000</v>
@@ -2078,38 +2311,38 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B42" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C42" s="14" t="n">
         <v>0.9</v>
       </c>
       <c r="D42" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E42" s="0" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B43" s="0" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C43" s="14" t="n">
         <v>0.08</v>
       </c>
       <c r="D43" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B45" s="11"/>
       <c r="C45" s="11"/>
@@ -2123,120 +2356,120 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B46" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C46" s="18" t="n">
         <v>3535</v>
       </c>
       <c r="D46" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E46" s="0" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="0" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B47" s="0" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="C47" s="20" t="n">
         <v>2027</v>
       </c>
       <c r="D47" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E47" s="0" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B48" s="0" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C48" s="18" t="n">
         <v>310</v>
       </c>
       <c r="D48" s="0" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="E48" s="0" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B49" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C49" s="14" t="n">
         <v>0.12</v>
       </c>
       <c r="D49" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E49" s="0" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B50" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C50" s="14" t="n">
         <v>0.4</v>
       </c>
       <c r="D50" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B51" s="0" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C51" s="18" t="n">
         <v>110</v>
       </c>
       <c r="D51" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B52" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C52" s="14" t="n">
         <v>0.05</v>
       </c>
       <c r="D52" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E52" s="0" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B54" s="11"/>
       <c r="C54" s="11"/>
@@ -2250,95 +2483,95 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="0" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B55" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C55" s="14" t="n">
         <v>0.049</v>
       </c>
       <c r="D55" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E55" s="0" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B56" s="0" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="C56" s="16" t="n">
         <v>0.85</v>
       </c>
       <c r="D56" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B57" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C57" s="14" t="n">
         <v>0.05</v>
       </c>
       <c r="D57" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B58" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C58" s="14" t="n">
         <v>0.05</v>
       </c>
       <c r="D58" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B59" s="0" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C59" s="14" t="n">
         <v>0.15</v>
       </c>
       <c r="D59" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E59" s="0" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B60" s="0" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C60" s="21" t="n">
         <v>25</v>
       </c>
       <c r="D60" s="0" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E60" s="0" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>
@@ -2366,17 +2599,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="9" t="n">
@@ -2403,30 +2636,30 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C5" s="23" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D5" s="23" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="E5" s="23" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="F5" s="23" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="G5" s="23" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H5" s="23" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I5" s="23" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B7" s="11"/>
       <c r="C7" s="11"/>
@@ -2439,7 +2672,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C8" s="18" t="n">
         <v>3859</v>
@@ -2470,7 +2703,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C9" s="18" t="n">
         <v>911</v>
@@ -2501,7 +2734,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C10" s="18" t="n">
         <v>531</v>
@@ -2532,7 +2765,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C11" s="18" t="n">
         <v>3180</v>
@@ -2563,7 +2796,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C12" s="18" t="n">
         <v>13</v>
@@ -2594,7 +2827,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="25" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C13" s="26" t="n">
         <f aca="false">SUM(C8:C12)</f>
@@ -2627,7 +2860,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C14" s="24"/>
       <c r="D14" s="24"/>
@@ -2654,7 +2887,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="25" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C15" s="27" t="n">
         <f aca="false">C13</f>
@@ -2687,7 +2920,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="C16" s="13"/>
       <c r="D16" s="13" t="n">
@@ -2717,7 +2950,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C17" s="18" t="n">
         <v>364</v>
@@ -2748,7 +2981,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B19" s="11"/>
       <c r="C19" s="11"/>
@@ -2761,7 +2994,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C20" s="13"/>
       <c r="D20" s="13"/>
@@ -2788,7 +3021,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="25" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C21" s="28" t="n">
         <v>4148</v>
@@ -2819,7 +3052,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C22" s="13" t="n">
         <f aca="false">C21/C15</f>
@@ -2852,7 +3085,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="0" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C23" s="18" t="n">
         <v>983</v>
@@ -2883,7 +3116,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="25" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C24" s="26" t="n">
         <f aca="false">C21-C23</f>
@@ -2916,7 +3149,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="0" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C25" s="18" t="n">
         <v>195</v>
@@ -2947,7 +3180,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C26" s="24" t="n">
         <f aca="false">C24-C25</f>
@@ -2980,7 +3213,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C27" s="24"/>
       <c r="D27" s="24"/>
@@ -3007,7 +3240,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C28" s="24"/>
       <c r="D28" s="24"/>
@@ -3034,7 +3267,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="0" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C29" s="24"/>
       <c r="D29" s="24"/>
@@ -3061,7 +3294,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="25" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C30" s="26"/>
       <c r="D30" s="26"/>
@@ -3088,7 +3321,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="25" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C31" s="29" t="n">
         <v>363.5</v>
@@ -3119,7 +3352,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="0" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C32" s="13"/>
       <c r="D32" s="13" t="n">
@@ -3149,7 +3382,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="B34" s="11"/>
       <c r="C34" s="11"/>
@@ -3162,7 +3395,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="0" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C35" s="18" t="n">
         <v>1499</v>
@@ -3193,7 +3426,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="0" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C36" s="24"/>
       <c r="D36" s="24"/>
@@ -3220,7 +3453,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="0" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C37" s="24"/>
       <c r="D37" s="24"/>
@@ -3247,7 +3480,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="0" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="C38" s="24"/>
       <c r="D38" s="24"/>
@@ -3274,7 +3507,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="0" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C39" s="24"/>
       <c r="D39" s="24"/>
@@ -3301,7 +3534,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B41" s="11"/>
       <c r="C41" s="11"/>
@@ -3314,7 +3547,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="0" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C42" s="24"/>
       <c r="D42" s="24"/>
@@ -3341,7 +3574,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="0" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C43" s="18" t="n">
         <v>957</v>
@@ -3372,7 +3605,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="0" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C44" s="24"/>
       <c r="D44" s="24"/>
@@ -3399,7 +3632,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="0" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C45" s="24"/>
       <c r="D45" s="24"/>
@@ -3426,7 +3659,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="0" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C46" s="24"/>
       <c r="D46" s="24"/>
@@ -3453,7 +3686,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="25" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="C47" s="32" t="n">
         <v>2184</v>
@@ -3484,7 +3717,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="0" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C48" s="24"/>
       <c r="D48" s="24"/>
@@ -3511,7 +3744,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="0" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C49" s="24"/>
       <c r="D49" s="24"/>
@@ -3538,7 +3771,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="0" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="C50" s="24"/>
       <c r="D50" s="24"/>
@@ -3565,7 +3798,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="0" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C51" s="24"/>
       <c r="D51" s="24"/>
@@ -3592,7 +3825,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="0" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="C52" s="18" t="n">
         <v>1052</v>
@@ -3623,7 +3856,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="25" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C53" s="26"/>
       <c r="D53" s="26"/>
@@ -3650,7 +3883,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="10" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B55" s="11"/>
       <c r="C55" s="11"/>
@@ -3663,7 +3896,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="0" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="C56" s="33"/>
       <c r="D56" s="33"/>
@@ -3690,7 +3923,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="0" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="C57" s="35"/>
       <c r="D57" s="35"/>
@@ -3717,7 +3950,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="0" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="C58" s="33"/>
       <c r="D58" s="33"/>
@@ -3744,7 +3977,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="0" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C59" s="17" t="n">
         <v>532</v>
@@ -3775,7 +4008,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="0" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C60" s="36" t="n">
         <v>130</v>
@@ -3806,7 +4039,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="10" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B62" s="11"/>
       <c r="C62" s="11"/>
@@ -3819,7 +4052,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="0" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C63" s="24"/>
       <c r="D63" s="18" t="n">
@@ -3848,7 +4081,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="0" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C64" s="24"/>
       <c r="D64" s="18" t="n">
@@ -3877,7 +4110,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="0" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C65" s="24"/>
       <c r="D65" s="24" t="n">
@@ -3907,7 +4140,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="0" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="C66" s="24"/>
       <c r="D66" s="18" t="n">
@@ -3936,7 +4169,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="0" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="C67" s="24"/>
       <c r="D67" s="18" t="n">
@@ -3965,7 +4198,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="25" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C68" s="27"/>
       <c r="D68" s="27" t="n">
@@ -3995,7 +4228,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="0" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="C69" s="38"/>
       <c r="D69" s="38" t="n">
@@ -4025,7 +4258,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="0" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="C70" s="39"/>
       <c r="D70" s="39" t="n">
@@ -4055,7 +4288,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A72" s="10" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B72" s="11"/>
       <c r="C72" s="11"/>
@@ -4068,7 +4301,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="25" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="C73" s="27"/>
       <c r="D73" s="27"/>
@@ -4119,12 +4352,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B3" s="13" t="n">
         <f aca="false">Inputs!$C$55+Inputs!$C$56*Inputs!$C$57</f>
@@ -4133,7 +4366,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B4" s="13" t="n">
         <f aca="false">Inputs!$C$58*(1-Inputs!$C$33)</f>
@@ -4142,7 +4375,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B5" s="40" t="n">
         <f aca="false">(1-Inputs!$C$59)*B3+Inputs!$C$59*B4</f>
@@ -4151,7 +4384,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="B6" s="13" t="n">
         <f aca="false">Inputs!$C$10</f>
@@ -4160,7 +4393,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>2027</v>
@@ -4177,7 +4410,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B9" s="0" t="n">
         <v>1</v>
@@ -4194,7 +4427,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="B10" s="31" t="n">
         <f aca="false">Model!F73</f>
@@ -4215,7 +4448,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="B11" s="41" t="n">
         <f aca="false">1/(1+$B$5)^(B9-0.5)</f>
@@ -4236,7 +4469,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B12" s="24" t="n">
         <f aca="false">B10*B11</f>
@@ -4257,12 +4490,12 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="D14" s="25" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B15" s="24" t="n">
         <f aca="false">SUM(B12:E12)</f>
@@ -4286,7 +4519,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B16" s="24" t="n">
         <f aca="false">E10*(1+B6)/(B5-B6)</f>
@@ -4318,7 +4551,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="0" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B17" s="24" t="n">
         <f aca="false">B16/(1+B5)^(E9-0.5)</f>
@@ -4350,7 +4583,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="25" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B18" s="42" t="n">
         <f aca="false">B15+B17</f>
@@ -4382,7 +4615,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="0" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="B19" s="24" t="n">
         <f aca="false">-Model!E69</f>
@@ -4414,7 +4647,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="0" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="B20" s="24" t="n">
         <f aca="false">-Model!F29*Inputs!$C$60</f>
@@ -4446,7 +4679,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="25" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B21" s="42" t="n">
         <f aca="false">B18+B19+B20</f>
@@ -4455,7 +4688,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="0" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="B22" s="33" t="n">
         <f aca="false">Model!E58</f>
@@ -4464,7 +4697,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="25" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B23" s="43" t="n">
         <f aca="false">B21/B22*100</f>
@@ -4473,7 +4706,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="0" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B24" s="35" t="n">
         <f aca="false">Inputs!$C$13</f>
@@ -4491,7 +4724,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="0" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B26" s="13" t="n">
         <f aca="false">B17/B18</f>
@@ -4500,7 +4733,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="0" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B27" s="39" t="n">
         <f aca="false">B16/Model!I21</f>
@@ -4509,7 +4742,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="0" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="B28" s="39" t="n">
         <f aca="false">B24/Model!F31</f>
@@ -4532,186 +4765,547 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:I34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="5" style="0" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="9"/>
+      <c r="A4" s="9" t="s">
+        <v>197</v>
+      </c>
       <c r="B4" s="9" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="C4" s="9" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="D4" s="9" t="s">
-        <v>197</v>
+        <v>200</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>203</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>204</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>205</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>198</v>
-      </c>
-      <c r="B5" s="13" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D5" s="13" t="n">
-        <v>0.25</v>
+        <v>206</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>207</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>130.54</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>142.16</v>
+      </c>
+      <c r="G5" s="21" t="n">
+        <v>23.99</v>
+      </c>
+      <c r="H5" s="21" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>0.5051</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>199</v>
-      </c>
-      <c r="B6" s="13" t="n">
-        <v>-0.025</v>
-      </c>
-      <c r="C6" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D6" s="13" t="n">
-        <v>0.015</v>
+        <v>210</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>211</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>89.36</v>
+      </c>
+      <c r="G6" s="21" t="n">
+        <v>26.83</v>
+      </c>
+      <c r="H6" s="21" t="n">
+        <v>22.07</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>0.4952</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>200</v>
-      </c>
-      <c r="B7" s="13" t="n">
-        <v>-0.01</v>
-      </c>
-      <c r="C7" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="13" t="n">
-        <v>0.006</v>
+        <v>212</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>212</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>44.02</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>50.65</v>
+      </c>
+      <c r="G7" s="21" t="n">
+        <v>28.41</v>
+      </c>
+      <c r="H7" s="21" t="n">
+        <v>25.09</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>0.5881</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>27</v>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="C8" s="13" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="D8" s="13" t="n">
-        <v>0.035</v>
+        <v>213</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>214</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="G8" s="21" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="H8" s="21" t="n">
+        <v>14.39</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>0.3636</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>201</v>
-      </c>
-      <c r="B9" s="24" t="n">
-        <v>10467.4754177689</v>
-      </c>
-      <c r="C9" s="24" t="n">
-        <v>11216.4896758939</v>
-      </c>
-      <c r="D9" s="24" t="n">
-        <v>11683.0887317689</v>
+        <v>215</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>216</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>61.57</v>
+      </c>
+      <c r="G9" s="21" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="H9" s="21" t="n">
+        <v>18.26</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>0.3387</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>202</v>
-      </c>
-      <c r="B10" s="13" t="n">
-        <v>0.514679038310472</v>
-      </c>
-      <c r="C10" s="13" t="n">
-        <v>0.524638161730451</v>
-      </c>
-      <c r="D10" s="13" t="n">
-        <v>0.530621134292044</v>
+        <v>218</v>
+      </c>
+      <c r="B10" s="0" t="s">
+        <v>219</v>
+      </c>
+      <c r="C10" s="0" t="s">
+        <v>208</v>
+      </c>
+      <c r="D10" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>26.78</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>30.79</v>
+      </c>
+      <c r="G10" s="21" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="H10" s="21" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>0.3008</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>203</v>
-      </c>
-      <c r="B11" s="37" t="n">
-        <v>562.730346965614</v>
-      </c>
-      <c r="C11" s="37" t="n">
-        <v>624.460890711389</v>
-      </c>
-      <c r="D11" s="37" t="n">
-        <v>663.74034321464</v>
+        <v>220</v>
+      </c>
+      <c r="B11" s="0" t="s">
+        <v>221</v>
+      </c>
+      <c r="C11" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="D11" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>91.36</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>110.82</v>
+      </c>
+      <c r="G11" s="21" t="n">
+        <v>19.58</v>
+      </c>
+      <c r="H11" s="21" t="n">
+        <v>16.51</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>0.6359</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>204</v>
-      </c>
-      <c r="B12" s="35" t="n">
-        <v>8315.66262743206</v>
-      </c>
-      <c r="C12" s="35" t="n">
-        <v>10989.3165729073</v>
-      </c>
-      <c r="D12" s="35" t="n">
-        <v>13568.0909038087</v>
+        <v>223</v>
+      </c>
+      <c r="B12" s="0" t="s">
+        <v>224</v>
+      </c>
+      <c r="C12" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="D12" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>57.33</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>66.03</v>
+      </c>
+      <c r="G12" s="21" t="n">
+        <v>22.45</v>
+      </c>
+      <c r="H12" s="21" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>0.6036</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" s="13" t="n">
-        <v>-0.12558752603238</v>
-      </c>
-      <c r="C13" s="13" t="n">
-        <v>0.155553793155339</v>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>0.426718286415212</v>
+        <v>225</v>
+      </c>
+      <c r="B13" s="0" t="s">
+        <v>226</v>
+      </c>
+      <c r="C13" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="D13" s="0" t="s">
+        <v>209</v>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>109.42</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>110.95</v>
+      </c>
+      <c r="G13" s="21" t="n">
+        <v>23.62</v>
+      </c>
+      <c r="H13" s="21" t="n">
+        <v>22.46</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>0.7103</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>227</v>
+      </c>
+      <c r="B14" s="0" t="s">
+        <v>228</v>
+      </c>
+      <c r="C14" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="D14" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>60.39</v>
+      </c>
+      <c r="G14" s="21" t="n">
+        <v>23.49</v>
+      </c>
+      <c r="H14" s="21" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="I14" s="14" t="n">
+        <v>0.4319</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="B15" s="43" t="n">
-        <f aca="false">SUMPRODUCT(B5:D5,B12:D12)</f>
-        <v>10965.5966692638</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>205</v>
-      </c>
-      <c r="B16" s="13" t="n">
-        <f aca="false">B15/Inputs!$C$13-1</f>
-        <v>0.153059586673377</v>
+      <c r="A15" s="0" t="s">
+        <v>230</v>
+      </c>
+      <c r="B15" s="0" t="s">
+        <v>231</v>
+      </c>
+      <c r="C15" s="0" t="s">
+        <v>222</v>
+      </c>
+      <c r="D15" s="0" t="s">
+        <v>229</v>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>19.55</v>
+      </c>
+      <c r="G15" s="21" t="n">
+        <v>18.93</v>
+      </c>
+      <c r="H15" s="21" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>0.5906</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="25" t="s">
+        <v>232</v>
+      </c>
+      <c r="G17" s="39" t="n">
+        <f aca="false">MEDIAN(G5:G15)</f>
+        <v>22.45</v>
+      </c>
+      <c r="H17" s="39" t="n">
+        <f aca="false">MEDIAN(H5:H15)</f>
+        <v>17.5</v>
+      </c>
+      <c r="I17" s="13" t="n">
+        <f aca="false">MEDIAN(I5:I15)</f>
+        <v>0.5051</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
-        <v>206</v>
+      <c r="A18" s="25" t="s">
+        <v>233</v>
+      </c>
+      <c r="G18" s="39" t="n">
+        <f aca="false">AVERAGE(G5:G15)</f>
+        <v>22.2727272727273</v>
+      </c>
+      <c r="H18" s="39" t="n">
+        <f aca="false">AVERAGE(H5:H15)</f>
+        <v>18.5536363636364</v>
+      </c>
+      <c r="I18" s="13" t="n">
+        <f aca="false">AVERAGE(I5:I15)</f>
+        <v>0.5058</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
-        <v>207</v>
+      <c r="A19" s="25" t="s">
+        <v>234</v>
+      </c>
+      <c r="G19" s="39" t="n">
+        <f aca="false">MAX(G5:G15)</f>
+        <v>28.41</v>
+      </c>
+      <c r="H19" s="39" t="n">
+        <f aca="false">MAX(H5:H15)</f>
+        <v>25.09</v>
+      </c>
+      <c r="I19" s="13" t="n">
+        <f aca="false">MAX(I5:I15)</f>
+        <v>0.7103</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="G20" s="39" t="n">
+        <f aca="false">MIN(G5:G15)</f>
+        <v>16.89</v>
+      </c>
+      <c r="H20" s="39" t="n">
+        <f aca="false">MIN(H5:H15)</f>
+        <v>14.39</v>
+      </c>
+      <c r="I20" s="13" t="n">
+        <f aca="false">MIN(I5:I15)</f>
+        <v>0.3008</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="25" t="s">
+        <v>236</v>
+      </c>
+      <c r="G21" s="39" t="n">
+        <f aca="false">MEDIAN(G5:G10)</f>
+        <v>22.235</v>
+      </c>
+      <c r="H21" s="39" t="n">
+        <f aca="false">MEDIAN(H5:H10)</f>
+        <v>17.86</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="G22" s="39" t="n">
+        <f aca="false">MEDIAN(G11:G15)</f>
+        <v>22.45</v>
+      </c>
+      <c r="H22" s="39" t="n">
+        <f aca="false">MEDIAN(H11:H15)</f>
+        <v>17.5</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="25" t="s">
+        <v>238</v>
+      </c>
+      <c r="D24" s="0" t="s">
+        <v>217</v>
+      </c>
+      <c r="E24" s="17" t="n">
+        <v>45.57</v>
+      </c>
+      <c r="F24" s="17" t="n">
+        <v>57.25</v>
+      </c>
+      <c r="G24" s="21" t="n">
+        <v>18.39</v>
+      </c>
+      <c r="H24" s="21" t="n">
+        <v>17.4</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="s">
+        <v>239</v>
+      </c>
+      <c r="G25" s="13" t="n">
+        <f aca="false">G24/G17-1</f>
+        <v>-0.180846325167038</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="25" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="B28" s="15" t="n">
+        <v>9490</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="0" t="s">
+        <v>242</v>
+      </c>
+      <c r="B29" s="35" t="n">
+        <f aca="false">B28*G17/G24</f>
+        <v>11585.1277868407</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="0" t="s">
+        <v>243</v>
+      </c>
+      <c r="B30" s="35" t="n">
+        <f aca="false">B28*G21/G24</f>
+        <v>11474.1789015769</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="0" t="s">
+        <v>244</v>
+      </c>
+      <c r="B31" s="35" t="n">
+        <f aca="false">B28*G22/G24</f>
+        <v>11585.1277868407</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="0" t="s">
+        <v>245</v>
+      </c>
+      <c r="B32" s="35" t="n">
+        <f aca="false">B28*G20/G24</f>
+        <v>8715.93800978793</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="0" t="s">
+        <v>246</v>
       </c>
     </row>
   </sheetData>
@@ -4730,6 +5324,578 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:J14"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="2" style="0" width="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="H4" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="I4" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="J4" s="9" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>259</v>
+      </c>
+      <c r="B5" s="31" t="n">
+        <f aca="false">Model!E8</f>
+        <v>4137.12</v>
+      </c>
+      <c r="C5" s="31" t="n">
+        <f aca="false">Model!F8</f>
+        <v>4343.976</v>
+      </c>
+      <c r="D5" s="31" t="n">
+        <f aca="false">Model!G8</f>
+        <v>4582.89468</v>
+      </c>
+      <c r="E5" s="18" t="n">
+        <v>4143</v>
+      </c>
+      <c r="F5" s="18" t="n">
+        <v>4394</v>
+      </c>
+      <c r="G5" s="18" t="n">
+        <v>4649</v>
+      </c>
+      <c r="H5" s="13" t="n">
+        <f aca="false">B5/E5-1</f>
+        <v>-0.00141926140477922</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <f aca="false">C5/F5-1</f>
+        <v>-0.0113846153846154</v>
+      </c>
+      <c r="J5" s="13" t="n">
+        <f aca="false">D5/G5-1</f>
+        <v>-0.0142192557539257</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>260</v>
+      </c>
+      <c r="B6" s="31" t="n">
+        <f aca="false">Model!E9</f>
+        <v>1035.09</v>
+      </c>
+      <c r="C6" s="31" t="n">
+        <f aca="false">Model!F9</f>
+        <v>1123.07265</v>
+      </c>
+      <c r="D6" s="31" t="n">
+        <f aca="false">Model!G9</f>
+        <v>1212.918462</v>
+      </c>
+      <c r="E6" s="18" t="n">
+        <v>1035</v>
+      </c>
+      <c r="F6" s="18" t="n">
+        <v>1130</v>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>1226</v>
+      </c>
+      <c r="H6" s="13" t="n">
+        <f aca="false">B6/E6-1</f>
+        <v>8.69565217389567E-005</v>
+      </c>
+      <c r="I6" s="13" t="n">
+        <f aca="false">C6/F6-1</f>
+        <v>-0.00613039823008865</v>
+      </c>
+      <c r="J6" s="13" t="n">
+        <f aca="false">D6/G6-1</f>
+        <v>-0.010670096247961</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>261</v>
+      </c>
+      <c r="B7" s="31" t="n">
+        <f aca="false">Model!E10</f>
+        <v>631.11</v>
+      </c>
+      <c r="C7" s="31" t="n">
+        <f aca="false">Model!F10</f>
+        <v>691.06545</v>
+      </c>
+      <c r="D7" s="31" t="n">
+        <f aca="false">Model!G10</f>
+        <v>753.2613405</v>
+      </c>
+      <c r="E7" s="18" t="n">
+        <v>632</v>
+      </c>
+      <c r="F7" s="18" t="n">
+        <v>701</v>
+      </c>
+      <c r="G7" s="18" t="n">
+        <v>775</v>
+      </c>
+      <c r="H7" s="13" t="n">
+        <f aca="false">B7/E7-1</f>
+        <v>-0.00140822784810124</v>
+      </c>
+      <c r="I7" s="13" t="n">
+        <f aca="false">C7/F7-1</f>
+        <v>-0.0141719686162626</v>
+      </c>
+      <c r="J7" s="13" t="n">
+        <f aca="false">D7/G7-1</f>
+        <v>-0.0280498832258065</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>262</v>
+      </c>
+      <c r="B8" s="31" t="n">
+        <f aca="false">Model!E11</f>
+        <v>3848.37</v>
+      </c>
+      <c r="C8" s="31" t="n">
+        <f aca="false">Model!F11</f>
+        <v>4117.7559</v>
+      </c>
+      <c r="D8" s="31" t="n">
+        <f aca="false">Model!G11</f>
+        <v>4364.821254</v>
+      </c>
+      <c r="E8" s="18" t="n">
+        <v>3804</v>
+      </c>
+      <c r="F8" s="18" t="n">
+        <v>4091</v>
+      </c>
+      <c r="G8" s="18" t="n">
+        <v>4380</v>
+      </c>
+      <c r="H8" s="13" t="n">
+        <f aca="false">B8/E8-1</f>
+        <v>0.0116640378548898</v>
+      </c>
+      <c r="I8" s="13" t="n">
+        <f aca="false">C8/F8-1</f>
+        <v>0.00654018577364979</v>
+      </c>
+      <c r="J8" s="13" t="n">
+        <f aca="false">D8/G8-1</f>
+        <v>-0.00346546712328732</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>122</v>
+      </c>
+      <c r="B9" s="31" t="n">
+        <f aca="false">Model!E15</f>
+        <v>9659.69</v>
+      </c>
+      <c r="C9" s="31" t="n">
+        <f aca="false">Model!F15</f>
+        <v>10546.9003030303</v>
+      </c>
+      <c r="D9" s="31" t="n">
+        <f aca="false">Model!G15</f>
+        <v>11216.4896758939</v>
+      </c>
+      <c r="E9" s="18" t="n">
+        <v>9622</v>
+      </c>
+      <c r="F9" s="18" t="n">
+        <v>10324</v>
+      </c>
+      <c r="G9" s="18" t="n">
+        <v>11038</v>
+      </c>
+      <c r="H9" s="13" t="n">
+        <f aca="false">B9/E9-1</f>
+        <v>0.00391706505923928</v>
+      </c>
+      <c r="I9" s="13" t="n">
+        <f aca="false">C9/F9-1</f>
+        <v>0.0215904981625634</v>
+      </c>
+      <c r="J9" s="13" t="n">
+        <f aca="false">D9/G9-1</f>
+        <v>0.0161704725397662</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" s="31" t="n">
+        <f aca="false">Model!E21</f>
+        <v>4974.74035</v>
+      </c>
+      <c r="C10" s="31" t="n">
+        <f aca="false">Model!F21</f>
+        <v>5473.39226121212</v>
+      </c>
+      <c r="D10" s="31" t="n">
+        <f aca="false">Model!G21</f>
+        <v>5884.59852462958</v>
+      </c>
+      <c r="E10" s="18" t="n">
+        <v>4972</v>
+      </c>
+      <c r="F10" s="18" t="n">
+        <v>5388</v>
+      </c>
+      <c r="G10" s="18" t="n">
+        <v>5821</v>
+      </c>
+      <c r="H10" s="13" t="n">
+        <f aca="false">B10/E10-1</f>
+        <v>0.000551156476267023</v>
+      </c>
+      <c r="I10" s="13" t="n">
+        <f aca="false">C10/F10-1</f>
+        <v>0.0158486008188792</v>
+      </c>
+      <c r="J10" s="13" t="n">
+        <f aca="false">D10/G10-1</f>
+        <v>0.0109257042826967</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>137</v>
+      </c>
+      <c r="B11" s="5" t="n">
+        <f aca="false">Model!E31</f>
+        <v>493.588598717251</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <f aca="false">Model!F31</f>
+        <v>562.623490935893</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <f aca="false">Model!G31</f>
+        <v>624.460890711389</v>
+      </c>
+      <c r="E11" s="36" t="n">
+        <v>480.6</v>
+      </c>
+      <c r="F11" s="36" t="n">
+        <v>550.9</v>
+      </c>
+      <c r="G11" s="36" t="n">
+        <v>615.5</v>
+      </c>
+      <c r="H11" s="13" t="n">
+        <f aca="false">B11/E11-1</f>
+        <v>0.0270257984129241</v>
+      </c>
+      <c r="I11" s="13" t="n">
+        <f aca="false">C11/F11-1</f>
+        <v>0.0212806152403213</v>
+      </c>
+      <c r="J11" s="13" t="n">
+        <f aca="false">D11/G11-1</f>
+        <v>0.014558717646449</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>162</v>
+      </c>
+      <c r="B12" s="5" t="n">
+        <f aca="false">Model!E60</f>
+        <v>172.403836337276</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <f aca="false">Model!F60</f>
+        <v>199.280546912671</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <f aca="false">Model!G60</f>
+        <v>221.095360827874</v>
+      </c>
+      <c r="E12" s="36" t="n">
+        <v>167.3</v>
+      </c>
+      <c r="F12" s="36" t="n">
+        <v>189.4</v>
+      </c>
+      <c r="G12" s="36" t="n">
+        <v>209.9</v>
+      </c>
+      <c r="H12" s="13" t="n">
+        <f aca="false">B12/E12-1</f>
+        <v>0.030507091077564</v>
+      </c>
+      <c r="I12" s="13" t="n">
+        <f aca="false">C12/F12-1</f>
+        <v>0.0521676183351143</v>
+      </c>
+      <c r="J12" s="13" t="n">
+        <f aca="false">D12/G12-1</f>
+        <v>0.0533366404377038</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="s">
+        <v>263</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D19"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="8" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="B5" s="13" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="B6" s="13" t="n">
+        <v>-0.025</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>0.015</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="B7" s="13" t="n">
+        <v>-0.01</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>0.006</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" s="13" t="n">
+        <v>0.025</v>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>0.035</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>272</v>
+      </c>
+      <c r="B9" s="24" t="n">
+        <v>10467.4754177689</v>
+      </c>
+      <c r="C9" s="24" t="n">
+        <v>11216.4896758939</v>
+      </c>
+      <c r="D9" s="24" t="n">
+        <v>11683.0887317689</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="s">
+        <v>273</v>
+      </c>
+      <c r="B10" s="13" t="n">
+        <v>0.514679038310472</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>0.524638161730451</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>0.530621134292044</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>274</v>
+      </c>
+      <c r="B11" s="37" t="n">
+        <v>562.730346965614</v>
+      </c>
+      <c r="C11" s="37" t="n">
+        <v>624.460890711389</v>
+      </c>
+      <c r="D11" s="37" t="n">
+        <v>663.74034321464</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="B12" s="35" t="n">
+        <v>8315.66262743206</v>
+      </c>
+      <c r="C12" s="35" t="n">
+        <v>10989.3165729073</v>
+      </c>
+      <c r="D12" s="35" t="n">
+        <v>13568.0909038087</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="B13" s="13" t="n">
+        <v>-0.12558752603238</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>0.155553793155339</v>
+      </c>
+      <c r="D13" s="13" t="n">
+        <v>0.426718286415212</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="43" t="n">
+        <f aca="false">SUMPRODUCT(B5:D5,B12:D12)</f>
+        <v>10965.5966692638</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="s">
+        <v>276</v>
+      </c>
+      <c r="B16" s="13" t="n">
+        <f aca="false">B15/Inputs!$C$13-1</f>
+        <v>0.153059586673377</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="s">
+        <v>278</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -4738,52 +5904,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>208</v>
+        <v>279</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>209</v>
+        <v>280</v>
       </c>
       <c r="B3" s="0" t="s">
-        <v>210</v>
+        <v>281</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>211</v>
+        <v>282</v>
       </c>
       <c r="B4" s="0" t="s">
-        <v>212</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>213</v>
+        <v>284</v>
       </c>
       <c r="B5" s="0" t="s">
-        <v>214</v>
+        <v>285</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>215</v>
+        <v>286</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>216</v>
+        <v>287</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>217</v>
+        <v>288</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>218</v>
+        <v>289</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PM-proofing: Tradeweb stub, beta box, P/E history, peak-volume normalisation, EDGAR cross-check, charts; pitch rewritten
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SS5TWs33kf5v4j8orcJC9a
</commit_message>
<xml_diff>
--- a/projects/01-equity-pitch-kit/models/LSEG_Model.xlsx
+++ b/projects/01-equity-pitch-kit/models/LSEG_Model.xlsx
@@ -14,12 +14,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Model" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vs Consensus" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse DCF" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pair trade" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stub ex-Tradeweb" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation history" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vs Consensus" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse DCF" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pair trade" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -115,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -168,6 +170,7 @@
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -243,6 +246,168 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>LSEG trailing P/E</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Valuation history'!D4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Valuation history'!$A$5:$A$62</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Valuation history'!$D$5:$D$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Valuation history'!E4</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Valuation history'!$A$5:$A$62</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Valuation history'!$E$5:$E$62</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>x</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>10</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -534,7 +699,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -686,10 +851,32 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>Stub (ex-Tradeweb) forward P/E</t>
+        </is>
+      </c>
+      <c r="B16" s="6">
+        <f>'Stub ex-Tradeweb'!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Trailing P/E vs 5y average</t>
+        </is>
+      </c>
+      <c r="B17" s="6">
+        <f>'Valuation history'!I4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>Balance sheet checks (sum, should be 0)</t>
         </is>
       </c>
-      <c r="B16" s="7">
+      <c r="B18" s="7">
         <f>SUM(Model!E53:Model!J53)</f>
         <v/>
       </c>
@@ -700,6 +887,1351 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LSEG – Trading comparables</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Prices 20–23 Oct 2026; stockanalysis.com, accessed 25 Oct 2026. Forward P/E is the primary metric; trailing EV/EBITDA uses each provider's own EBITDA definition.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Company</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Peer group</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Ccy</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Mkt cap (bn)</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>EV (bn)</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Fwd P/E</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>EV/EBITDA TTM</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>EBITDA margin</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>S&amp;P Global</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>SPGI</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Data &amp; analytics</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>130.54</v>
+      </c>
+      <c r="F5" s="17" t="n">
+        <v>142.16</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>23.99</v>
+      </c>
+      <c r="H5" s="23" t="n">
+        <v>17.46</v>
+      </c>
+      <c r="I5" s="14" t="n">
+        <v>0.5051</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Moody's</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Data &amp; analytics</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>83.36</v>
+      </c>
+      <c r="F6" s="17" t="n">
+        <v>89.36</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>26.83</v>
+      </c>
+      <c r="H6" s="23" t="n">
+        <v>22.07</v>
+      </c>
+      <c r="I6" s="14" t="n">
+        <v>0.4952</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>MSCI</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MSCI</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Data &amp; analytics</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E7" s="17" t="n">
+        <v>44.02</v>
+      </c>
+      <c r="F7" s="17" t="n">
+        <v>50.65</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <v>28.41</v>
+      </c>
+      <c r="H7" s="23" t="n">
+        <v>25.09</v>
+      </c>
+      <c r="I7" s="14" t="n">
+        <v>0.5881</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>FactSet</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>FDS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Data &amp; analytics</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E8" s="17" t="n">
+        <v>11.68</v>
+      </c>
+      <c r="F8" s="17" t="n">
+        <v>12.96</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>16.89</v>
+      </c>
+      <c r="H8" s="23" t="n">
+        <v>14.39</v>
+      </c>
+      <c r="I8" s="14" t="n">
+        <v>0.3636</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>RELX</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>REL.L</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Data &amp; analytics</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E9" s="17" t="n">
+        <v>52.87</v>
+      </c>
+      <c r="F9" s="17" t="n">
+        <v>61.57</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>20.33</v>
+      </c>
+      <c r="H9" s="23" t="n">
+        <v>18.26</v>
+      </c>
+      <c r="I9" s="14" t="n">
+        <v>0.3387</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Experian</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>EXPN.L</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Data &amp; analytics</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GBP</t>
+        </is>
+      </c>
+      <c r="E10" s="17" t="n">
+        <v>26.78</v>
+      </c>
+      <c r="F10" s="17" t="n">
+        <v>30.79</v>
+      </c>
+      <c r="G10" s="23" t="n">
+        <v>20.48</v>
+      </c>
+      <c r="H10" s="23" t="n">
+        <v>15.84</v>
+      </c>
+      <c r="I10" s="14" t="n">
+        <v>0.3008</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Intercontinental Exchange</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Exchanges &amp; infrastructure</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E11" s="17" t="n">
+        <v>91.36</v>
+      </c>
+      <c r="F11" s="17" t="n">
+        <v>110.82</v>
+      </c>
+      <c r="G11" s="23" t="n">
+        <v>19.58</v>
+      </c>
+      <c r="H11" s="23" t="n">
+        <v>16.51</v>
+      </c>
+      <c r="I11" s="14" t="n">
+        <v>0.6359</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Nasdaq</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>NDAQ</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Exchanges &amp; infrastructure</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E12" s="17" t="n">
+        <v>57.33</v>
+      </c>
+      <c r="F12" s="17" t="n">
+        <v>66.03</v>
+      </c>
+      <c r="G12" s="23" t="n">
+        <v>22.45</v>
+      </c>
+      <c r="H12" s="23" t="n">
+        <v>18.92</v>
+      </c>
+      <c r="I12" s="14" t="n">
+        <v>0.6036</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CME Group</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>CME</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Exchanges &amp; infrastructure</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="n">
+        <v>109.42</v>
+      </c>
+      <c r="F13" s="17" t="n">
+        <v>110.95</v>
+      </c>
+      <c r="G13" s="23" t="n">
+        <v>23.62</v>
+      </c>
+      <c r="H13" s="23" t="n">
+        <v>22.46</v>
+      </c>
+      <c r="I13" s="14" t="n">
+        <v>0.7103</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Deutsche Börse</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>DB1.DE</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Exchanges &amp; infrastructure</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E14" s="17" t="n">
+        <v>55.6</v>
+      </c>
+      <c r="F14" s="17" t="n">
+        <v>60.39</v>
+      </c>
+      <c r="G14" s="23" t="n">
+        <v>23.49</v>
+      </c>
+      <c r="H14" s="23" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="I14" s="14" t="n">
+        <v>0.4319</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Euronext</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>ENX.PA</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Exchanges &amp; infrastructure</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="n">
+        <v>17.71</v>
+      </c>
+      <c r="F15" s="17" t="n">
+        <v>19.55</v>
+      </c>
+      <c r="G15" s="23" t="n">
+        <v>18.93</v>
+      </c>
+      <c r="H15" s="23" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="I15" s="14" t="n">
+        <v>0.5906</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Median – all peers</t>
+        </is>
+      </c>
+      <c r="G17" s="44">
+        <f>MEDIAN(G5:G15)</f>
+        <v/>
+      </c>
+      <c r="H17" s="44">
+        <f>MEDIAN(H5:H15)</f>
+        <v/>
+      </c>
+      <c r="I17" s="13">
+        <f>MEDIAN(I5:I15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Mean</t>
+        </is>
+      </c>
+      <c r="G18" s="44">
+        <f>AVERAGE(G5:G15)</f>
+        <v/>
+      </c>
+      <c r="H18" s="44">
+        <f>AVERAGE(H5:H15)</f>
+        <v/>
+      </c>
+      <c r="I18" s="13">
+        <f>AVERAGE(I5:I15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Max</t>
+        </is>
+      </c>
+      <c r="G19" s="44">
+        <f>MAX(G5:G15)</f>
+        <v/>
+      </c>
+      <c r="H19" s="44">
+        <f>MAX(H5:H15)</f>
+        <v/>
+      </c>
+      <c r="I19" s="13">
+        <f>MAX(I5:I15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Min</t>
+        </is>
+      </c>
+      <c r="G20" s="44">
+        <f>MIN(G5:G15)</f>
+        <v/>
+      </c>
+      <c r="H20" s="44">
+        <f>MIN(H5:H15)</f>
+        <v/>
+      </c>
+      <c r="I20" s="13">
+        <f>MIN(I5:I15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="12" t="inlineStr">
+        <is>
+          <t>LSEG (same source)</t>
+        </is>
+      </c>
+      <c r="E22" s="17" t="n">
+        <v>45.57</v>
+      </c>
+      <c r="F22" s="17" t="n">
+        <v>57.25</v>
+      </c>
+      <c r="G22" s="23" t="n">
+        <v>18.39</v>
+      </c>
+      <c r="H22" s="23" t="n">
+        <v>17.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>LSEG discount to peer median (fwd P/E)</t>
+        </is>
+      </c>
+      <c r="G23" s="13">
+        <f>G22/G17-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>LSEG price on same source (p)</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="n">
+        <v>9490</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>Implied value at peer median fwd P/E (p)</t>
+        </is>
+      </c>
+      <c r="B25" s="40">
+        <f>B24*G17/G22</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
+          <t>SEC EDGAR cross-check (US peers, latest 10-K, audited GAAP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>Ticker</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>FY end</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Revenue ($m)</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Operating income ($m)</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Operating margin</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>Net income ($m)</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="inlineStr">
+        <is>
+          <t>Diluted EPS ($)</t>
+        </is>
+      </c>
+      <c r="H29" s="8" t="inlineStr">
+        <is>
+          <t>Cash ($m)</t>
+        </is>
+      </c>
+      <c r="I29" s="8" t="inlineStr">
+        <is>
+          <t>Debt ($m)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SPGI</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="n">
+        <v>15336</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <v>6478</v>
+      </c>
+      <c r="E30" s="13">
+        <f>D30/C30</f>
+        <v/>
+      </c>
+      <c r="F30" s="27" t="n">
+        <v>4471</v>
+      </c>
+      <c r="G30" s="30" t="n">
+        <v>14.66</v>
+      </c>
+      <c r="H30" s="27" t="n">
+        <v>1745</v>
+      </c>
+      <c r="I30" s="27" t="n">
+        <v>13088</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>MCO</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C31" s="27" t="n">
+        <v>7718</v>
+      </c>
+      <c r="D31" s="27" t="n">
+        <v>3351</v>
+      </c>
+      <c r="E31" s="13">
+        <f>D31/C31</f>
+        <v/>
+      </c>
+      <c r="F31" s="27" t="n">
+        <v>2459</v>
+      </c>
+      <c r="G31" s="30" t="n">
+        <v>13.67</v>
+      </c>
+      <c r="H31" s="27" t="n">
+        <v>2384</v>
+      </c>
+      <c r="I31" s="27" t="n">
+        <v>6994</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>MSCI</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="n">
+        <v>3134.459</v>
+      </c>
+      <c r="D32" s="27" t="n">
+        <v>1713.567</v>
+      </c>
+      <c r="E32" s="13">
+        <f>D32/C32</f>
+        <v/>
+      </c>
+      <c r="F32" s="27" t="n">
+        <v>1202.305</v>
+      </c>
+      <c r="G32" s="30" t="n">
+        <v>15.69</v>
+      </c>
+      <c r="H32" s="27" t="n">
+        <v>515.332</v>
+      </c>
+      <c r="I32" s="27" t="n">
+        <v>6202.286</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>FDS</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="C33" s="27" t="n">
+        <v>2476.256</v>
+      </c>
+      <c r="D33" s="27" t="n">
+        <v>699.957</v>
+      </c>
+      <c r="E33" s="13">
+        <f>D33/C33</f>
+        <v/>
+      </c>
+      <c r="F33" s="27" t="n">
+        <v>533.481</v>
+      </c>
+      <c r="G33" s="30" t="n">
+        <v>14.57</v>
+      </c>
+      <c r="H33" s="27" t="n">
+        <v>233.339</v>
+      </c>
+      <c r="I33" s="27" t="n">
+        <v>1370.022</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>ICE</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C34" s="27" t="n">
+        <v>12640</v>
+      </c>
+      <c r="D34" s="27" t="n">
+        <v>4929</v>
+      </c>
+      <c r="E34" s="13">
+        <f>D34/C34</f>
+        <v/>
+      </c>
+      <c r="F34" s="27" t="n">
+        <v>3315</v>
+      </c>
+      <c r="G34" s="30" t="n">
+        <v>5.77</v>
+      </c>
+      <c r="H34" s="27" t="n">
+        <v>837</v>
+      </c>
+      <c r="I34" s="27" t="n">
+        <v>19644</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>NDAQ</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="n">
+        <v>8262</v>
+      </c>
+      <c r="D35" s="27" t="n">
+        <v>2331</v>
+      </c>
+      <c r="E35" s="13">
+        <f>D35/C35</f>
+        <v/>
+      </c>
+      <c r="F35" s="27" t="n">
+        <v>1788</v>
+      </c>
+      <c r="G35" s="30" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="H35" s="27" t="n">
+        <v>604</v>
+      </c>
+      <c r="I35" s="27" t="n">
+        <v>9004</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>CME</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="n">
+        <v>6520.6</v>
+      </c>
+      <c r="D36" s="27" t="n">
+        <v>4229.5</v>
+      </c>
+      <c r="E36" s="13">
+        <f>D36/C36</f>
+        <v/>
+      </c>
+      <c r="F36" s="27" t="n">
+        <v>4072.2</v>
+      </c>
+      <c r="G36" s="30" t="n">
+        <v>11.16</v>
+      </c>
+      <c r="H36" s="27" t="n">
+        <v>4416.9</v>
+      </c>
+      <c r="I36" s="27" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>2025-12-31</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="n">
+        <v>2052.429</v>
+      </c>
+      <c r="D37" s="27" t="n">
+        <v>835.338</v>
+      </c>
+      <c r="E37" s="13">
+        <f>D37/C37</f>
+        <v/>
+      </c>
+      <c r="F37" s="27" t="n">
+        <v>812.792</v>
+      </c>
+      <c r="G37" s="30" t="n">
+        <v>3.78</v>
+      </c>
+      <c r="H37" s="27" t="n">
+        <v>2084.739</v>
+      </c>
+      <c r="I37" s="27" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Source: data.sec.gov XBRL company facts, refreshed weekly by GitHub Actions (common/edgar.py). D&amp;A not used: XBRL tagging differs across filers.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="32" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>LSEG – Model vs company-compiled consensus</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Consensus: LSEG IR, 13 Oct 2026 (12 analysts), before the Octus deal and Q3 upgrade. Model income shown ex-Octus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Line</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Model 2026</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Model 2027</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Model 2028</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Cons 2026</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Cons 2027</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Cons 2028</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Diff 2026</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Diff 2027</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Diff 2028</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Data &amp; Analytics</t>
+        </is>
+      </c>
+      <c r="B5" s="28">
+        <f>Divisions!F16-Divisions!F15</f>
+        <v/>
+      </c>
+      <c r="C5" s="28">
+        <f>Divisions!G16-Divisions!G15</f>
+        <v/>
+      </c>
+      <c r="D5" s="28">
+        <f>Divisions!H16-Divisions!H15</f>
+        <v/>
+      </c>
+      <c r="E5" s="19" t="n">
+        <v>4143</v>
+      </c>
+      <c r="F5" s="19" t="n">
+        <v>4394</v>
+      </c>
+      <c r="G5" s="19" t="n">
+        <v>4649</v>
+      </c>
+      <c r="H5" s="13">
+        <f>B5/E5-1</f>
+        <v/>
+      </c>
+      <c r="I5" s="13">
+        <f>C5/F5-1</f>
+        <v/>
+      </c>
+      <c r="J5" s="13">
+        <f>D5/G5-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FTSE Russell</t>
+        </is>
+      </c>
+      <c r="B6" s="28">
+        <f>Divisions!F23</f>
+        <v/>
+      </c>
+      <c r="C6" s="28">
+        <f>Divisions!G23</f>
+        <v/>
+      </c>
+      <c r="D6" s="28">
+        <f>Divisions!H23</f>
+        <v/>
+      </c>
+      <c r="E6" s="19" t="n">
+        <v>1035</v>
+      </c>
+      <c r="F6" s="19" t="n">
+        <v>1130</v>
+      </c>
+      <c r="G6" s="19" t="n">
+        <v>1226</v>
+      </c>
+      <c r="H6" s="13">
+        <f>B6/E6-1</f>
+        <v/>
+      </c>
+      <c r="I6" s="13">
+        <f>C6/F6-1</f>
+        <v/>
+      </c>
+      <c r="J6" s="13">
+        <f>D6/G6-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Risk Intelligence</t>
+        </is>
+      </c>
+      <c r="B7" s="28">
+        <f>Divisions!F27</f>
+        <v/>
+      </c>
+      <c r="C7" s="28">
+        <f>Divisions!G27</f>
+        <v/>
+      </c>
+      <c r="D7" s="28">
+        <f>Divisions!H27</f>
+        <v/>
+      </c>
+      <c r="E7" s="19" t="n">
+        <v>632</v>
+      </c>
+      <c r="F7" s="19" t="n">
+        <v>701</v>
+      </c>
+      <c r="G7" s="19" t="n">
+        <v>775</v>
+      </c>
+      <c r="H7" s="13">
+        <f>B7/E7-1</f>
+        <v/>
+      </c>
+      <c r="I7" s="13">
+        <f>C7/F7-1</f>
+        <v/>
+      </c>
+      <c r="J7" s="13">
+        <f>D7/G7-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Markets</t>
+        </is>
+      </c>
+      <c r="B8" s="28">
+        <f>Divisions!F41</f>
+        <v/>
+      </c>
+      <c r="C8" s="28">
+        <f>Divisions!G41</f>
+        <v/>
+      </c>
+      <c r="D8" s="28">
+        <f>Divisions!H41</f>
+        <v/>
+      </c>
+      <c r="E8" s="19" t="n">
+        <v>3804</v>
+      </c>
+      <c r="F8" s="19" t="n">
+        <v>4091</v>
+      </c>
+      <c r="G8" s="19" t="n">
+        <v>4380</v>
+      </c>
+      <c r="H8" s="13">
+        <f>B8/E8-1</f>
+        <v/>
+      </c>
+      <c r="I8" s="13">
+        <f>C8/F8-1</f>
+        <v/>
+      </c>
+      <c r="J8" s="13">
+        <f>D8/G8-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Total income excl. recoveries</t>
+        </is>
+      </c>
+      <c r="B9" s="28">
+        <f>Divisions!F48-Divisions!F15</f>
+        <v/>
+      </c>
+      <c r="C9" s="28">
+        <f>Divisions!G48-Divisions!G15</f>
+        <v/>
+      </c>
+      <c r="D9" s="28">
+        <f>Divisions!H48-Divisions!H15</f>
+        <v/>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>9622</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>10324</v>
+      </c>
+      <c r="G9" s="19" t="n">
+        <v>11038</v>
+      </c>
+      <c r="H9" s="13">
+        <f>B9/E9-1</f>
+        <v/>
+      </c>
+      <c r="I9" s="13">
+        <f>C9/F9-1</f>
+        <v/>
+      </c>
+      <c r="J9" s="13">
+        <f>D9/G9-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Adjusted EBITDA</t>
+        </is>
+      </c>
+      <c r="B10" s="28">
+        <f>Model!F10</f>
+        <v/>
+      </c>
+      <c r="C10" s="28">
+        <f>Model!G10</f>
+        <v/>
+      </c>
+      <c r="D10" s="28">
+        <f>Model!H10</f>
+        <v/>
+      </c>
+      <c r="E10" s="19" t="n">
+        <v>4972</v>
+      </c>
+      <c r="F10" s="19" t="n">
+        <v>5388</v>
+      </c>
+      <c r="G10" s="19" t="n">
+        <v>5821</v>
+      </c>
+      <c r="H10" s="13">
+        <f>B10/E10-1</f>
+        <v/>
+      </c>
+      <c r="I10" s="13">
+        <f>C10/F10-1</f>
+        <v/>
+      </c>
+      <c r="J10" s="13">
+        <f>D10/G10-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Adjusted EPS (p)</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>Model!F20</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>Model!G20</f>
+        <v/>
+      </c>
+      <c r="D11" s="5">
+        <f>Model!H20</f>
+        <v/>
+      </c>
+      <c r="E11" s="41" t="n">
+        <v>480.6</v>
+      </c>
+      <c r="F11" s="41" t="n">
+        <v>550.9</v>
+      </c>
+      <c r="G11" s="41" t="n">
+        <v>615.5</v>
+      </c>
+      <c r="H11" s="13">
+        <f>B11/E11-1</f>
+        <v/>
+      </c>
+      <c r="I11" s="13">
+        <f>C11/F11-1</f>
+        <v/>
+      </c>
+      <c r="J11" s="13">
+        <f>D11/G11-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>DPS (p)</t>
+        </is>
+      </c>
+      <c r="B12" s="5">
+        <f>Model!F45</f>
+        <v/>
+      </c>
+      <c r="C12" s="5">
+        <f>Model!G45</f>
+        <v/>
+      </c>
+      <c r="D12" s="5">
+        <f>Model!H45</f>
+        <v/>
+      </c>
+      <c r="E12" s="41" t="n">
+        <v>167.3</v>
+      </c>
+      <c r="F12" s="41" t="n">
+        <v>189.4</v>
+      </c>
+      <c r="G12" s="41" t="n">
+        <v>209.9</v>
+      </c>
+      <c r="H12" s="13">
+        <f>B12/E12-1</f>
+        <v/>
+      </c>
+      <c r="I12" s="13">
+        <f>C12/F12-1</f>
+        <v/>
+      </c>
+      <c r="J12" s="13">
+        <f>D12/G12-1</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -765,14 +2297,14 @@
           <t>Revenue retention</t>
         </is>
       </c>
-      <c r="B5" s="50" t="n">
+      <c r="B5" s="51" t="n">
         <v>0.928</v>
       </c>
-      <c r="C5" s="50" t="n">
-        <v>0.8975839873497693</v>
-      </c>
-      <c r="D5" s="50" t="n">
-        <v>-0.03041601265023069</v>
+      <c r="C5" s="51" t="n">
+        <v>0.9131487262864029</v>
+      </c>
+      <c r="D5" s="51" t="n">
+        <v>-0.01485127371359712</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -783,21 +2315,21 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tradeweb ADV growth (all volume drivers shift together)</t>
-        </is>
-      </c>
-      <c r="B6" s="50" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="C6" s="50" t="n">
-        <v>0.01554531610125137</v>
-      </c>
-      <c r="D6" s="50" t="n">
-        <v>-0.04445468389874863</v>
+          <t>Markets volume growth, all drivers (shown on 2028 ADV growth)</t>
+        </is>
+      </c>
+      <c r="B6" s="51" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C6" s="51" t="n">
+        <v>0.02734297461659459</v>
+      </c>
+      <c r="D6" s="51" t="n">
+        <v>-0.02265702538340542</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Volumes broadly flat for four years</t>
+          <t>Volumes shrink in real terms after a flat 2027</t>
         </is>
       </c>
     </row>
@@ -807,14 +2339,14 @@
           <t>Divisional margin change per year</t>
         </is>
       </c>
-      <c r="B7" s="50" t="n">
+      <c r="B7" s="51" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="50" t="n">
-        <v>-0.006270602924408328</v>
-      </c>
-      <c r="D7" s="50" t="n">
-        <v>-0.006270602924408328</v>
+      <c r="C7" s="51" t="n">
+        <v>-0.00319678945687564</v>
+      </c>
+      <c r="D7" s="51" t="n">
+        <v>-0.00319678945687564</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -828,14 +2360,14 @@
           <t>Terminal growth</t>
         </is>
       </c>
-      <c r="B8" s="50" t="n">
+      <c r="B8" s="51" t="n">
         <v>0.03</v>
       </c>
-      <c r="C8" s="50" t="n">
-        <v>0.02660473246727198</v>
-      </c>
-      <c r="D8" s="50" t="n">
-        <v>-0.003395267532728015</v>
+      <c r="C8" s="51" t="n">
+        <v>0.02831755048183757</v>
+      </c>
+      <c r="D8" s="51" t="n">
+        <v>-0.001682449518162425</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -856,25 +2388,25 @@
           <t>Retention (2027–2030)</t>
         </is>
       </c>
-      <c r="B12" s="50" t="n">
+      <c r="B12" s="51" t="n">
         <v>0.88</v>
       </c>
-      <c r="C12" s="50" t="n">
+      <c r="C12" s="51" t="n">
         <v>0.89</v>
       </c>
-      <c r="D12" s="50" t="n">
+      <c r="D12" s="51" t="n">
         <v>0.9</v>
       </c>
-      <c r="E12" s="50" t="n">
+      <c r="E12" s="51" t="n">
         <v>0.91</v>
       </c>
-      <c r="F12" s="50" t="n">
+      <c r="F12" s="51" t="n">
         <v>0.92</v>
       </c>
-      <c r="G12" s="50" t="n">
+      <c r="G12" s="51" t="n">
         <v>0.928</v>
       </c>
-      <c r="H12" s="50" t="n">
+      <c r="H12" s="51" t="n">
         <v>0.9350000000000001</v>
       </c>
     </row>
@@ -885,25 +2417,25 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>9109.04016255193</v>
+        <v>8737.295229161417</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>9334.62827629769</v>
+        <v>8962.883342907178</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>9566.654191958733</v>
+        <v>9194.909258568223</v>
       </c>
       <c r="E13" s="40" t="n">
-        <v>9805.241890012927</v>
+        <v>9433.496956622415</v>
       </c>
       <c r="F13" s="40" t="n">
-        <v>10050.51654392404</v>
+        <v>9678.771610533535</v>
       </c>
       <c r="G13" s="40" t="n">
-        <v>10251.63575343983</v>
+        <v>9879.890820049326</v>
       </c>
       <c r="H13" s="40" t="n">
-        <v>10431.24331983838</v>
+        <v>10059.49838644787</v>
       </c>
     </row>
   </sheetData>
@@ -911,7 +2443,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1042,13 +2574,13 @@
         </is>
       </c>
       <c r="B10" s="27" t="n">
-        <v>10381.45305307494</v>
+        <v>10184.02407456774</v>
       </c>
       <c r="C10" s="27" t="n">
-        <v>10965.62376846694</v>
+        <v>10762.38939376294</v>
       </c>
       <c r="D10" s="27" t="n">
-        <v>11251.00958594794</v>
+        <v>11043.90494711274</v>
       </c>
     </row>
     <row r="11">
@@ -1058,13 +2590,13 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>0.5118569125172872</v>
+        <v>0.5107685144213289</v>
       </c>
       <c r="C11" s="13" t="n">
-        <v>0.5200978911846079</v>
+        <v>0.5190422491971218</v>
       </c>
       <c r="D11" s="13" t="n">
-        <v>0.5244304355937279</v>
+        <v>0.5233883481598264</v>
       </c>
     </row>
     <row r="12">
@@ -1074,13 +2606,13 @@
         </is>
       </c>
       <c r="B12" s="42" t="n">
-        <v>551.6754723139632</v>
+        <v>538.2991884287204</v>
       </c>
       <c r="C12" s="42" t="n">
-        <v>599.6335336776857</v>
+        <v>585.5949087960627</v>
       </c>
       <c r="D12" s="42" t="n">
-        <v>624.1106145842509</v>
+        <v>609.6672907494376</v>
       </c>
     </row>
     <row r="13">
@@ -1090,13 +2622,13 @@
         </is>
       </c>
       <c r="B13" s="40" t="n">
-        <v>7574.902480306229</v>
+        <v>7260.703211111596</v>
       </c>
       <c r="C13" s="40" t="n">
-        <v>10251.63575343983</v>
+        <v>9879.890820049326</v>
       </c>
       <c r="D13" s="40" t="n">
-        <v>12607.51753335546</v>
+        <v>12179.62531709587</v>
       </c>
     </row>
     <row r="14">
@@ -1106,13 +2638,13 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>-0.2034802859825205</v>
+        <v>-0.2365191155508312</v>
       </c>
       <c r="C14" s="13" t="n">
-        <v>0.0779848321177532</v>
+        <v>0.03889493375913</v>
       </c>
       <c r="D14" s="13" t="n">
-        <v>0.325711622855464</v>
+        <v>0.2807176989585565</v>
       </c>
     </row>
     <row r="16">
@@ -1156,7 +2688,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1284,7 +2816,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1405,7 +2937,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -2693,16 +4225,16 @@
       <c r="E56" t="inlineStr"/>
       <c r="F56" s="18" t="n"/>
       <c r="G56" s="14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="14" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I56" s="14" t="n">
         <v>0.06</v>
       </c>
-      <c r="H56" s="14" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="I56" s="14" t="n">
-        <v>0.07000000000000001</v>
-      </c>
       <c r="J56" s="14" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
     </row>
     <row r="57">
@@ -2763,10 +4295,10 @@
       </c>
       <c r="F58" s="18" t="n"/>
       <c r="G58" s="14" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="H58" s="14" t="n">
         <v>0.05</v>
-      </c>
-      <c r="H58" s="14" t="n">
-        <v>0.06</v>
       </c>
       <c r="I58" s="14" t="n">
         <v>0.06</v>
@@ -2920,10 +4452,10 @@
       </c>
       <c r="F63" s="18" t="n"/>
       <c r="G63" s="14" t="n">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="H63" s="14" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="I63" s="14" t="n">
         <v>0.05</v>
@@ -2955,7 +4487,7 @@
       </c>
       <c r="F64" s="18" t="n"/>
       <c r="G64" s="14" t="n">
-        <v>0.04</v>
+        <v>0.02</v>
       </c>
       <c r="H64" s="14" t="n">
         <v>0.04</v>
@@ -3876,7 +5408,11 @@
           <t>A</t>
         </is>
       </c>
-      <c r="E103" t="inlineStr"/>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Conservative: above observed 0.41 and Blume 0.60. See DCF sheet for sensitivity.</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3948,25 +5484,191 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
+          <t>Beta (observed, 5y)</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C107" s="16" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>stockanalysis.com; shown for reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Beta (Blume-adjusted)</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="C108" s="16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>0.67 × observed + 0.33</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="9" t="inlineStr">
+        <is>
+          <t>Tradeweb (listed subsidiary)</t>
+        </is>
+      </c>
+      <c r="B110" s="10" t="n"/>
+      <c r="C110" s="10" t="n"/>
+      <c r="D110" s="10" t="n"/>
+      <c r="E110" s="10" t="n"/>
+      <c r="F110" s="10" t="n"/>
+      <c r="G110" s="10" t="n"/>
+      <c r="H110" s="10" t="n"/>
+      <c r="I110" s="10" t="n"/>
+      <c r="J110" s="10" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Tradeweb share price</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>$</t>
+        </is>
+      </c>
+      <c r="C111" s="16" t="n">
+        <v>121.89</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Close 22 Oct 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Tradeweb shares</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C112" s="16" t="n">
+        <v>234.03</v>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Class A+B+C+D, Tradeweb 10-Q filed 30 Jul 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
           <t>Tradeweb forward P/E</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B113" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="C107" s="23" t="n">
+      <c r="C113" s="23" t="n">
         <v>28.06</v>
       </c>
-      <c r="D107" t="inlineStr">
+      <c r="D113" t="inlineStr">
         <is>
           <t>S</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>Applied to the NCI share of earnings (market value of the minority)</t>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>stockanalysis.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>LSEG economic interest in Tradeweb</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="C114" s="14" t="n">
+        <v>0.512</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Tradeweb 10-Q, 30 Jun 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>LSEG shares outstanding</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C115" s="16" t="n">
+        <v>480.22</v>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>stockanalysis.com</t>
         </is>
       </c>
     </row>
@@ -8231,12 +9933,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8573,11 +10275,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Less: Tradeweb minority at market P/E</t>
+          <t>Less: Tradeweb minority at market value</t>
         </is>
       </c>
       <c r="B20" s="27">
-        <f>-Model!F18*Inputs!$C$107</f>
+        <f>-Inputs!$C$111*Inputs!$C$112*(1-Inputs!$C$114)/Inputs!$C$19</f>
         <v/>
       </c>
       <c r="D20" s="45">
@@ -8637,6 +10339,11 @@
         <f>B21/B22*100</f>
         <v/>
       </c>
+      <c r="D23" s="12" t="inlineStr">
+        <is>
+          <t>Beta check</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -8648,6 +10355,15 @@
         <f>Inputs!$C$18</f>
         <v/>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Observed 5y beta</t>
+        </is>
+      </c>
+      <c r="E24" s="30">
+        <f>Inputs!$C$107</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
@@ -8659,6 +10375,15 @@
         <f>B23/B24-1</f>
         <v/>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Blume-adjusted</t>
+        </is>
+      </c>
+      <c r="E25" s="30">
+        <f>Inputs!$C$108</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8670,6 +10395,15 @@
         <f>B17/B18</f>
         <v/>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Used in WACC</t>
+        </is>
+      </c>
+      <c r="E26" s="30">
+        <f>Inputs!$C$103</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8691,6 +10425,43 @@
       <c r="B28" s="44">
         <f>B24/Model!G20</f>
         <v/>
+      </c>
+      <c r="D28" s="12" t="inlineStr">
+        <is>
+          <t>DCF value (p) by beta, base case (engine snapshot)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Beta</t>
+        </is>
+      </c>
+      <c r="E29" s="30" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F29" s="30" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G29" s="30" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Value (p)</t>
+        </is>
+      </c>
+      <c r="E30" s="40" t="n">
+        <v>13292.04463500932</v>
+      </c>
+      <c r="F30" s="40" t="n">
+        <v>9879.890820049326</v>
+      </c>
+      <c r="G30" s="40" t="n">
+        <v>8414.584142436806</v>
       </c>
     </row>
   </sheetData>
@@ -9075,606 +10846,175 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LSEG – Trading comparables</t>
+          <t>LSEG excluding its Tradeweb stake</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Prices 20–23 Oct 2026; stockanalysis.com, accessed 25 Oct 2026. Forward P/E is the primary metric; trailing EV/EBITDA uses each provider's own EBITDA definition.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>Company</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>Ticker</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Peer group</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Ccy</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>Mkt cap (bn)</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>EV (bn)</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Fwd P/E</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>EV/EBITDA TTM</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>EBITDA margin</t>
+          <t>Tradeweb is listed. Remove LSEG's 51.2% stake at market value and see what the rest of the group costs, on the same forward-earnings source as the comps.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>S&amp;P Global</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>SPGI</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Data &amp; analytics</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E5" s="17" t="n">
-        <v>130.54</v>
-      </c>
-      <c r="F5" s="17" t="n">
-        <v>142.16</v>
-      </c>
-      <c r="G5" s="23" t="n">
-        <v>23.99</v>
-      </c>
-      <c r="H5" s="23" t="n">
-        <v>17.46</v>
-      </c>
-      <c r="I5" s="14" t="n">
-        <v>0.5051</v>
+          <t>LSEG market cap (£m)</t>
+        </is>
+      </c>
+      <c r="B5" s="27">
+        <f>Comps!B24*Inputs!$C$115/100</f>
+        <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Moody's</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>MCO</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Data &amp; analytics</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E6" s="17" t="n">
-        <v>83.36</v>
-      </c>
-      <c r="F6" s="17" t="n">
-        <v>89.36</v>
-      </c>
-      <c r="G6" s="23" t="n">
-        <v>26.83</v>
-      </c>
-      <c r="H6" s="23" t="n">
-        <v>22.07</v>
-      </c>
-      <c r="I6" s="14" t="n">
-        <v>0.4952</v>
+          <t>Tradeweb market cap (£m)</t>
+        </is>
+      </c>
+      <c r="B6" s="27">
+        <f>Inputs!$C$111*Inputs!$C$112/Inputs!$C$19</f>
+        <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>MSCI</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>MSCI</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Data &amp; analytics</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E7" s="17" t="n">
-        <v>44.02</v>
-      </c>
-      <c r="F7" s="17" t="n">
-        <v>50.65</v>
-      </c>
-      <c r="G7" s="23" t="n">
-        <v>28.41</v>
-      </c>
-      <c r="H7" s="23" t="n">
-        <v>25.09</v>
-      </c>
-      <c r="I7" s="14" t="n">
-        <v>0.5881</v>
+          <t>LSEG stake in Tradeweb (£m)</t>
+        </is>
+      </c>
+      <c r="B7" s="27">
+        <f>B6*Inputs!$C$114</f>
+        <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FactSet</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>FDS</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Data &amp; analytics</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E8" s="17" t="n">
-        <v>11.68</v>
-      </c>
-      <c r="F8" s="17" t="n">
-        <v>12.96</v>
-      </c>
-      <c r="G8" s="23" t="n">
-        <v>16.89</v>
-      </c>
-      <c r="H8" s="23" t="n">
-        <v>14.39</v>
-      </c>
-      <c r="I8" s="14" t="n">
-        <v>0.3636</v>
+          <t xml:space="preserve">  as % of LSEG market cap</t>
+        </is>
+      </c>
+      <c r="B8" s="13">
+        <f>B7/B5</f>
+        <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>RELX</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>REL.L</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Data &amp; analytics</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="E9" s="17" t="n">
-        <v>52.87</v>
-      </c>
-      <c r="F9" s="17" t="n">
-        <v>61.57</v>
-      </c>
-      <c r="G9" s="23" t="n">
-        <v>20.33</v>
-      </c>
-      <c r="H9" s="23" t="n">
-        <v>18.26</v>
-      </c>
-      <c r="I9" s="14" t="n">
-        <v>0.3387</v>
+          <t>Stub value: LSEG ex-Tradeweb (£m)</t>
+        </is>
+      </c>
+      <c r="B9" s="27">
+        <f>B5-B7</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Experian</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>EXPN.L</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Data &amp; analytics</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>GBP</t>
-        </is>
-      </c>
-      <c r="E10" s="17" t="n">
-        <v>26.78</v>
-      </c>
-      <c r="F10" s="17" t="n">
-        <v>30.79</v>
-      </c>
-      <c r="G10" s="23" t="n">
-        <v>20.48</v>
-      </c>
-      <c r="H10" s="23" t="n">
-        <v>15.84</v>
-      </c>
-      <c r="I10" s="14" t="n">
-        <v>0.3008</v>
+          <t>LSEG forward earnings (£m)</t>
+        </is>
+      </c>
+      <c r="B10" s="27">
+        <f>B5/Comps!G22</f>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Intercontinental Exchange</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>ICE</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Exchanges &amp; infrastructure</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E11" s="17" t="n">
-        <v>91.36</v>
-      </c>
-      <c r="F11" s="17" t="n">
-        <v>110.82</v>
-      </c>
-      <c r="G11" s="23" t="n">
-        <v>19.58</v>
-      </c>
-      <c r="H11" s="23" t="n">
-        <v>16.51</v>
-      </c>
-      <c r="I11" s="14" t="n">
-        <v>0.6359</v>
+          <t>Tradeweb forward earnings attributable to LSEG (£m)</t>
+        </is>
+      </c>
+      <c r="B11" s="27">
+        <f>B6/Inputs!$C$113*Inputs!$C$114</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Nasdaq</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>NDAQ</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Exchanges &amp; infrastructure</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E12" s="17" t="n">
-        <v>57.33</v>
-      </c>
-      <c r="F12" s="17" t="n">
-        <v>66.03</v>
-      </c>
-      <c r="G12" s="23" t="n">
-        <v>22.45</v>
-      </c>
-      <c r="H12" s="23" t="n">
-        <v>18.92</v>
-      </c>
-      <c r="I12" s="14" t="n">
-        <v>0.6036</v>
+          <t>Stub forward earnings (£m)</t>
+        </is>
+      </c>
+      <c r="B12" s="27">
+        <f>B10-B11</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>CME Group</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>CME</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Exchanges &amp; infrastructure</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E13" s="17" t="n">
-        <v>109.42</v>
-      </c>
-      <c r="F13" s="17" t="n">
-        <v>110.95</v>
-      </c>
-      <c r="G13" s="23" t="n">
-        <v>23.62</v>
-      </c>
-      <c r="H13" s="23" t="n">
-        <v>22.46</v>
-      </c>
-      <c r="I13" s="14" t="n">
-        <v>0.7103</v>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Stub forward P/E</t>
+        </is>
+      </c>
+      <c r="B13" s="50">
+        <f>B9/B12</f>
+        <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Deutsche Börse</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>DB1.DE</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>Exchanges &amp; infrastructure</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="n">
-        <v>55.6</v>
-      </c>
-      <c r="F14" s="17" t="n">
-        <v>60.39</v>
-      </c>
-      <c r="G14" s="23" t="n">
-        <v>23.49</v>
-      </c>
-      <c r="H14" s="23" t="n">
-        <v>17.5</v>
-      </c>
-      <c r="I14" s="14" t="n">
-        <v>0.4319</v>
+          <t>LSEG group forward P/E</t>
+        </is>
+      </c>
+      <c r="B14" s="44">
+        <f>Comps!G22</f>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Euronext</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>ENX.PA</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Exchanges &amp; infrastructure</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>EUR</t>
-        </is>
-      </c>
-      <c r="E15" s="17" t="n">
-        <v>17.71</v>
-      </c>
-      <c r="F15" s="17" t="n">
-        <v>19.55</v>
-      </c>
-      <c r="G15" s="23" t="n">
-        <v>18.93</v>
-      </c>
-      <c r="H15" s="23" t="n">
-        <v>15.59</v>
-      </c>
-      <c r="I15" s="14" t="n">
-        <v>0.5906</v>
+          <t>FactSet forward P/E</t>
+        </is>
+      </c>
+      <c r="B15" s="44">
+        <f>Comps!G8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Data &amp; analytics peer median</t>
+        </is>
+      </c>
+      <c r="B16" s="44">
+        <f>SOTP!K5</f>
+        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
-        <is>
-          <t>Median – all peers</t>
-        </is>
-      </c>
-      <c r="G17" s="44">
-        <f>MEDIAN(G5:G15)</f>
-        <v/>
-      </c>
-      <c r="H17" s="44">
-        <f>MEDIAN(H5:H15)</f>
-        <v/>
-      </c>
-      <c r="I17" s="13">
-        <f>MEDIAN(I5:I15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="12" t="inlineStr">
-        <is>
-          <t>Mean</t>
-        </is>
-      </c>
-      <c r="G18" s="44">
-        <f>AVERAGE(G5:G15)</f>
-        <v/>
-      </c>
-      <c r="H18" s="44">
-        <f>AVERAGE(H5:H15)</f>
-        <v/>
-      </c>
-      <c r="I18" s="13">
-        <f>AVERAGE(I5:I15)</f>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Stub discount to data &amp; analytics peers</t>
+        </is>
+      </c>
+      <c r="B17" s="13">
+        <f>B13/B16-1</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
-        <is>
-          <t>Max</t>
-        </is>
-      </c>
-      <c r="G19" s="44">
-        <f>MAX(G5:G15)</f>
-        <v/>
-      </c>
-      <c r="H19" s="44">
-        <f>MAX(H5:H15)</f>
-        <v/>
-      </c>
-      <c r="I19" s="13">
-        <f>MAX(I5:I15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>Min</t>
-        </is>
-      </c>
-      <c r="G20" s="44">
-        <f>MIN(G5:G15)</f>
-        <v/>
-      </c>
-      <c r="H20" s="44">
-        <f>MIN(H5:H15)</f>
-        <v/>
-      </c>
-      <c r="I20" s="13">
-        <f>MIN(I5:I15)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>LSEG (same source)</t>
-        </is>
-      </c>
-      <c r="E22" s="17" t="n">
-        <v>45.57</v>
-      </c>
-      <c r="F22" s="17" t="n">
-        <v>57.25</v>
-      </c>
-      <c r="G22" s="23" t="n">
-        <v>18.39</v>
-      </c>
-      <c r="H22" s="23" t="n">
-        <v>17.4</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>LSEG discount to peer median (fwd P/E)</t>
-        </is>
-      </c>
-      <c r="G23" s="13">
-        <f>G22/G17-1</f>
-        <v/>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>LSEG price on same source (p)</t>
-        </is>
-      </c>
-      <c r="B24" s="15" t="n">
-        <v>9490</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="12" t="inlineStr">
-        <is>
-          <t>Implied value at peer median fwd P/E (p)</t>
-        </is>
-      </c>
-      <c r="B25" s="40">
-        <f>B24*G17/G22</f>
-        <v/>
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Read: the rest of LSEG (Data &amp; Analytics, FTSE Russell, Risk Intelligence, LCH, equities) costs less than FactSet on forward earnings.</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -9688,399 +11028,1319 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>LSEG – Model vs company-compiled consensus</t>
+          <t>LSEG trailing P/E, Jan 2022 – Oct 2026</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Consensus: LSEG IR, 13 Oct 2026 (12 analysts), before the Octus deal and Q3 upgrade. Model income shown ex-Octus.</t>
+          <t>Month-end price ÷ LTM adjusted EPS (interpolated between reported half and full years; Dec 2026 = model). Prices: Alpha Vantage.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>Line</t>
+          <t>Month</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Model 2026</t>
+          <t>Price (p)</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>Model 2027</t>
+          <t>LTM adj EPS (p)</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>Model 2028</t>
+          <t>Trailing P/E</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Cons 2026</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>Cons 2027</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="inlineStr">
-        <is>
-          <t>Cons 2028</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>Diff 2026</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>Diff 2027</t>
-        </is>
-      </c>
-      <c r="J4" s="8" t="inlineStr">
-        <is>
-          <t>Diff 2028</t>
-        </is>
+          <t>5y average</t>
+        </is>
+      </c>
+      <c r="H4" s="12" t="inlineStr">
+        <is>
+          <t>Current</t>
+        </is>
+      </c>
+      <c r="I4" s="44">
+        <f>D62</f>
+        <v/>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Data &amp; Analytics</t>
-        </is>
-      </c>
-      <c r="B5" s="28">
-        <f>Divisions!F16-Divisions!F15</f>
-        <v/>
-      </c>
-      <c r="C5" s="28">
-        <f>Divisions!G16-Divisions!G15</f>
-        <v/>
-      </c>
-      <c r="D5" s="28">
-        <f>Divisions!H16-Divisions!H15</f>
-        <v/>
-      </c>
-      <c r="E5" s="19" t="n">
-        <v>4143</v>
-      </c>
-      <c r="F5" s="19" t="n">
-        <v>4394</v>
-      </c>
-      <c r="G5" s="19" t="n">
-        <v>4649</v>
-      </c>
-      <c r="H5" s="13">
-        <f>B5/E5-1</f>
-        <v/>
-      </c>
-      <c r="I5" s="13">
-        <f>C5/F5-1</f>
-        <v/>
-      </c>
-      <c r="J5" s="13">
-        <f>D5/G5-1</f>
+          <t>2022-01</t>
+        </is>
+      </c>
+      <c r="B5" s="40" t="n">
+        <v>7220</v>
+      </c>
+      <c r="C5" s="42" t="n">
+        <v>276.1833333333333</v>
+      </c>
+      <c r="D5" s="44">
+        <f>B5/C5</f>
+        <v/>
+      </c>
+      <c r="E5" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+      <c r="H5" s="12" t="inlineStr">
+        <is>
+          <t>5y average</t>
+        </is>
+      </c>
+      <c r="I5" s="44">
+        <f>AVERAGE(D5:D62)</f>
         <v/>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FTSE Russell</t>
-        </is>
-      </c>
-      <c r="B6" s="28">
-        <f>Divisions!F23</f>
-        <v/>
-      </c>
-      <c r="C6" s="28">
-        <f>Divisions!G23</f>
-        <v/>
-      </c>
-      <c r="D6" s="28">
-        <f>Divisions!H23</f>
-        <v/>
-      </c>
-      <c r="E6" s="19" t="n">
-        <v>1035</v>
-      </c>
-      <c r="F6" s="19" t="n">
-        <v>1130</v>
-      </c>
-      <c r="G6" s="19" t="n">
-        <v>1226</v>
-      </c>
-      <c r="H6" s="13">
-        <f>B6/E6-1</f>
-        <v/>
-      </c>
-      <c r="I6" s="13">
-        <f>C6/F6-1</f>
-        <v/>
-      </c>
-      <c r="J6" s="13">
-        <f>D6/G6-1</f>
+          <t>2022-02</t>
+        </is>
+      </c>
+      <c r="B6" s="40" t="n">
+        <v>6574</v>
+      </c>
+      <c r="C6" s="42" t="n">
+        <v>279.9666666666667</v>
+      </c>
+      <c r="D6" s="44">
+        <f>B6/C6</f>
+        <v/>
+      </c>
+      <c r="E6" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+      <c r="H6" s="12" t="inlineStr">
+        <is>
+          <t>5y low</t>
+        </is>
+      </c>
+      <c r="I6" s="44">
+        <f>MIN(D5:D62)</f>
         <v/>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Risk Intelligence</t>
-        </is>
-      </c>
-      <c r="B7" s="28">
-        <f>Divisions!F27</f>
-        <v/>
-      </c>
-      <c r="C7" s="28">
-        <f>Divisions!G27</f>
-        <v/>
-      </c>
-      <c r="D7" s="28">
-        <f>Divisions!H27</f>
-        <v/>
-      </c>
-      <c r="E7" s="19" t="n">
-        <v>632</v>
-      </c>
-      <c r="F7" s="19" t="n">
-        <v>701</v>
-      </c>
-      <c r="G7" s="19" t="n">
-        <v>775</v>
-      </c>
-      <c r="H7" s="13">
-        <f>B7/E7-1</f>
-        <v/>
-      </c>
-      <c r="I7" s="13">
-        <f>C7/F7-1</f>
-        <v/>
-      </c>
-      <c r="J7" s="13">
-        <f>D7/G7-1</f>
+          <t>2022-03</t>
+        </is>
+      </c>
+      <c r="B7" s="40" t="n">
+        <v>7966</v>
+      </c>
+      <c r="C7" s="42" t="n">
+        <v>283.75</v>
+      </c>
+      <c r="D7" s="44">
+        <f>B7/C7</f>
+        <v/>
+      </c>
+      <c r="E7" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+      <c r="H7" s="12" t="inlineStr">
+        <is>
+          <t>5y high</t>
+        </is>
+      </c>
+      <c r="I7" s="44">
+        <f>MAX(D5:D62)</f>
         <v/>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Markets</t>
-        </is>
-      </c>
-      <c r="B8" s="28">
-        <f>Divisions!F41</f>
-        <v/>
-      </c>
-      <c r="C8" s="28">
-        <f>Divisions!G41</f>
-        <v/>
-      </c>
-      <c r="D8" s="28">
-        <f>Divisions!H41</f>
-        <v/>
-      </c>
-      <c r="E8" s="19" t="n">
-        <v>3804</v>
-      </c>
-      <c r="F8" s="19" t="n">
-        <v>4091</v>
-      </c>
-      <c r="G8" s="19" t="n">
-        <v>4380</v>
-      </c>
-      <c r="H8" s="13">
-        <f>B8/E8-1</f>
-        <v/>
+          <t>2022-04</t>
+        </is>
+      </c>
+      <c r="B8" s="40" t="n">
+        <v>7916</v>
+      </c>
+      <c r="C8" s="42" t="n">
+        <v>287.5333333333333</v>
+      </c>
+      <c r="D8" s="44">
+        <f>B8/C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+      <c r="H8" s="12" t="inlineStr">
+        <is>
+          <t>Percentile of current</t>
+        </is>
       </c>
       <c r="I8" s="13">
-        <f>C8/F8-1</f>
-        <v/>
-      </c>
-      <c r="J8" s="13">
-        <f>D8/G8-1</f>
+        <f>PERCENTRANK(D5:D62,D62)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Total income excl. recoveries</t>
-        </is>
-      </c>
-      <c r="B9" s="28">
-        <f>Divisions!F48-Divisions!F15</f>
-        <v/>
-      </c>
-      <c r="C9" s="28">
-        <f>Divisions!G48-Divisions!G15</f>
-        <v/>
-      </c>
-      <c r="D9" s="28">
-        <f>Divisions!H48-Divisions!H15</f>
-        <v/>
-      </c>
-      <c r="E9" s="19" t="n">
-        <v>9622</v>
-      </c>
-      <c r="F9" s="19" t="n">
-        <v>10324</v>
-      </c>
-      <c r="G9" s="19" t="n">
-        <v>11038</v>
-      </c>
-      <c r="H9" s="13">
-        <f>B9/E9-1</f>
-        <v/>
-      </c>
-      <c r="I9" s="13">
-        <f>C9/F9-1</f>
-        <v/>
-      </c>
-      <c r="J9" s="13">
-        <f>D9/G9-1</f>
+          <t>2022-05</t>
+        </is>
+      </c>
+      <c r="B9" s="40" t="n">
+        <v>7402</v>
+      </c>
+      <c r="C9" s="42" t="n">
+        <v>291.3166666666667</v>
+      </c>
+      <c r="D9" s="44">
+        <f>B9/C9</f>
+        <v/>
+      </c>
+      <c r="E9" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Adjusted EBITDA</t>
-        </is>
-      </c>
-      <c r="B10" s="28">
-        <f>Model!F10</f>
-        <v/>
-      </c>
-      <c r="C10" s="28">
-        <f>Model!G10</f>
-        <v/>
-      </c>
-      <c r="D10" s="28">
-        <f>Model!H10</f>
-        <v/>
-      </c>
-      <c r="E10" s="19" t="n">
-        <v>4972</v>
-      </c>
-      <c r="F10" s="19" t="n">
-        <v>5388</v>
-      </c>
-      <c r="G10" s="19" t="n">
-        <v>5821</v>
-      </c>
-      <c r="H10" s="13">
-        <f>B10/E10-1</f>
-        <v/>
-      </c>
-      <c r="I10" s="13">
-        <f>C10/F10-1</f>
-        <v/>
-      </c>
-      <c r="J10" s="13">
-        <f>D10/G10-1</f>
+          <t>2022-06</t>
+        </is>
+      </c>
+      <c r="B10" s="40" t="n">
+        <v>7632</v>
+      </c>
+      <c r="C10" s="42" t="n">
+        <v>295.1</v>
+      </c>
+      <c r="D10" s="44">
+        <f>B10/C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Adjusted EPS (p)</t>
-        </is>
-      </c>
-      <c r="B11" s="5">
-        <f>Model!F20</f>
-        <v/>
-      </c>
-      <c r="C11" s="5">
-        <f>Model!G20</f>
-        <v/>
-      </c>
-      <c r="D11" s="5">
-        <f>Model!H20</f>
-        <v/>
-      </c>
-      <c r="E11" s="41" t="n">
-        <v>480.6</v>
-      </c>
-      <c r="F11" s="41" t="n">
-        <v>550.9</v>
-      </c>
-      <c r="G11" s="41" t="n">
-        <v>615.5</v>
-      </c>
-      <c r="H11" s="13">
-        <f>B11/E11-1</f>
-        <v/>
-      </c>
-      <c r="I11" s="13">
-        <f>C11/F11-1</f>
-        <v/>
-      </c>
-      <c r="J11" s="13">
-        <f>D11/G11-1</f>
+          <t>2022-07</t>
+        </is>
+      </c>
+      <c r="B11" s="40" t="n">
+        <v>7998</v>
+      </c>
+      <c r="C11" s="42" t="n">
+        <v>298.8833333333333</v>
+      </c>
+      <c r="D11" s="44">
+        <f>B11/C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DPS (p)</t>
-        </is>
-      </c>
-      <c r="B12" s="5">
-        <f>Model!F45</f>
-        <v/>
-      </c>
-      <c r="C12" s="5">
-        <f>Model!G45</f>
-        <v/>
-      </c>
-      <c r="D12" s="5">
-        <f>Model!H45</f>
-        <v/>
-      </c>
-      <c r="E12" s="41" t="n">
-        <v>167.3</v>
-      </c>
-      <c r="F12" s="41" t="n">
-        <v>189.4</v>
-      </c>
-      <c r="G12" s="41" t="n">
-        <v>209.9</v>
-      </c>
-      <c r="H12" s="13">
-        <f>B12/E12-1</f>
-        <v/>
-      </c>
-      <c r="I12" s="13">
-        <f>C12/F12-1</f>
-        <v/>
-      </c>
-      <c r="J12" s="13">
-        <f>D12/G12-1</f>
+          <t>2022-08</t>
+        </is>
+      </c>
+      <c r="B12" s="40" t="n">
+        <v>8102</v>
+      </c>
+      <c r="C12" s="42" t="n">
+        <v>302.6666666666667</v>
+      </c>
+      <c r="D12" s="44">
+        <f>B12/C12</f>
+        <v/>
+      </c>
+      <c r="E12" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2022-09</t>
+        </is>
+      </c>
+      <c r="B13" s="40" t="n">
+        <v>7628</v>
+      </c>
+      <c r="C13" s="42" t="n">
+        <v>306.45</v>
+      </c>
+      <c r="D13" s="44">
+        <f>B13/C13</f>
+        <v/>
+      </c>
+      <c r="E13" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2022-10</t>
+        </is>
+      </c>
+      <c r="B14" s="40" t="n">
+        <v>7566</v>
+      </c>
+      <c r="C14" s="42" t="n">
+        <v>310.2333333333333</v>
+      </c>
+      <c r="D14" s="44">
+        <f>B14/C14</f>
+        <v/>
+      </c>
+      <c r="E14" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2022-11</t>
+        </is>
+      </c>
+      <c r="B15" s="40" t="n">
+        <v>8248</v>
+      </c>
+      <c r="C15" s="42" t="n">
+        <v>314.0166666666667</v>
+      </c>
+      <c r="D15" s="44">
+        <f>B15/C15</f>
+        <v/>
+      </c>
+      <c r="E15" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2022-12</t>
+        </is>
+      </c>
+      <c r="B16" s="40" t="n">
+        <v>7136</v>
+      </c>
+      <c r="C16" s="42" t="n">
+        <v>317.8</v>
+      </c>
+      <c r="D16" s="44">
+        <f>B16/C16</f>
+        <v/>
+      </c>
+      <c r="E16" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2023-01</t>
+        </is>
+      </c>
+      <c r="B17" s="40" t="n">
+        <v>7406</v>
+      </c>
+      <c r="C17" s="42" t="n">
+        <v>318.3083333333333</v>
+      </c>
+      <c r="D17" s="44">
+        <f>B17/C17</f>
+        <v/>
+      </c>
+      <c r="E17" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2023-02</t>
+        </is>
+      </c>
+      <c r="B18" s="40" t="n">
+        <v>7432</v>
+      </c>
+      <c r="C18" s="42" t="n">
+        <v>318.8166666666667</v>
+      </c>
+      <c r="D18" s="44">
+        <f>B18/C18</f>
+        <v/>
+      </c>
+      <c r="E18" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2023-03</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="n">
+        <v>7868</v>
+      </c>
+      <c r="C19" s="42" t="n">
+        <v>319.325</v>
+      </c>
+      <c r="D19" s="44">
+        <f>B19/C19</f>
+        <v/>
+      </c>
+      <c r="E19" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2023-04</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="n">
+        <v>8346</v>
+      </c>
+      <c r="C20" s="42" t="n">
+        <v>319.8333333333334</v>
+      </c>
+      <c r="D20" s="44">
+        <f>B20/C20</f>
+        <v/>
+      </c>
+      <c r="E20" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2023-05</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n">
+        <v>8550</v>
+      </c>
+      <c r="C21" s="42" t="n">
+        <v>320.3416666666667</v>
+      </c>
+      <c r="D21" s="44">
+        <f>B21/C21</f>
+        <v/>
+      </c>
+      <c r="E21" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2023-06</t>
+        </is>
+      </c>
+      <c r="B22" s="40" t="n">
+        <v>8366</v>
+      </c>
+      <c r="C22" s="42" t="n">
+        <v>320.85</v>
+      </c>
+      <c r="D22" s="44">
+        <f>B22/C22</f>
+        <v/>
+      </c>
+      <c r="E22" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2023-07</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="n">
+        <v>8462</v>
+      </c>
+      <c r="C23" s="42" t="n">
+        <v>321.3583333333333</v>
+      </c>
+      <c r="D23" s="44">
+        <f>B23/C23</f>
+        <v/>
+      </c>
+      <c r="E23" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2023-08</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="n">
+        <v>8178</v>
+      </c>
+      <c r="C24" s="42" t="n">
+        <v>321.8666666666667</v>
+      </c>
+      <c r="D24" s="44">
+        <f>B24/C24</f>
+        <v/>
+      </c>
+      <c r="E24" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2023-09</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="n">
+        <v>8234</v>
+      </c>
+      <c r="C25" s="42" t="n">
+        <v>322.375</v>
+      </c>
+      <c r="D25" s="44">
+        <f>B25/C25</f>
+        <v/>
+      </c>
+      <c r="E25" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2023-10</t>
+        </is>
+      </c>
+      <c r="B26" s="40" t="n">
+        <v>8280</v>
+      </c>
+      <c r="C26" s="42" t="n">
+        <v>322.8833333333333</v>
+      </c>
+      <c r="D26" s="44">
+        <f>B26/C26</f>
+        <v/>
+      </c>
+      <c r="E26" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2023-11</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="n">
+        <v>8906</v>
+      </c>
+      <c r="C27" s="42" t="n">
+        <v>323.3916666666667</v>
+      </c>
+      <c r="D27" s="44">
+        <f>B27/C27</f>
+        <v/>
+      </c>
+      <c r="E27" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2023-12</t>
+        </is>
+      </c>
+      <c r="B28" s="40" t="n">
+        <v>9274</v>
+      </c>
+      <c r="C28" s="42" t="n">
+        <v>323.9</v>
+      </c>
+      <c r="D28" s="44">
+        <f>B28/C28</f>
+        <v/>
+      </c>
+      <c r="E28" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2024-01</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="n">
+        <v>8942</v>
+      </c>
+      <c r="C29" s="42" t="n">
+        <v>327.2</v>
+      </c>
+      <c r="D29" s="44">
+        <f>B29/C29</f>
+        <v/>
+      </c>
+      <c r="E29" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2024-02</t>
+        </is>
+      </c>
+      <c r="B30" s="40" t="n">
+        <v>8876</v>
+      </c>
+      <c r="C30" s="42" t="n">
+        <v>330.5</v>
+      </c>
+      <c r="D30" s="44">
+        <f>B30/C30</f>
+        <v/>
+      </c>
+      <c r="E30" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2024-03</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="n">
+        <v>9490</v>
+      </c>
+      <c r="C31" s="42" t="n">
+        <v>333.8</v>
+      </c>
+      <c r="D31" s="44">
+        <f>B31/C31</f>
+        <v/>
+      </c>
+      <c r="E31" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2024-04</t>
+        </is>
+      </c>
+      <c r="B32" s="40" t="n">
+        <v>8846</v>
+      </c>
+      <c r="C32" s="42" t="n">
+        <v>337.1</v>
+      </c>
+      <c r="D32" s="44">
+        <f>B32/C32</f>
+        <v/>
+      </c>
+      <c r="E32" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2024-05</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="n">
+        <v>9162</v>
+      </c>
+      <c r="C33" s="42" t="n">
+        <v>340.4</v>
+      </c>
+      <c r="D33" s="44">
+        <f>B33/C33</f>
+        <v/>
+      </c>
+      <c r="E33" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2024-06</t>
+        </is>
+      </c>
+      <c r="B34" s="40" t="n">
+        <v>9400</v>
+      </c>
+      <c r="C34" s="42" t="n">
+        <v>343.7</v>
+      </c>
+      <c r="D34" s="44">
+        <f>B34/C34</f>
+        <v/>
+      </c>
+      <c r="E34" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2024-07</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="n">
+        <v>9470</v>
+      </c>
+      <c r="C35" s="42" t="n">
+        <v>347</v>
+      </c>
+      <c r="D35" s="44">
+        <f>B35/C35</f>
+        <v/>
+      </c>
+      <c r="E35" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2024-08</t>
+        </is>
+      </c>
+      <c r="B36" s="40" t="n">
+        <v>10250</v>
+      </c>
+      <c r="C36" s="42" t="n">
+        <v>350.3</v>
+      </c>
+      <c r="D36" s="44">
+        <f>B36/C36</f>
+        <v/>
+      </c>
+      <c r="E36" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2024-09</t>
+        </is>
+      </c>
+      <c r="B37" s="40" t="n">
+        <v>10220</v>
+      </c>
+      <c r="C37" s="42" t="n">
+        <v>353.6</v>
+      </c>
+      <c r="D37" s="44">
+        <f>B37/C37</f>
+        <v/>
+      </c>
+      <c r="E37" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2024-10</t>
+        </is>
+      </c>
+      <c r="B38" s="40" t="n">
+        <v>10515</v>
+      </c>
+      <c r="C38" s="42" t="n">
+        <v>356.9</v>
+      </c>
+      <c r="D38" s="44">
+        <f>B38/C38</f>
+        <v/>
+      </c>
+      <c r="E38" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2024-11</t>
+        </is>
+      </c>
+      <c r="B39" s="40" t="n">
+        <v>11270</v>
+      </c>
+      <c r="C39" s="42" t="n">
+        <v>360.2</v>
+      </c>
+      <c r="D39" s="44">
+        <f>B39/C39</f>
+        <v/>
+      </c>
+      <c r="E39" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2024-12</t>
+        </is>
+      </c>
+      <c r="B40" s="40" t="n">
+        <v>11285</v>
+      </c>
+      <c r="C40" s="42" t="n">
+        <v>363.5</v>
+      </c>
+      <c r="D40" s="44">
+        <f>B40/C40</f>
+        <v/>
+      </c>
+      <c r="E40" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2025-01</t>
+        </is>
+      </c>
+      <c r="B41" s="40" t="n">
+        <v>12035</v>
+      </c>
+      <c r="C41" s="42" t="n">
+        <v>368.2583333333333</v>
+      </c>
+      <c r="D41" s="44">
+        <f>B41/C41</f>
+        <v/>
+      </c>
+      <c r="E41" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2025-02</t>
+        </is>
+      </c>
+      <c r="B42" s="40" t="n">
+        <v>11845</v>
+      </c>
+      <c r="C42" s="42" t="n">
+        <v>373.0166666666667</v>
+      </c>
+      <c r="D42" s="44">
+        <f>B42/C42</f>
+        <v/>
+      </c>
+      <c r="E42" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2025-03</t>
+        </is>
+      </c>
+      <c r="B43" s="40" t="n">
+        <v>11460</v>
+      </c>
+      <c r="C43" s="42" t="n">
+        <v>377.775</v>
+      </c>
+      <c r="D43" s="44">
+        <f>B43/C43</f>
+        <v/>
+      </c>
+      <c r="E43" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2025-04</t>
+        </is>
+      </c>
+      <c r="B44" s="40" t="n">
+        <v>11625</v>
+      </c>
+      <c r="C44" s="42" t="n">
+        <v>382.5333333333334</v>
+      </c>
+      <c r="D44" s="44">
+        <f>B44/C44</f>
+        <v/>
+      </c>
+      <c r="E44" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2025-05</t>
+        </is>
+      </c>
+      <c r="B45" s="40" t="n">
+        <v>11275</v>
+      </c>
+      <c r="C45" s="42" t="n">
+        <v>387.2916666666666</v>
+      </c>
+      <c r="D45" s="44">
+        <f>B45/C45</f>
+        <v/>
+      </c>
+      <c r="E45" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2025-06</t>
+        </is>
+      </c>
+      <c r="B46" s="40" t="n">
+        <v>10635</v>
+      </c>
+      <c r="C46" s="42" t="n">
+        <v>392.05</v>
+      </c>
+      <c r="D46" s="44">
+        <f>B46/C46</f>
+        <v/>
+      </c>
+      <c r="E46" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2025-07</t>
+        </is>
+      </c>
+      <c r="B47" s="40" t="n">
+        <v>9260</v>
+      </c>
+      <c r="C47" s="42" t="n">
+        <v>396.8083333333333</v>
+      </c>
+      <c r="D47" s="44">
+        <f>B47/C47</f>
+        <v/>
+      </c>
+      <c r="E47" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2025-08</t>
+        </is>
+      </c>
+      <c r="B48" s="40" t="n">
+        <v>9168</v>
+      </c>
+      <c r="C48" s="42" t="n">
+        <v>401.5666666666667</v>
+      </c>
+      <c r="D48" s="44">
+        <f>B48/C48</f>
+        <v/>
+      </c>
+      <c r="E48" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2025-09</t>
+        </is>
+      </c>
+      <c r="B49" s="40" t="n">
+        <v>8516</v>
+      </c>
+      <c r="C49" s="42" t="n">
+        <v>406.325</v>
+      </c>
+      <c r="D49" s="44">
+        <f>B49/C49</f>
+        <v/>
+      </c>
+      <c r="E49" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2025-10</t>
+        </is>
+      </c>
+      <c r="B50" s="40" t="n">
+        <v>9486</v>
+      </c>
+      <c r="C50" s="42" t="n">
+        <v>411.0833333333334</v>
+      </c>
+      <c r="D50" s="44">
+        <f>B50/C50</f>
+        <v/>
+      </c>
+      <c r="E50" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2025-11</t>
+        </is>
+      </c>
+      <c r="B51" s="40" t="n">
+        <v>8908</v>
+      </c>
+      <c r="C51" s="42" t="n">
+        <v>415.8416666666667</v>
+      </c>
+      <c r="D51" s="44">
+        <f>B51/C51</f>
+        <v/>
+      </c>
+      <c r="E51" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2025-12</t>
+        </is>
+      </c>
+      <c r="B52" s="40" t="n">
+        <v>8952</v>
+      </c>
+      <c r="C52" s="42" t="n">
+        <v>420.6</v>
+      </c>
+      <c r="D52" s="44">
+        <f>B52/C52</f>
+        <v/>
+      </c>
+      <c r="E52" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-01</t>
+        </is>
+      </c>
+      <c r="B53" s="40" t="n">
+        <v>8122</v>
+      </c>
+      <c r="C53" s="42" t="n">
+        <v>426.6</v>
+      </c>
+      <c r="D53" s="44">
+        <f>B53/C53</f>
+        <v/>
+      </c>
+      <c r="E53" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-02</t>
+        </is>
+      </c>
+      <c r="B54" s="40" t="n">
+        <v>8860</v>
+      </c>
+      <c r="C54" s="42" t="n">
+        <v>432.6</v>
+      </c>
+      <c r="D54" s="44">
+        <f>B54/C54</f>
+        <v/>
+      </c>
+      <c r="E54" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-03</t>
+        </is>
+      </c>
+      <c r="B55" s="40" t="n">
+        <v>8864</v>
+      </c>
+      <c r="C55" s="42" t="n">
+        <v>438.6</v>
+      </c>
+      <c r="D55" s="44">
+        <f>B55/C55</f>
+        <v/>
+      </c>
+      <c r="E55" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-04</t>
+        </is>
+      </c>
+      <c r="B56" s="40" t="n">
+        <v>9550</v>
+      </c>
+      <c r="C56" s="42" t="n">
+        <v>444.6</v>
+      </c>
+      <c r="D56" s="44">
+        <f>B56/C56</f>
+        <v/>
+      </c>
+      <c r="E56" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-05</t>
+        </is>
+      </c>
+      <c r="B57" s="40" t="n">
+        <v>9022</v>
+      </c>
+      <c r="C57" s="42" t="n">
+        <v>450.6</v>
+      </c>
+      <c r="D57" s="44">
+        <f>B57/C57</f>
+        <v/>
+      </c>
+      <c r="E57" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-06</t>
+        </is>
+      </c>
+      <c r="B58" s="40" t="n">
+        <v>8162</v>
+      </c>
+      <c r="C58" s="42" t="n">
+        <v>456.6</v>
+      </c>
+      <c r="D58" s="44">
+        <f>B58/C58</f>
+        <v/>
+      </c>
+      <c r="E58" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07</t>
+        </is>
+      </c>
+      <c r="B59" s="40" t="n">
+        <v>8398</v>
+      </c>
+      <c r="C59" s="42" t="n">
+        <v>462.2931993135644</v>
+      </c>
+      <c r="D59" s="44">
+        <f>B59/C59</f>
+        <v/>
+      </c>
+      <c r="E59" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-08</t>
+        </is>
+      </c>
+      <c r="B60" s="40" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C60" s="42" t="n">
+        <v>467.9863986271287</v>
+      </c>
+      <c r="D60" s="44">
+        <f>B60/C60</f>
+        <v/>
+      </c>
+      <c r="E60" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-09</t>
+        </is>
+      </c>
+      <c r="B61" s="40" t="n">
+        <v>8160</v>
+      </c>
+      <c r="C61" s="42" t="n">
+        <v>473.679597940693</v>
+      </c>
+      <c r="D61" s="44">
+        <f>B61/C61</f>
+        <v/>
+      </c>
+      <c r="E61" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10</t>
+        </is>
+      </c>
+      <c r="B62" s="40" t="n">
+        <v>9510</v>
+      </c>
+      <c r="C62" s="42" t="n">
+        <v>479.3727972542574</v>
+      </c>
+      <c r="D62" s="44">
+        <f>B62/C62</f>
+        <v/>
+      </c>
+      <c r="E62" s="44">
+        <f>AVERAGE($D$5:$D$62)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add industry evidence, hiring and stub trackers to the model; pitch reframed as outright long
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SS5TWs33kf5v4j8orcJC9a
</commit_message>
<xml_diff>
--- a/projects/01-equity-pitch-kit/models/LSEG_Model.xlsx
+++ b/projects/01-equity-pitch-kit/models/LSEG_Model.xlsx
@@ -16,12 +16,14 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SOTP" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stub ex-Tradeweb" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Valuation history" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vs Consensus" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse DCF" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pair trade" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Industry evidence" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Trackers" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="vs Consensus" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reverse DCF" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pair trade" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -30,7 +32,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="0.0%;(0.0%);&quot;–&quot;"/>
     <numFmt numFmtId="165" formatCode="#,##0&quot;p&quot;"/>
     <numFmt numFmtId="166" formatCode="0.0"/>
@@ -40,6 +42,7 @@
     <numFmt numFmtId="170" formatCode="#,##0.0&quot;p&quot;"/>
     <numFmt numFmtId="171" formatCode="0.00&quot;x&quot;"/>
     <numFmt numFmtId="172" formatCode="0.0%"/>
+    <numFmt numFmtId="173" formatCode="0.0000"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -117,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -171,6 +174,11 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="171" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="172" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -383,6 +391,288 @@
 </chartSpace>
 </file>
 
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Share of open roles by function</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="bar"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Trackers'!C5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Trackers'!$A$6:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trackers'!$C$6:$C$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Trackers'!E5</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Trackers'!$A$6:$A$13</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trackers'!$E$6:$E$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Tradeweb stake as % of LSEG market cap</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Trackers'!F17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Trackers'!$A$18:$A$162</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trackers'!$F$18:$F$162</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>LSEG vs FactSet, GBP, Jan 2024 = 100</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Trackers'!G17</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Trackers'!$A$18:$A$162</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Trackers'!$G$18:$G$162</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
@@ -402,6 +692,77 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>3</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5040000" cy="2520000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="3" name="Chart 3"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -892,6 +1253,4159 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:F9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>What third-party data says about AI and market-data demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Credible industry studies and filings, Apr–Oct 2026. These inform the retention and scenario assumptions; they are not inputs to formulas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>Sample</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>Finding</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Read for LSEG</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="51" t="inlineStr">
+        <is>
+          <t>Burton-Taylor (TP ICAP), via FOW</t>
+        </is>
+      </c>
+      <c r="B5" s="51" t="inlineStr">
+        <is>
+          <t>8 Apr 2026</t>
+        </is>
+      </c>
+      <c r="C5" s="51" t="inlineStr">
+        <is>
+          <t>Industry spend data</t>
+        </is>
+      </c>
+      <c r="D5" s="51" t="inlineStr">
+        <is>
+          <t>Global financial market data spend reached $49.2bn in 2025, up 6.5%; AI, automated trading and volatility outweighed cost pressure.</t>
+        </is>
+      </c>
+      <c r="E5" s="51" t="inlineStr">
+        <is>
+          <t>Demand for data is still growing.</t>
+        </is>
+      </c>
+      <c r="F5" s="51" t="inlineStr">
+        <is>
+          <t>https://www.fow.com/insights/market-data-spend-hits-usd49-2bn-as-ai-volatility-and-algos-drive-growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="51" t="inlineStr">
+        <is>
+          <t>Expand Research (BCG), via A-Team Insight</t>
+        </is>
+      </c>
+      <c r="B6" s="51" t="inlineStr">
+        <is>
+          <t>20 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C6" s="51" t="inlineStr">
+        <is>
+          <t>Industry spend data</t>
+        </is>
+      </c>
+      <c r="D6" s="51" t="inlineStr">
+        <is>
+          <t>Market and reference data spend passed $50bn; a further 7% rise expected in 2026. Data teams manage 34% more vendors than four years ago.</t>
+        </is>
+      </c>
+      <c r="E6" s="51" t="inlineStr">
+        <is>
+          <t>Spend growth is broadening, not shrinking.</t>
+        </is>
+      </c>
+      <c r="F6" s="51" t="inlineStr">
+        <is>
+          <t>https://a-teaminsight.com/blog/substantive-research-finds-ai-driving-market-data-costs-higher-as-investment-research-budgets-stall/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="51" t="inlineStr">
+        <is>
+          <t>Crisil Coalition Greenwich and SIX, Market Data Study</t>
+        </is>
+      </c>
+      <c r="B7" s="51" t="inlineStr">
+        <is>
+          <t>13 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C7" s="51" t="inlineStr">
+        <is>
+          <t>73 buy- and sell-side institutions</t>
+        </is>
+      </c>
+      <c r="D7" s="51" t="inlineStr">
+        <is>
+          <t>Market data spending could rise by more than 50% by 2027, driven largely by AI adoption; licences built for human users are mismatched to AI use.</t>
+        </is>
+      </c>
+      <c r="E7" s="51" t="inlineStr">
+        <is>
+          <t>AI increases data consumption and gives data owners pricing power.</t>
+        </is>
+      </c>
+      <c r="F7" s="51" t="inlineStr">
+        <is>
+          <t>https://fintech.garden/news/2026-10-13-ai-expected-to-push-market-data-costs-up-more-than-50-by-2027-study-finds/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="51" t="inlineStr">
+        <is>
+          <t>Substantive Research, via A-Team Insight</t>
+        </is>
+      </c>
+      <c r="B8" s="51" t="inlineStr">
+        <is>
+          <t>20 Oct 2026</t>
+        </is>
+      </c>
+      <c r="C8" s="51" t="inlineStr">
+        <is>
+          <t>50 asset managers, c.$20trn AUM</t>
+        </is>
+      </c>
+      <c r="D8" s="51" t="inlineStr">
+        <is>
+          <t>AI-related charges in 2026 vendor proposals ranged from $30k to $1m; some agreements could rise up to 50% in 2027. Research budgets rose only 0.4% in H1 2026; AI research tooling spend rose 40%.</t>
+        </is>
+      </c>
+      <c r="E8" s="51" t="inlineStr">
+        <is>
+          <t>Budgets are tight, so money moves from people and screens to data and AI tooling.</t>
+        </is>
+      </c>
+      <c r="F8" s="51" t="inlineStr">
+        <is>
+          <t>https://a-teaminsight.com/blog/substantive-research-finds-ai-driving-market-data-costs-higher-as-investment-research-budgets-stall/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="51" t="inlineStr">
+        <is>
+          <t>FactSet Q4 FY2026 results (8-K)</t>
+        </is>
+      </c>
+      <c r="B9" s="51" t="inlineStr">
+        <is>
+          <t>30 Sep 2026</t>
+        </is>
+      </c>
+      <c r="C9" s="51" t="inlineStr">
+        <is>
+          <t>Company filing</t>
+        </is>
+      </c>
+      <c r="D9" s="51" t="inlineStr">
+        <is>
+          <t>Organic ASV +7.0% to $2.57bn; ASV retention above 95%; AI solutions ASV more than doubled. FY27 guide: organic ASV +5.0% to 6.5%.</t>
+        </is>
+      </c>
+      <c r="E9" s="51" t="inlineStr">
+        <is>
+          <t>Even the purest 'AI loser' is not losing customers. Also a reason not to short it.</t>
+        </is>
+      </c>
+      <c r="F9" s="51" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/Archives/edgar/data/0001013237/000162828026063888/fdsq42026earningsrelease.htm</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G164"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Trackers: hiring mix and the Tradeweb stub</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Data in /data, refreshed every Monday by .github/workflows/refresh-data.yml (Workday career sites; weekly prices).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="12" t="inlineStr">
+        <is>
+          <t>Open roles by function, snapshot 2026-10-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Function</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>LSEG</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>LSEG %</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>FactSet</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>FactSet %</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>AI &amp; data science</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>49</v>
+      </c>
+      <c r="C6" s="13">
+        <f>B6/B14</f>
+        <v/>
+      </c>
+      <c r="D6" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="13">
+        <f>D6/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Sales &amp; client</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>87</v>
+      </c>
+      <c r="C7" s="13">
+        <f>B7/B14</f>
+        <v/>
+      </c>
+      <c r="D7" t="n">
+        <v>25</v>
+      </c>
+      <c r="E7" s="13">
+        <f>D7/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>286</v>
+      </c>
+      <c r="C8" s="13">
+        <f>B8/B14</f>
+        <v/>
+      </c>
+      <c r="D8" t="n">
+        <v>29</v>
+      </c>
+      <c r="E8" s="13">
+        <f>D8/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Content &amp; data ops</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>79</v>
+      </c>
+      <c r="C9" s="13">
+        <f>B9/B14</f>
+        <v/>
+      </c>
+      <c r="D9" t="n">
+        <v>9</v>
+      </c>
+      <c r="E9" s="13">
+        <f>D9/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Product</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>24</v>
+      </c>
+      <c r="C10" s="13">
+        <f>B10/B14</f>
+        <v/>
+      </c>
+      <c r="D10" t="n">
+        <v>4</v>
+      </c>
+      <c r="E10" s="13">
+        <f>D10/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>54</v>
+      </c>
+      <c r="C11" s="13">
+        <f>B11/B14</f>
+        <v/>
+      </c>
+      <c r="D11" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="13">
+        <f>D11/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Corporate</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>36</v>
+      </c>
+      <c r="C12" s="13">
+        <f>B12/B14</f>
+        <v/>
+      </c>
+      <c r="D12" t="n">
+        <v>5</v>
+      </c>
+      <c r="E12" s="13">
+        <f>D12/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>53</v>
+      </c>
+      <c r="C13" s="13">
+        <f>B13/B14</f>
+        <v/>
+      </c>
+      <c r="D13" t="n">
+        <v>16</v>
+      </c>
+      <c r="E13" s="13">
+        <f>D13/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="12" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B14" s="12">
+        <f>SUM(B6:B13)</f>
+        <v/>
+      </c>
+      <c r="D14" s="12">
+        <f>SUM(D6:D13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
+        <is>
+          <t>Weekly: Tradeweb stake as % of LSEG market cap, and LSEG vs FactSet relative price in GBP (Jan 2024 = 100)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Week</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="inlineStr">
+        <is>
+          <t>LSEG (p)</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Tradeweb ($)</t>
+        </is>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>FactSet ($)</t>
+        </is>
+      </c>
+      <c r="E17" s="8" t="inlineStr">
+        <is>
+          <t>GBPUSD</t>
+        </is>
+      </c>
+      <c r="F17" s="8" t="inlineStr">
+        <is>
+          <t>Tradeweb stake % of LSEG</t>
+        </is>
+      </c>
+      <c r="G17" s="8" t="inlineStr">
+        <is>
+          <t>LSEG vs FactSet (rebased)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="52" t="inlineStr">
+        <is>
+          <t>2024-01-01</t>
+        </is>
+      </c>
+      <c r="B18" s="40" t="n">
+        <v>8980</v>
+      </c>
+      <c r="C18" s="30" t="n">
+        <v>93</v>
+      </c>
+      <c r="D18" s="30" t="n">
+        <v>456.5799865722656</v>
+      </c>
+      <c r="E18" s="53" t="n">
+        <v>1.272599816322327</v>
+      </c>
+      <c r="F18" s="13" t="n">
+        <v>0.182264658935901</v>
+      </c>
+      <c r="G18" s="33" t="n">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="52" t="inlineStr">
+        <is>
+          <t>2024-01-08</t>
+        </is>
+      </c>
+      <c r="B19" s="40" t="n">
+        <v>9184</v>
+      </c>
+      <c r="C19" s="30" t="n">
+        <v>95.91000366210938</v>
+      </c>
+      <c r="D19" s="30" t="n">
+        <v>466.5599975585938</v>
+      </c>
+      <c r="E19" s="53" t="n">
+        <v>1.274700522422791</v>
+      </c>
+      <c r="F19" s="13" t="n">
+        <v>0.1835159672927071</v>
+      </c>
+      <c r="G19" s="33" t="n">
+        <v>100.2492695602747</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="52" t="inlineStr">
+        <is>
+          <t>2024-01-15</t>
+        </is>
+      </c>
+      <c r="B20" s="40" t="n">
+        <v>9140</v>
+      </c>
+      <c r="C20" s="30" t="n">
+        <v>97.94999694824219</v>
+      </c>
+      <c r="D20" s="30" t="n">
+        <v>463.4500122070312</v>
+      </c>
+      <c r="E20" s="53" t="n">
+        <v>1.270499587059021</v>
+      </c>
+      <c r="F20" s="13" t="n">
+        <v>0.188971354979676</v>
+      </c>
+      <c r="G20" s="33" t="n">
+        <v>100.1074742596748</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="52" t="inlineStr">
+        <is>
+          <t>2024-01-22</t>
+        </is>
+      </c>
+      <c r="B21" s="40" t="n">
+        <v>9070</v>
+      </c>
+      <c r="C21" s="30" t="n">
+        <v>97.83000183105469</v>
+      </c>
+      <c r="D21" s="30" t="n">
+        <v>470.6700134277344</v>
+      </c>
+      <c r="E21" s="53" t="n">
+        <v>1.271000027656555</v>
+      </c>
+      <c r="F21" s="13" t="n">
+        <v>0.1901488852057663</v>
+      </c>
+      <c r="G21" s="33" t="n">
+        <v>97.85544473214937</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="52" t="inlineStr">
+        <is>
+          <t>2024-01-29</t>
+        </is>
+      </c>
+      <c r="B22" s="40" t="n">
+        <v>8876</v>
+      </c>
+      <c r="C22" s="30" t="n">
+        <v>96.83000183105469</v>
+      </c>
+      <c r="D22" s="30" t="n">
+        <v>486.7699890136719</v>
+      </c>
+      <c r="E22" s="53" t="n">
+        <v>1.263399958610535</v>
+      </c>
+      <c r="F22" s="13" t="n">
+        <v>0.1935034269837231</v>
+      </c>
+      <c r="G22" s="33" t="n">
+        <v>92.04136172663286</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="52" t="inlineStr">
+        <is>
+          <t>2024-02-05</t>
+        </is>
+      </c>
+      <c r="B23" s="40" t="n">
+        <v>8836</v>
+      </c>
+      <c r="C23" s="30" t="n">
+        <v>102.3899993896484</v>
+      </c>
+      <c r="D23" s="30" t="n">
+        <v>477.5899963378906</v>
+      </c>
+      <c r="E23" s="53" t="n">
+        <v>1.262999415397644</v>
+      </c>
+      <c r="F23" s="13" t="n">
+        <v>0.2056353946559263</v>
+      </c>
+      <c r="G23" s="33" t="n">
+        <v>93.35816641024542</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="52" t="inlineStr">
+        <is>
+          <t>2024-02-12</t>
+        </is>
+      </c>
+      <c r="B24" s="40" t="n">
+        <v>8888</v>
+      </c>
+      <c r="C24" s="30" t="n">
+        <v>101.5100021362305</v>
+      </c>
+      <c r="D24" s="30" t="n">
+        <v>458.4200134277344</v>
+      </c>
+      <c r="E24" s="53" t="n">
+        <v>1.260299801826477</v>
+      </c>
+      <c r="F24" s="13" t="n">
+        <v>0.2031385882360129</v>
+      </c>
+      <c r="G24" s="33" t="n">
+        <v>97.62544409129855</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="52" t="inlineStr">
+        <is>
+          <t>2024-02-19</t>
+        </is>
+      </c>
+      <c r="B25" s="40" t="n">
+        <v>8922</v>
+      </c>
+      <c r="C25" s="30" t="n">
+        <v>105.0899963378906</v>
+      </c>
+      <c r="D25" s="30" t="n">
+        <v>463.4700012207031</v>
+      </c>
+      <c r="E25" s="53" t="n">
+        <v>1.267999172210693</v>
+      </c>
+      <c r="F25" s="13" t="n">
+        <v>0.2082591182760366</v>
+      </c>
+      <c r="G25" s="33" t="n">
+        <v>97.52326619389395</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="52" t="inlineStr">
+        <is>
+          <t>2024-02-26</t>
+        </is>
+      </c>
+      <c r="B26" s="40" t="n">
+        <v>9016</v>
+      </c>
+      <c r="C26" s="30" t="n">
+        <v>104.8099975585938</v>
+      </c>
+      <c r="D26" s="30" t="n">
+        <v>461.3200073242188</v>
+      </c>
+      <c r="E26" s="53" t="n">
+        <v>1.265800356864929</v>
+      </c>
+      <c r="F26" s="13" t="n">
+        <v>0.205925330122822</v>
+      </c>
+      <c r="G26" s="33" t="n">
+        <v>98.83835408774048</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="52" t="inlineStr">
+        <is>
+          <t>2024-03-04</t>
+        </is>
+      </c>
+      <c r="B27" s="40" t="n">
+        <v>9264</v>
+      </c>
+      <c r="C27" s="30" t="n">
+        <v>102.879997253418</v>
+      </c>
+      <c r="D27" s="30" t="n">
+        <v>466.1199951171875</v>
+      </c>
+      <c r="E27" s="53" t="n">
+        <v>1.285900712013245</v>
+      </c>
+      <c r="F27" s="13" t="n">
+        <v>0.1936749649505239</v>
+      </c>
+      <c r="G27" s="33" t="n">
+        <v>102.1073318942184</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="52" t="inlineStr">
+        <is>
+          <t>2024-03-11</t>
+        </is>
+      </c>
+      <c r="B28" s="40" t="n">
+        <v>9450</v>
+      </c>
+      <c r="C28" s="30" t="n">
+        <v>104.1900024414062</v>
+      </c>
+      <c r="D28" s="30" t="n">
+        <v>475.9599914550781</v>
+      </c>
+      <c r="E28" s="53" t="n">
+        <v>1.273199319839478</v>
+      </c>
+      <c r="F28" s="13" t="n">
+        <v>0.1942266074140616</v>
+      </c>
+      <c r="G28" s="33" t="n">
+        <v>100.9965262298678</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="52" t="inlineStr">
+        <is>
+          <t>2024-03-18</t>
+        </is>
+      </c>
+      <c r="B29" s="40" t="n">
+        <v>9652</v>
+      </c>
+      <c r="C29" s="30" t="n">
+        <v>105.2300033569336</v>
+      </c>
+      <c r="D29" s="30" t="n">
+        <v>447.4599914550781</v>
+      </c>
+      <c r="E29" s="53" t="n">
+        <v>1.260199785232544</v>
+      </c>
+      <c r="F29" s="13" t="n">
+        <v>0.1940689779340321</v>
+      </c>
+      <c r="G29" s="33" t="n">
+        <v>108.6053407664602</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="52" t="inlineStr">
+        <is>
+          <t>2024-03-31</t>
+        </is>
+      </c>
+      <c r="B30" s="40" t="n">
+        <v>9378</v>
+      </c>
+      <c r="C30" s="30" t="n">
+        <v>104.1699981689453</v>
+      </c>
+      <c r="D30" s="30" t="n">
+        <v>454.3900146484375</v>
+      </c>
+      <c r="E30" s="53" t="n">
+        <v>1.263899683952332</v>
+      </c>
+      <c r="F30" s="13" t="n">
+        <v>0.1972009118128356</v>
+      </c>
+      <c r="G30" s="33" t="n">
+        <v>104.2179995519169</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="52" t="inlineStr">
+        <is>
+          <t>2024-04-07</t>
+        </is>
+      </c>
+      <c r="B31" s="40" t="n">
+        <v>9314</v>
+      </c>
+      <c r="C31" s="30" t="n">
+        <v>102.4000015258789</v>
+      </c>
+      <c r="D31" s="30" t="n">
+        <v>433.1700134277344</v>
+      </c>
+      <c r="E31" s="53" t="n">
+        <v>1.245800137519836</v>
+      </c>
+      <c r="F31" s="13" t="n">
+        <v>0.1980463500020924</v>
+      </c>
+      <c r="G31" s="33" t="n">
+        <v>107.0224531570183</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="52" t="inlineStr">
+        <is>
+          <t>2024-04-14</t>
+        </is>
+      </c>
+      <c r="B32" s="40" t="n">
+        <v>8984</v>
+      </c>
+      <c r="C32" s="30" t="n">
+        <v>102.129997253418</v>
+      </c>
+      <c r="D32" s="30" t="n">
+        <v>426.239990234375</v>
+      </c>
+      <c r="E32" s="53" t="n">
+        <v>1.237000703811646</v>
+      </c>
+      <c r="F32" s="13" t="n">
+        <v>0.2062659393042311</v>
+      </c>
+      <c r="G32" s="33" t="n">
+        <v>104.1679637795144</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="52" t="inlineStr">
+        <is>
+          <t>2024-04-21</t>
+        </is>
+      </c>
+      <c r="B33" s="40" t="n">
+        <v>8934</v>
+      </c>
+      <c r="C33" s="30" t="n">
+        <v>101.0500030517578</v>
+      </c>
+      <c r="D33" s="30" t="n">
+        <v>434.0199890136719</v>
+      </c>
+      <c r="E33" s="53" t="n">
+        <v>1.263899683952332</v>
+      </c>
+      <c r="F33" s="13" t="n">
+        <v>0.20088803745942</v>
+      </c>
+      <c r="G33" s="33" t="n">
+        <v>103.9435391330819</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="52" t="inlineStr">
+        <is>
+          <t>2024-04-28</t>
+        </is>
+      </c>
+      <c r="B34" s="40" t="n">
+        <v>9162</v>
+      </c>
+      <c r="C34" s="30" t="n">
+        <v>101.8399963378906</v>
+      </c>
+      <c r="D34" s="30" t="n">
+        <v>421.4700012207031</v>
+      </c>
+      <c r="E34" s="53" t="n">
+        <v>1.254900336265564</v>
+      </c>
+      <c r="F34" s="13" t="n">
+        <v>0.1988646403708517</v>
+      </c>
+      <c r="G34" s="33" t="n">
+        <v>108.9887151390269</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="52" t="inlineStr">
+        <is>
+          <t>2024-05-05</t>
+        </is>
+      </c>
+      <c r="B35" s="40" t="n">
+        <v>9128</v>
+      </c>
+      <c r="C35" s="30" t="n">
+        <v>104.5400009155273</v>
+      </c>
+      <c r="D35" s="30" t="n">
+        <v>428.25</v>
+      </c>
+      <c r="E35" s="53" t="n">
+        <v>1.247599959373474</v>
+      </c>
+      <c r="F35" s="13" t="n">
+        <v>0.2061259457268322</v>
+      </c>
+      <c r="G35" s="33" t="n">
+        <v>106.2434805556205</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="52" t="inlineStr">
+        <is>
+          <t>2024-05-12</t>
+        </is>
+      </c>
+      <c r="B36" s="40" t="n">
+        <v>9336</v>
+      </c>
+      <c r="C36" s="30" t="n">
+        <v>110.4100036621094</v>
+      </c>
+      <c r="D36" s="30" t="n">
+        <v>439.1600036621094</v>
+      </c>
+      <c r="E36" s="53" t="n">
+        <v>1.266600370407104</v>
+      </c>
+      <c r="F36" s="13" t="n">
+        <v>0.2096870222429605</v>
+      </c>
+      <c r="G36" s="33" t="n">
+        <v>107.5787148438785</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="52" t="inlineStr">
+        <is>
+          <t>2024-05-19</t>
+        </is>
+      </c>
+      <c r="B37" s="40" t="n">
+        <v>9324</v>
+      </c>
+      <c r="C37" s="30" t="n">
+        <v>112.8099975585938</v>
+      </c>
+      <c r="D37" s="30" t="n">
+        <v>448.8800048828125</v>
+      </c>
+      <c r="E37" s="53" t="n">
+        <v>1.266600370407104</v>
+      </c>
+      <c r="F37" s="13" t="n">
+        <v>0.2145515922006041</v>
+      </c>
+      <c r="G37" s="33" t="n">
+        <v>105.1139347048453</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="52" t="inlineStr">
+        <is>
+          <t>2024-05-26</t>
+        </is>
+      </c>
+      <c r="B38" s="40" t="n">
+        <v>9162</v>
+      </c>
+      <c r="C38" s="30" t="n">
+        <v>112.25</v>
+      </c>
+      <c r="D38" s="30" t="n">
+        <v>436.0400085449219</v>
+      </c>
+      <c r="E38" s="53" t="n">
+        <v>1.273799300193787</v>
+      </c>
+      <c r="F38" s="13" t="n">
+        <v>0.2160645604837109</v>
+      </c>
+      <c r="G38" s="33" t="n">
+        <v>106.9334631243783</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="52" t="inlineStr">
+        <is>
+          <t>2024-06-02</t>
+        </is>
+      </c>
+      <c r="B39" s="40" t="n">
+        <v>9432</v>
+      </c>
+      <c r="C39" s="30" t="n">
+        <v>109.0100021362305</v>
+      </c>
+      <c r="D39" s="30" t="n">
+        <v>404.260009765625</v>
+      </c>
+      <c r="E39" s="53" t="n">
+        <v>1.270199298858643</v>
+      </c>
+      <c r="F39" s="13" t="n">
+        <v>0.2044285900632309</v>
+      </c>
+      <c r="G39" s="33" t="n">
+        <v>118.4032318437814</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="52" t="inlineStr">
+        <is>
+          <t>2024-06-09</t>
+        </is>
+      </c>
+      <c r="B40" s="40" t="n">
+        <v>9434</v>
+      </c>
+      <c r="C40" s="30" t="n">
+        <v>105.3099975585938</v>
+      </c>
+      <c r="D40" s="30" t="n">
+        <v>409.9299926757812</v>
+      </c>
+      <c r="E40" s="53" t="n">
+        <v>1.26610004901886</v>
+      </c>
+      <c r="F40" s="13" t="n">
+        <v>0.1981158051676622</v>
+      </c>
+      <c r="G40" s="33" t="n">
+        <v>116.413375149298</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="52" t="inlineStr">
+        <is>
+          <t>2024-06-16</t>
+        </is>
+      </c>
+      <c r="B41" s="40" t="n">
+        <v>9654</v>
+      </c>
+      <c r="C41" s="30" t="n">
+        <v>104.3099975585938</v>
+      </c>
+      <c r="D41" s="30" t="n">
+        <v>401.739990234375</v>
+      </c>
+      <c r="E41" s="53" t="n">
+        <v>1.265499114990234</v>
+      </c>
+      <c r="F41" s="13" t="n">
+        <v>0.1918813190509435</v>
+      </c>
+      <c r="G41" s="33" t="n">
+        <v>121.4990140471131</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="52" t="inlineStr">
+        <is>
+          <t>2024-06-23</t>
+        </is>
+      </c>
+      <c r="B42" s="40" t="n">
+        <v>9400</v>
+      </c>
+      <c r="C42" s="30" t="n">
+        <v>105.7200012207031</v>
+      </c>
+      <c r="D42" s="30" t="n">
+        <v>423.7300109863281</v>
+      </c>
+      <c r="E42" s="53" t="n">
+        <v>1.264999747276306</v>
+      </c>
+      <c r="F42" s="13" t="n">
+        <v>0.1998376242934096</v>
+      </c>
+      <c r="G42" s="33" t="n">
+        <v>112.1186206422094</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="52" t="inlineStr">
+        <is>
+          <t>2024-06-30</t>
+        </is>
+      </c>
+      <c r="B43" s="40" t="n">
+        <v>9312</v>
+      </c>
+      <c r="C43" s="30" t="n">
+        <v>106</v>
+      </c>
+      <c r="D43" s="30" t="n">
+        <v>408.2699890136719</v>
+      </c>
+      <c r="E43" s="53" t="n">
+        <v>1.27970027923584</v>
+      </c>
+      <c r="F43" s="13" t="n">
+        <v>0.1999657074081692</v>
+      </c>
+      <c r="G43" s="33" t="n">
+        <v>116.6144727432116</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="52" t="inlineStr">
+        <is>
+          <t>2024-07-07</t>
+        </is>
+      </c>
+      <c r="B44" s="40" t="n">
+        <v>9428</v>
+      </c>
+      <c r="C44" s="30" t="n">
+        <v>106.4899978637695</v>
+      </c>
+      <c r="D44" s="30" t="n">
+        <v>423.4100036621094</v>
+      </c>
+      <c r="E44" s="53" t="n">
+        <v>1.270299315452576</v>
+      </c>
+      <c r="F44" s="13" t="n">
+        <v>0.1999155516544502</v>
+      </c>
+      <c r="G44" s="33" t="n">
+        <v>113.0090440938032</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="52" t="inlineStr">
+        <is>
+          <t>2024-07-14</t>
+        </is>
+      </c>
+      <c r="B45" s="40" t="n">
+        <v>9422</v>
+      </c>
+      <c r="C45" s="30" t="n">
+        <v>104.9400024414062</v>
+      </c>
+      <c r="D45" s="30" t="n">
+        <v>423.8999938964844</v>
+      </c>
+      <c r="E45" s="53" t="n">
+        <v>1.291799426078796</v>
+      </c>
+      <c r="F45" s="13" t="n">
+        <v>0.1938781199662657</v>
+      </c>
+      <c r="G45" s="33" t="n">
+        <v>114.7158572722581</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="52" t="inlineStr">
+        <is>
+          <t>2024-07-21</t>
+        </is>
+      </c>
+      <c r="B46" s="40" t="n">
+        <v>9478</v>
+      </c>
+      <c r="C46" s="30" t="n">
+        <v>109.4000015258789</v>
+      </c>
+      <c r="D46" s="30" t="n">
+        <v>424.3200073242188</v>
+      </c>
+      <c r="E46" s="53" t="n">
+        <v>1.285700678825378</v>
+      </c>
+      <c r="F46" s="13" t="n">
+        <v>0.2019059856247249</v>
+      </c>
+      <c r="G46" s="33" t="n">
+        <v>114.739181051264</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="52" t="inlineStr">
+        <is>
+          <t>2024-07-28</t>
+        </is>
+      </c>
+      <c r="B47" s="40" t="n">
+        <v>9740</v>
+      </c>
+      <c r="C47" s="30" t="n">
+        <v>106.8399963378906</v>
+      </c>
+      <c r="D47" s="30" t="n">
+        <v>415.3299865722656</v>
+      </c>
+      <c r="E47" s="53" t="n">
+        <v>1.280799984931946</v>
+      </c>
+      <c r="F47" s="13" t="n">
+        <v>0.1926391587389683</v>
+      </c>
+      <c r="G47" s="33" t="n">
+        <v>120.0039829951848</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="52" t="inlineStr">
+        <is>
+          <t>2024-08-04</t>
+        </is>
+      </c>
+      <c r="B48" s="40" t="n">
+        <v>9828</v>
+      </c>
+      <c r="C48" s="30" t="n">
+        <v>109.870002746582</v>
+      </c>
+      <c r="D48" s="30" t="n">
+        <v>414.5599975585938</v>
+      </c>
+      <c r="E48" s="53" t="n">
+        <v>1.275900721549988</v>
+      </c>
+      <c r="F48" s="13" t="n">
+        <v>0.1971108943240464</v>
+      </c>
+      <c r="G48" s="33" t="n">
+        <v>120.8490709032957</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="52" t="inlineStr">
+        <is>
+          <t>2024-08-11</t>
+        </is>
+      </c>
+      <c r="B49" s="40" t="n">
+        <v>9970</v>
+      </c>
+      <c r="C49" s="30" t="n">
+        <v>115.4000015258789</v>
+      </c>
+      <c r="D49" s="30" t="n">
+        <v>403.0299987792969</v>
+      </c>
+      <c r="E49" s="53" t="n">
+        <v>1.29449999332428</v>
+      </c>
+      <c r="F49" s="13" t="n">
+        <v>0.2011799432341421</v>
+      </c>
+      <c r="G49" s="33" t="n">
+        <v>127.9406390710803</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="52" t="inlineStr">
+        <is>
+          <t>2024-08-18</t>
+        </is>
+      </c>
+      <c r="B50" s="40" t="n">
+        <v>10010</v>
+      </c>
+      <c r="C50" s="30" t="n">
+        <v>116.0100021362305</v>
+      </c>
+      <c r="D50" s="30" t="n">
+        <v>410.8699951171875</v>
+      </c>
+      <c r="E50" s="53" t="n">
+        <v>1.321899771690369</v>
+      </c>
+      <c r="F50" s="13" t="n">
+        <v>0.1972883633171223</v>
+      </c>
+      <c r="G50" s="33" t="n">
+        <v>128.6698682480694</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="52" t="inlineStr">
+        <is>
+          <t>2024-08-25</t>
+        </is>
+      </c>
+      <c r="B51" s="40" t="n">
+        <v>10250</v>
+      </c>
+      <c r="C51" s="30" t="n">
+        <v>117.4499969482422</v>
+      </c>
+      <c r="D51" s="30" t="n">
+        <v>408.9700012207031</v>
+      </c>
+      <c r="E51" s="53" t="n">
+        <v>1.313199400901794</v>
+      </c>
+      <c r="F51" s="13" t="n">
+        <v>0.196381096427449</v>
+      </c>
+      <c r="G51" s="33" t="n">
+        <v>131.4957651892358</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="52" t="inlineStr">
+        <is>
+          <t>2024-09-01</t>
+        </is>
+      </c>
+      <c r="B52" s="40" t="n">
+        <v>10180</v>
+      </c>
+      <c r="C52" s="30" t="n">
+        <v>118.2399978637695</v>
+      </c>
+      <c r="D52" s="30" t="n">
+        <v>422.8399963378906</v>
+      </c>
+      <c r="E52" s="53" t="n">
+        <v>1.313299417495728</v>
+      </c>
+      <c r="F52" s="13" t="n">
+        <v>0.1990749779076619</v>
+      </c>
+      <c r="G52" s="33" t="n">
+        <v>126.3234992266403</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="52" t="inlineStr">
+        <is>
+          <t>2024-09-08</t>
+        </is>
+      </c>
+      <c r="B53" s="40" t="n">
+        <v>10480</v>
+      </c>
+      <c r="C53" s="30" t="n">
+        <v>111.8099975585938</v>
+      </c>
+      <c r="D53" s="30" t="n">
+        <v>424.0299987792969</v>
+      </c>
+      <c r="E53" s="53" t="n">
+        <v>1.312499523162842</v>
+      </c>
+      <c r="F53" s="13" t="n">
+        <v>0.1829981011674686</v>
+      </c>
+      <c r="G53" s="33" t="n">
+        <v>129.6022473468332</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="52" t="inlineStr">
+        <is>
+          <t>2024-09-15</t>
+        </is>
+      </c>
+      <c r="B54" s="40" t="n">
+        <v>10315</v>
+      </c>
+      <c r="C54" s="30" t="n">
+        <v>117.5400009155273</v>
+      </c>
+      <c r="D54" s="30" t="n">
+        <v>445.3599853515625</v>
+      </c>
+      <c r="E54" s="53" t="n">
+        <v>1.331800818443298</v>
+      </c>
+      <c r="F54" s="13" t="n">
+        <v>0.1926487347746139</v>
+      </c>
+      <c r="G54" s="33" t="n">
+        <v>123.2383837113741</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="52" t="inlineStr">
+        <is>
+          <t>2024-09-22</t>
+        </is>
+      </c>
+      <c r="B55" s="40" t="n">
+        <v>10265</v>
+      </c>
+      <c r="C55" s="30" t="n">
+        <v>119.4800033569336</v>
+      </c>
+      <c r="D55" s="30" t="n">
+        <v>465.9100036621094</v>
+      </c>
+      <c r="E55" s="53" t="n">
+        <v>1.337200522422791</v>
+      </c>
+      <c r="F55" s="13" t="n">
+        <v>0.1960159102745835</v>
+      </c>
+      <c r="G55" s="33" t="n">
+        <v>117.706957460708</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="52" t="inlineStr">
+        <is>
+          <t>2024-09-29</t>
+        </is>
+      </c>
+      <c r="B56" s="40" t="n">
+        <v>10235</v>
+      </c>
+      <c r="C56" s="30" t="n">
+        <v>121.75</v>
+      </c>
+      <c r="D56" s="30" t="n">
+        <v>458.489990234375</v>
+      </c>
+      <c r="E56" s="53" t="n">
+        <v>1.312299728393555</v>
+      </c>
+      <c r="F56" s="13" t="n">
+        <v>0.2041560665561671</v>
+      </c>
+      <c r="G56" s="33" t="n">
+        <v>117.0414532180989</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="52" t="inlineStr">
+        <is>
+          <t>2024-10-06</t>
+        </is>
+      </c>
+      <c r="B57" s="40" t="n">
+        <v>10120</v>
+      </c>
+      <c r="C57" s="30" t="n">
+        <v>131.4100036621094</v>
+      </c>
+      <c r="D57" s="30" t="n">
+        <v>457</v>
+      </c>
+      <c r="E57" s="53" t="n">
+        <v>1.306999802589417</v>
+      </c>
+      <c r="F57" s="13" t="n">
+        <v>0.223794404865307</v>
+      </c>
+      <c r="G57" s="33" t="n">
+        <v>115.6347890691153</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="52" t="inlineStr">
+        <is>
+          <t>2024-10-13</t>
+        </is>
+      </c>
+      <c r="B58" s="40" t="n">
+        <v>10535</v>
+      </c>
+      <c r="C58" s="30" t="n">
+        <v>133.4400024414062</v>
+      </c>
+      <c r="D58" s="30" t="n">
+        <v>456.8099975585938</v>
+      </c>
+      <c r="E58" s="53" t="n">
+        <v>1.304900407791138</v>
+      </c>
+      <c r="F58" s="13" t="n">
+        <v>0.2186822838254995</v>
+      </c>
+      <c r="G58" s="33" t="n">
+        <v>120.233360233646</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="52" t="inlineStr">
+        <is>
+          <t>2024-10-20</t>
+        </is>
+      </c>
+      <c r="B59" s="40" t="n">
+        <v>10605</v>
+      </c>
+      <c r="C59" s="30" t="n">
+        <v>133.0399932861328</v>
+      </c>
+      <c r="D59" s="30" t="n">
+        <v>471.5299987792969</v>
+      </c>
+      <c r="E59" s="53" t="n">
+        <v>1.296199798583984</v>
+      </c>
+      <c r="F59" s="13" t="n">
+        <v>0.2180729015550474</v>
+      </c>
+      <c r="G59" s="33" t="n">
+        <v>116.4721179379503</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="52" t="inlineStr">
+        <is>
+          <t>2024-10-28</t>
+        </is>
+      </c>
+      <c r="B60" s="40" t="n">
+        <v>10750</v>
+      </c>
+      <c r="C60" s="30" t="n">
+        <v>126.9000015258789</v>
+      </c>
+      <c r="D60" s="30" t="n">
+        <v>458.7999877929688</v>
+      </c>
+      <c r="E60" s="53" t="n">
+        <v>1.292200088500977</v>
+      </c>
+      <c r="F60" s="13" t="n">
+        <v>0.2058719181702734</v>
+      </c>
+      <c r="G60" s="33" t="n">
+        <v>120.9660532349615</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="52" t="inlineStr">
+        <is>
+          <t>2024-11-04</t>
+        </is>
+      </c>
+      <c r="B61" s="40" t="n">
+        <v>10745</v>
+      </c>
+      <c r="C61" s="30" t="n">
+        <v>131.9299926757812</v>
+      </c>
+      <c r="D61" s="30" t="n">
+        <v>477.4599914550781</v>
+      </c>
+      <c r="E61" s="53" t="n">
+        <v>1.291899561882019</v>
+      </c>
+      <c r="F61" s="13" t="n">
+        <v>0.2142124681611678</v>
+      </c>
+      <c r="G61" s="33" t="n">
+        <v>116.1573947806017</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="52" t="inlineStr">
+        <is>
+          <t>2024-11-11</t>
+        </is>
+      </c>
+      <c r="B62" s="40" t="n">
+        <v>10640</v>
+      </c>
+      <c r="C62" s="30" t="n">
+        <v>128.8500061035156</v>
+      </c>
+      <c r="D62" s="30" t="n">
+        <v>483.8999938964844</v>
+      </c>
+      <c r="E62" s="53" t="n">
+        <v>1.261899709701538</v>
+      </c>
+      <c r="F62" s="13" t="n">
+        <v>0.2163301368463889</v>
+      </c>
+      <c r="G62" s="33" t="n">
+        <v>110.8560831931484</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="52" t="inlineStr">
+        <is>
+          <t>2024-11-18</t>
+        </is>
+      </c>
+      <c r="B63" s="40" t="n">
+        <v>11100</v>
+      </c>
+      <c r="C63" s="30" t="n">
+        <v>135.9900054931641</v>
+      </c>
+      <c r="D63" s="30" t="n">
+        <v>487.6199951171875</v>
+      </c>
+      <c r="E63" s="53" t="n">
+        <v>1.25320041179657</v>
+      </c>
+      <c r="F63" s="13" t="n">
+        <v>0.2204069145261765</v>
+      </c>
+      <c r="G63" s="33" t="n">
+        <v>113.975283209216</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="52" t="inlineStr">
+        <is>
+          <t>2024-11-25</t>
+        </is>
+      </c>
+      <c r="B64" s="40" t="n">
+        <v>11270</v>
+      </c>
+      <c r="C64" s="30" t="n">
+        <v>135.5</v>
+      </c>
+      <c r="D64" s="30" t="n">
+        <v>490.6700134277344</v>
+      </c>
+      <c r="E64" s="53" t="n">
+        <v>1.273899912834167</v>
+      </c>
+      <c r="F64" s="13" t="n">
+        <v>0.2128161062676561</v>
+      </c>
+      <c r="G64" s="33" t="n">
+        <v>116.9010426057044</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="52" t="inlineStr">
+        <is>
+          <t>2024-12-02</t>
+        </is>
+      </c>
+      <c r="B65" s="40" t="n">
+        <v>11365</v>
+      </c>
+      <c r="C65" s="30" t="n">
+        <v>130.8399963378906</v>
+      </c>
+      <c r="D65" s="30" t="n">
+        <v>479.9700012207031</v>
+      </c>
+      <c r="E65" s="53" t="n">
+        <v>1.27459979057312</v>
+      </c>
+      <c r="F65" s="13" t="n">
+        <v>0.2036968727753862</v>
+      </c>
+      <c r="G65" s="33" t="n">
+        <v>120.580718326558</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="52" t="inlineStr">
+        <is>
+          <t>2024-12-09</t>
+        </is>
+      </c>
+      <c r="B66" s="40" t="n">
+        <v>11390</v>
+      </c>
+      <c r="C66" s="30" t="n">
+        <v>131.5</v>
+      </c>
+      <c r="D66" s="30" t="n">
+        <v>488.739990234375</v>
+      </c>
+      <c r="E66" s="53" t="n">
+        <v>1.262500405311584</v>
+      </c>
+      <c r="F66" s="13" t="n">
+        <v>0.2062625260728403</v>
+      </c>
+      <c r="G66" s="33" t="n">
+        <v>117.5509254548532</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="52" t="inlineStr">
+        <is>
+          <t>2024-12-16</t>
+        </is>
+      </c>
+      <c r="B67" s="40" t="n">
+        <v>11320</v>
+      </c>
+      <c r="C67" s="30" t="n">
+        <v>132.7299957275391</v>
+      </c>
+      <c r="D67" s="30" t="n">
+        <v>483.5199890136719</v>
+      </c>
+      <c r="E67" s="53" t="n">
+        <v>1.256799340248108</v>
+      </c>
+      <c r="F67" s="13" t="n">
+        <v>0.2104598501031619</v>
+      </c>
+      <c r="G67" s="33" t="n">
+        <v>117.5564915654933</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="52" t="inlineStr">
+        <is>
+          <t>2024-12-23</t>
+        </is>
+      </c>
+      <c r="B68" s="40" t="n">
+        <v>11330</v>
+      </c>
+      <c r="C68" s="30" t="n">
+        <v>134.9299926757812</v>
+      </c>
+      <c r="D68" s="30" t="n">
+        <v>486.5599975585938</v>
+      </c>
+      <c r="E68" s="53" t="n">
+        <v>1.257300138473511</v>
+      </c>
+      <c r="F68" s="13" t="n">
+        <v>0.2137051053206085</v>
+      </c>
+      <c r="G68" s="33" t="n">
+        <v>116.9717939967624</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="52" t="inlineStr">
+        <is>
+          <t>2024-12-30</t>
+        </is>
+      </c>
+      <c r="B69" s="40" t="n">
+        <v>11420</v>
+      </c>
+      <c r="C69" s="30" t="n">
+        <v>134.4299926757812</v>
+      </c>
+      <c r="D69" s="30" t="n">
+        <v>475.0599975585938</v>
+      </c>
+      <c r="E69" s="53" t="n">
+        <v>1.2423996925354</v>
+      </c>
+      <c r="F69" s="13" t="n">
+        <v>0.2137995296052809</v>
+      </c>
+      <c r="G69" s="33" t="n">
+        <v>119.3239592406978</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="52" t="inlineStr">
+        <is>
+          <t>2025-01-06</t>
+        </is>
+      </c>
+      <c r="B70" s="40" t="n">
+        <v>11675</v>
+      </c>
+      <c r="C70" s="30" t="n">
+        <v>131.0800018310547</v>
+      </c>
+      <c r="D70" s="30" t="n">
+        <v>453.0199890136719</v>
+      </c>
+      <c r="E70" s="53" t="n">
+        <v>1.220899820327759</v>
+      </c>
+      <c r="F70" s="13" t="n">
+        <v>0.2076485586235959</v>
+      </c>
+      <c r="G70" s="33" t="n">
+        <v>125.7095384806853</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="52" t="inlineStr">
+        <is>
+          <t>2025-01-13</t>
+        </is>
+      </c>
+      <c r="B71" s="40" t="n">
+        <v>11770</v>
+      </c>
+      <c r="C71" s="30" t="n">
+        <v>129.0200042724609</v>
+      </c>
+      <c r="D71" s="30" t="n">
+        <v>462.989990234375</v>
+      </c>
+      <c r="E71" s="53" t="n">
+        <v>1.216999530792236</v>
+      </c>
+      <c r="F71" s="13" t="n">
+        <v>0.2035397851546324</v>
+      </c>
+      <c r="G71" s="33" t="n">
+        <v>123.6072515927344</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="52" t="inlineStr">
+        <is>
+          <t>2025-01-20</t>
+        </is>
+      </c>
+      <c r="B72" s="40" t="n">
+        <v>11775</v>
+      </c>
+      <c r="C72" s="30" t="n">
+        <v>131</v>
+      </c>
+      <c r="D72" s="30" t="n">
+        <v>467.1199951171875</v>
+      </c>
+      <c r="E72" s="53" t="n">
+        <v>1.248600006103516</v>
+      </c>
+      <c r="F72" s="13" t="n">
+        <v>0.2015005163970789</v>
+      </c>
+      <c r="G72" s="33" t="n">
+        <v>125.7489793965552</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="52" t="inlineStr">
+        <is>
+          <t>2025-01-27</t>
+        </is>
+      </c>
+      <c r="B73" s="40" t="n">
+        <v>12035</v>
+      </c>
+      <c r="C73" s="30" t="n">
+        <v>126.9000015258789</v>
+      </c>
+      <c r="D73" s="30" t="n">
+        <v>474.4100036621094</v>
+      </c>
+      <c r="E73" s="53" t="n">
+        <v>1.239499926567078</v>
+      </c>
+      <c r="F73" s="13" t="n">
+        <v>0.1925255520900625</v>
+      </c>
+      <c r="G73" s="33" t="n">
+        <v>125.6282875405112</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="52" t="inlineStr">
+        <is>
+          <t>2025-02-03</t>
+        </is>
+      </c>
+      <c r="B74" s="40" t="n">
+        <v>11725</v>
+      </c>
+      <c r="C74" s="30" t="n">
+        <v>124.3499984741211</v>
+      </c>
+      <c r="D74" s="30" t="n">
+        <v>466.7900085449219</v>
+      </c>
+      <c r="E74" s="53" t="n">
+        <v>1.240399360656738</v>
+      </c>
+      <c r="F74" s="13" t="n">
+        <v>0.1936516645651882</v>
+      </c>
+      <c r="G74" s="33" t="n">
+        <v>124.4805537601418</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="52" t="inlineStr">
+        <is>
+          <t>2025-02-10</t>
+        </is>
+      </c>
+      <c r="B75" s="40" t="n">
+        <v>11690</v>
+      </c>
+      <c r="C75" s="30" t="n">
+        <v>127.0299987792969</v>
+      </c>
+      <c r="D75" s="30" t="n">
+        <v>456.0899963378906</v>
+      </c>
+      <c r="E75" s="53" t="n">
+        <v>1.258700728416443</v>
+      </c>
+      <c r="F75" s="13" t="n">
+        <v>0.1956815461459121</v>
+      </c>
+      <c r="G75" s="33" t="n">
+        <v>128.8947195946247</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="52" t="inlineStr">
+        <is>
+          <t>2025-02-17</t>
+        </is>
+      </c>
+      <c r="B76" s="40" t="n">
+        <v>11585</v>
+      </c>
+      <c r="C76" s="30" t="n">
+        <v>134.1499938964844</v>
+      </c>
+      <c r="D76" s="30" t="n">
+        <v>461.7799987792969</v>
+      </c>
+      <c r="E76" s="53" t="n">
+        <v>1.263200521469116</v>
+      </c>
+      <c r="F76" s="13" t="n">
+        <v>0.207938010129241</v>
+      </c>
+      <c r="G76" s="33" t="n">
+        <v>126.614048100671</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="52" t="inlineStr">
+        <is>
+          <t>2025-02-24</t>
+        </is>
+      </c>
+      <c r="B77" s="40" t="n">
+        <v>11845</v>
+      </c>
+      <c r="C77" s="30" t="n">
+        <v>135.3699951171875</v>
+      </c>
+      <c r="D77" s="30" t="n">
+        <v>461.739990234375</v>
+      </c>
+      <c r="E77" s="53" t="n">
+        <v>1.257399797439575</v>
+      </c>
+      <c r="F77" s="13" t="n">
+        <v>0.2063273328785049</v>
+      </c>
+      <c r="G77" s="33" t="n">
+        <v>128.8723178934401</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="52" t="inlineStr">
+        <is>
+          <t>2025-03-03</t>
+        </is>
+      </c>
+      <c r="B78" s="40" t="n">
+        <v>10830</v>
+      </c>
+      <c r="C78" s="30" t="n">
+        <v>133.2299957275391</v>
+      </c>
+      <c r="D78" s="30" t="n">
+        <v>440.7300109863281</v>
+      </c>
+      <c r="E78" s="53" t="n">
+        <v>1.29050076007843</v>
+      </c>
+      <c r="F78" s="13" t="n">
+        <v>0.2165656577965285</v>
+      </c>
+      <c r="G78" s="33" t="n">
+        <v>126.6959624857946</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="52" t="inlineStr">
+        <is>
+          <t>2025-03-10</t>
+        </is>
+      </c>
+      <c r="B79" s="40" t="n">
+        <v>10985</v>
+      </c>
+      <c r="C79" s="30" t="n">
+        <v>135.8000030517578</v>
+      </c>
+      <c r="D79" s="30" t="n">
+        <v>436.8500061035156</v>
+      </c>
+      <c r="E79" s="53" t="n">
+        <v>1.294399499893188</v>
+      </c>
+      <c r="F79" s="13" t="n">
+        <v>0.2171387960644936</v>
+      </c>
+      <c r="G79" s="33" t="n">
+        <v>130.0423262475085</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="52" t="inlineStr">
+        <is>
+          <t>2025-03-17</t>
+        </is>
+      </c>
+      <c r="B80" s="40" t="n">
+        <v>11235</v>
+      </c>
+      <c r="C80" s="30" t="n">
+        <v>142.4100036621094</v>
+      </c>
+      <c r="D80" s="30" t="n">
+        <v>432.8599853515625</v>
+      </c>
+      <c r="E80" s="53" t="n">
+        <v>1.291999578475952</v>
+      </c>
+      <c r="F80" s="13" t="n">
+        <v>0.2232251345394195</v>
+      </c>
+      <c r="G80" s="33" t="n">
+        <v>133.9789859517326</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="52" t="inlineStr">
+        <is>
+          <t>2025-03-30</t>
+        </is>
+      </c>
+      <c r="B81" s="40" t="n">
+        <v>11145</v>
+      </c>
+      <c r="C81" s="30" t="n">
+        <v>146.7700042724609</v>
+      </c>
+      <c r="D81" s="30" t="n">
+        <v>448.760009765625</v>
+      </c>
+      <c r="E81" s="53" t="n">
+        <v>1.287999153137207</v>
+      </c>
+      <c r="F81" s="13" t="n">
+        <v>0.2329683632164831</v>
+      </c>
+      <c r="G81" s="33" t="n">
+        <v>127.7998015955345</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="52" t="inlineStr">
+        <is>
+          <t>2025-04-06</t>
+        </is>
+      </c>
+      <c r="B82" s="40" t="n">
+        <v>11165</v>
+      </c>
+      <c r="C82" s="30" t="n">
+        <v>130.6000061035156</v>
+      </c>
+      <c r="D82" s="30" t="n">
+        <v>416.1900024414062</v>
+      </c>
+      <c r="E82" s="53" t="n">
+        <v>1.308299422264099</v>
+      </c>
+      <c r="F82" s="13" t="n">
+        <v>0.2038756411153908</v>
+      </c>
+      <c r="G82" s="33" t="n">
+        <v>140.2241808240387</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="52" t="inlineStr">
+        <is>
+          <t>2025-04-13</t>
+        </is>
+      </c>
+      <c r="B83" s="40" t="n">
+        <v>11360</v>
+      </c>
+      <c r="C83" s="30" t="n">
+        <v>128.0800018310547</v>
+      </c>
+      <c r="D83" s="30" t="n">
+        <v>425.4400024414062</v>
+      </c>
+      <c r="E83" s="53" t="n">
+        <v>1.323398947715759</v>
+      </c>
+      <c r="F83" s="13" t="n">
+        <v>0.1944165405780942</v>
+      </c>
+      <c r="G83" s="33" t="n">
+        <v>141.1820462005384</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="52" t="inlineStr">
+        <is>
+          <t>2025-04-20</t>
+        </is>
+      </c>
+      <c r="B84" s="40" t="n">
+        <v>11440</v>
+      </c>
+      <c r="C84" s="30" t="n">
+        <v>134.3800048828125</v>
+      </c>
+      <c r="D84" s="30" t="n">
+        <v>427.0499877929688</v>
+      </c>
+      <c r="E84" s="53" t="n">
+        <v>1.331400156021118</v>
+      </c>
+      <c r="F84" s="13" t="n">
+        <v>0.2014903564595063</v>
+      </c>
+      <c r="G84" s="33" t="n">
+        <v>142.4966295882045</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="52" t="inlineStr">
+        <is>
+          <t>2025-04-27</t>
+        </is>
+      </c>
+      <c r="B85" s="40" t="n">
+        <v>11565</v>
+      </c>
+      <c r="C85" s="30" t="n">
+        <v>135.2899932861328</v>
+      </c>
+      <c r="D85" s="30" t="n">
+        <v>424.4700012207031</v>
+      </c>
+      <c r="E85" s="53" t="n">
+        <v>1.326800227165222</v>
+      </c>
+      <c r="F85" s="13" t="n">
+        <v>0.2015126135547262</v>
+      </c>
+      <c r="G85" s="33" t="n">
+        <v>144.4284830631806</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="52" t="inlineStr">
+        <is>
+          <t>2025-05-04</t>
+        </is>
+      </c>
+      <c r="B86" s="40" t="n">
+        <v>11300</v>
+      </c>
+      <c r="C86" s="30" t="n">
+        <v>141.8600006103516</v>
+      </c>
+      <c r="D86" s="30" t="n">
+        <v>434.5599975585938</v>
+      </c>
+      <c r="E86" s="53" t="n">
+        <v>1.329999446868896</v>
+      </c>
+      <c r="F86" s="13" t="n">
+        <v>0.2158994514123574</v>
+      </c>
+      <c r="G86" s="33" t="n">
+        <v>138.1747972883678</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="52" t="inlineStr">
+        <is>
+          <t>2025-05-11</t>
+        </is>
+      </c>
+      <c r="B87" s="40" t="n">
+        <v>11520</v>
+      </c>
+      <c r="C87" s="30" t="n">
+        <v>147.4600067138672</v>
+      </c>
+      <c r="D87" s="30" t="n">
+        <v>454.6199951171875</v>
+      </c>
+      <c r="E87" s="53" t="n">
+        <v>1.32819938659668</v>
+      </c>
+      <c r="F87" s="13" t="n">
+        <v>0.2206043070740309</v>
+      </c>
+      <c r="G87" s="33" t="n">
+        <v>134.4670569138105</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="52" t="inlineStr">
+        <is>
+          <t>2025-05-18</t>
+        </is>
+      </c>
+      <c r="B88" s="40" t="n">
+        <v>11530</v>
+      </c>
+      <c r="C88" s="30" t="n">
+        <v>145.1699981689453</v>
+      </c>
+      <c r="D88" s="30" t="n">
+        <v>473.3200073242188</v>
+      </c>
+      <c r="E88" s="53" t="n">
+        <v>1.353700160980225</v>
+      </c>
+      <c r="F88" s="13" t="n">
+        <v>0.2130663372561966</v>
+      </c>
+      <c r="G88" s="33" t="n">
+        <v>131.7484769655509</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="52" t="inlineStr">
+        <is>
+          <t>2025-05-25</t>
+        </is>
+      </c>
+      <c r="B89" s="40" t="n">
+        <v>11275</v>
+      </c>
+      <c r="C89" s="30" t="n">
+        <v>145.6199951171875</v>
+      </c>
+      <c r="D89" s="30" t="n">
+        <v>462.7999877929688</v>
+      </c>
+      <c r="E89" s="53" t="n">
+        <v>1.346300959587097</v>
+      </c>
+      <c r="F89" s="13" t="n">
+        <v>0.2199310687190469</v>
+      </c>
+      <c r="G89" s="33" t="n">
+        <v>131.0430658483077</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="52" t="inlineStr">
+        <is>
+          <t>2025-06-01</t>
+        </is>
+      </c>
+      <c r="B90" s="40" t="n">
+        <v>11390</v>
+      </c>
+      <c r="C90" s="30" t="n">
+        <v>144.4499969482422</v>
+      </c>
+      <c r="D90" s="30" t="n">
+        <v>458.260009765625</v>
+      </c>
+      <c r="E90" s="53" t="n">
+        <v>1.352899789810181</v>
+      </c>
+      <c r="F90" s="13" t="n">
+        <v>0.2150736678220579</v>
+      </c>
+      <c r="G90" s="33" t="n">
+        <v>134.3464117774736</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="52" t="inlineStr">
+        <is>
+          <t>2025-06-08</t>
+        </is>
+      </c>
+      <c r="B91" s="40" t="n">
+        <v>11045</v>
+      </c>
+      <c r="C91" s="30" t="n">
+        <v>140.0500030517578</v>
+      </c>
+      <c r="D91" s="30" t="n">
+        <v>432.3500061035156</v>
+      </c>
+      <c r="E91" s="53" t="n">
+        <v>1.355700612068176</v>
+      </c>
+      <c r="F91" s="13" t="n">
+        <v>0.2147571866679035</v>
+      </c>
+      <c r="G91" s="33" t="n">
+        <v>138.3702485335137</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="52" t="inlineStr">
+        <is>
+          <t>2025-06-15</t>
+        </is>
+      </c>
+      <c r="B92" s="40" t="n">
+        <v>10835</v>
+      </c>
+      <c r="C92" s="30" t="n">
+        <v>137.2599945068359</v>
+      </c>
+      <c r="D92" s="30" t="n">
+        <v>419.8999938964844</v>
+      </c>
+      <c r="E92" s="53" t="n">
+        <v>1.345699429512024</v>
+      </c>
+      <c r="F92" s="13" t="n">
+        <v>0.2163198561573894</v>
+      </c>
+      <c r="G92" s="33" t="n">
+        <v>138.733005128917</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="52" t="inlineStr">
+        <is>
+          <t>2025-06-22</t>
+        </is>
+      </c>
+      <c r="B93" s="40" t="n">
+        <v>10700</v>
+      </c>
+      <c r="C93" s="30" t="n">
+        <v>139.3399963378906</v>
+      </c>
+      <c r="D93" s="30" t="n">
+        <v>422.3399963378906</v>
+      </c>
+      <c r="E93" s="53" t="n">
+        <v>1.355000734329224</v>
+      </c>
+      <c r="F93" s="13" t="n">
+        <v>0.2210128039103855</v>
+      </c>
+      <c r="G93" s="33" t="n">
+        <v>137.1544094545164</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="52" t="inlineStr">
+        <is>
+          <t>2025-06-29</t>
+        </is>
+      </c>
+      <c r="B94" s="40" t="n">
+        <v>10700</v>
+      </c>
+      <c r="C94" s="30" t="n">
+        <v>144.9299926757812</v>
+      </c>
+      <c r="D94" s="30" t="n">
+        <v>441.4299926757812</v>
+      </c>
+      <c r="E94" s="53" t="n">
+        <v>1.365700483322144</v>
+      </c>
+      <c r="F94" s="13" t="n">
+        <v>0.2282547333479397</v>
+      </c>
+      <c r="G94" s="33" t="n">
+        <v>132.2592577908576</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="52" t="inlineStr">
+        <is>
+          <t>2025-07-06</t>
+        </is>
+      </c>
+      <c r="B95" s="40" t="n">
+        <v>10740</v>
+      </c>
+      <c r="C95" s="30" t="n">
+        <v>138.9799957275391</v>
+      </c>
+      <c r="D95" s="30" t="n">
+        <v>447.9400024414062</v>
+      </c>
+      <c r="E95" s="53" t="n">
+        <v>1.349899291992188</v>
+      </c>
+      <c r="F95" s="13" t="n">
+        <v>0.2207920749155741</v>
+      </c>
+      <c r="G95" s="33" t="n">
+        <v>129.3107054518393</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="52" t="inlineStr">
+        <is>
+          <t>2025-07-13</t>
+        </is>
+      </c>
+      <c r="B96" s="40" t="n">
+        <v>10830</v>
+      </c>
+      <c r="C96" s="30" t="n">
+        <v>136.0700073242188</v>
+      </c>
+      <c r="D96" s="30" t="n">
+        <v>446.2099914550781</v>
+      </c>
+      <c r="E96" s="53" t="n">
+        <v>1.341399550437927</v>
+      </c>
+      <c r="F96" s="13" t="n">
+        <v>0.2158981733965213</v>
+      </c>
+      <c r="G96" s="33" t="n">
+        <v>130.075648712464</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="52" t="inlineStr">
+        <is>
+          <t>2025-07-20</t>
+        </is>
+      </c>
+      <c r="B97" s="40" t="n">
+        <v>10090</v>
+      </c>
+      <c r="C97" s="30" t="n">
+        <v>138.0050048828125</v>
+      </c>
+      <c r="D97" s="30" t="n">
+        <v>432.3200073242188</v>
+      </c>
+      <c r="E97" s="53" t="n">
+        <v>1.354400634765625</v>
+      </c>
+      <c r="F97" s="13" t="n">
+        <v>0.2329519180705937</v>
+      </c>
+      <c r="G97" s="33" t="n">
+        <v>126.2936916877147</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="52" t="inlineStr">
+        <is>
+          <t>2025-07-27</t>
+        </is>
+      </c>
+      <c r="B98" s="40" t="n">
+        <v>9314</v>
+      </c>
+      <c r="C98" s="30" t="n">
+        <v>139.0099945068359</v>
+      </c>
+      <c r="D98" s="30" t="n">
+        <v>419.5400085449219</v>
+      </c>
+      <c r="E98" s="53" t="n">
+        <v>1.328299999237061</v>
+      </c>
+      <c r="F98" s="13" t="n">
+        <v>0.2593941908891705</v>
+      </c>
+      <c r="G98" s="33" t="n">
+        <v>117.8169298408125</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="52" t="inlineStr">
+        <is>
+          <t>2025-08-03</t>
+        </is>
+      </c>
+      <c r="B99" s="40" t="n">
+        <v>9962</v>
+      </c>
+      <c r="C99" s="30" t="n">
+        <v>137.0399932861328</v>
+      </c>
+      <c r="D99" s="30" t="n">
+        <v>391.3299865722656</v>
+      </c>
+      <c r="E99" s="53" t="n">
+        <v>1.343199610710144</v>
+      </c>
+      <c r="F99" s="13" t="n">
+        <v>0.236615929055984</v>
+      </c>
+      <c r="G99" s="33" t="n">
+        <v>136.6131938601823</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="52" t="inlineStr">
+        <is>
+          <t>2025-08-10</t>
+        </is>
+      </c>
+      <c r="B100" s="40" t="n">
+        <v>9262</v>
+      </c>
+      <c r="C100" s="30" t="n">
+        <v>135.4400024414062</v>
+      </c>
+      <c r="D100" s="30" t="n">
+        <v>382.4299926757812</v>
+      </c>
+      <c r="E100" s="53" t="n">
+        <v>1.356099486351013</v>
+      </c>
+      <c r="F100" s="13" t="n">
+        <v>0.2493283994933432</v>
+      </c>
+      <c r="G100" s="33" t="n">
+        <v>131.2178933526745</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="52" t="inlineStr">
+        <is>
+          <t>2025-08-17</t>
+        </is>
+      </c>
+      <c r="B101" s="40" t="n">
+        <v>9464</v>
+      </c>
+      <c r="C101" s="30" t="n">
+        <v>130.1999969482422</v>
+      </c>
+      <c r="D101" s="30" t="n">
+        <v>369.6199951171875</v>
+      </c>
+      <c r="E101" s="53" t="n">
+        <v>1.341899991035461</v>
+      </c>
+      <c r="F101" s="13" t="n">
+        <v>0.2372328680965974</v>
+      </c>
+      <c r="G101" s="33" t="n">
+        <v>137.2739412308798</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="52" t="inlineStr">
+        <is>
+          <t>2025-08-24</t>
+        </is>
+      </c>
+      <c r="B102" s="40" t="n">
+        <v>9168</v>
+      </c>
+      <c r="C102" s="30" t="n">
+        <v>127.9899978637695</v>
+      </c>
+      <c r="D102" s="30" t="n">
+        <v>381.6199951171875</v>
+      </c>
+      <c r="E102" s="53" t="n">
+        <v>1.328499317169189</v>
+      </c>
+      <c r="F102" s="13" t="n">
+        <v>0.2433530333072172</v>
+      </c>
+      <c r="G102" s="33" t="n">
+        <v>127.5127161070843</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="52" t="inlineStr">
+        <is>
+          <t>2025-08-31</t>
+        </is>
+      </c>
+      <c r="B103" s="40" t="n">
+        <v>9270</v>
+      </c>
+      <c r="C103" s="30" t="n">
+        <v>123.3600006103516</v>
+      </c>
+      <c r="D103" s="30" t="n">
+        <v>373.3200073242188</v>
+      </c>
+      <c r="E103" s="53" t="n">
+        <v>1.350900411605835</v>
+      </c>
+      <c r="F103" s="13" t="n">
+        <v>0.2283001176938215</v>
+      </c>
+      <c r="G103" s="33" t="n">
+        <v>134.0202675446231</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="52" t="inlineStr">
+        <is>
+          <t>2025-09-07</t>
+        </is>
+      </c>
+      <c r="B104" s="40" t="n">
+        <v>8632</v>
+      </c>
+      <c r="C104" s="30" t="n">
+        <v>119.0899963378906</v>
+      </c>
+      <c r="D104" s="30" t="n">
+        <v>371.010009765625</v>
+      </c>
+      <c r="E104" s="53" t="n">
+        <v>1.355799794197083</v>
+      </c>
+      <c r="F104" s="13" t="n">
+        <v>0.2360160616933124</v>
+      </c>
+      <c r="G104" s="33" t="n">
+        <v>126.0288712154725</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="52" t="inlineStr">
+        <is>
+          <t>2025-09-14</t>
+        </is>
+      </c>
+      <c r="B105" s="40" t="n">
+        <v>8138</v>
+      </c>
+      <c r="C105" s="30" t="n">
+        <v>117.9199981689453</v>
+      </c>
+      <c r="D105" s="30" t="n">
+        <v>361.8399963378906</v>
+      </c>
+      <c r="E105" s="53" t="n">
+        <v>1.35560131072998</v>
+      </c>
+      <c r="F105" s="13" t="n">
+        <v>0.2481131409445767</v>
+      </c>
+      <c r="G105" s="33" t="n">
+        <v>121.809671889556</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="52" t="inlineStr">
+        <is>
+          <t>2025-09-21</t>
+        </is>
+      </c>
+      <c r="B106" s="40" t="n">
+        <v>8300</v>
+      </c>
+      <c r="C106" s="30" t="n">
+        <v>112.0800018310547</v>
+      </c>
+      <c r="D106" s="30" t="n">
+        <v>289.1499938964844</v>
+      </c>
+      <c r="E106" s="53" t="n">
+        <v>1.343199610710144</v>
+      </c>
+      <c r="F106" s="13" t="n">
+        <v>0.2335395335342465</v>
+      </c>
+      <c r="G106" s="33" t="n">
+        <v>154.0437705172178</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="52" t="inlineStr">
+        <is>
+          <t>2025-09-28</t>
+        </is>
+      </c>
+      <c r="B107" s="40" t="n">
+        <v>8606</v>
+      </c>
+      <c r="C107" s="30" t="n">
+        <v>110.9800033569336</v>
+      </c>
+      <c r="D107" s="30" t="n">
+        <v>289.6900024414062</v>
+      </c>
+      <c r="E107" s="53" t="n">
+        <v>1.35710072517395</v>
+      </c>
+      <c r="F107" s="13" t="n">
+        <v>0.2209130964187513</v>
+      </c>
+      <c r="G107" s="33" t="n">
+        <v>161.0751687446185</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="52" t="inlineStr">
+        <is>
+          <t>2025-10-05</t>
+        </is>
+      </c>
+      <c r="B108" s="40" t="n">
+        <v>8780</v>
+      </c>
+      <c r="C108" s="30" t="n">
+        <v>109.9800033569336</v>
+      </c>
+      <c r="D108" s="30" t="n">
+        <v>282.3299865722656</v>
+      </c>
+      <c r="E108" s="53" t="n">
+        <v>1.335400462150574</v>
+      </c>
+      <c r="F108" s="13" t="n">
+        <v>0.2182414981739703</v>
+      </c>
+      <c r="G108" s="33" t="n">
+        <v>165.9196063731266</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="52" t="inlineStr">
+        <is>
+          <t>2025-10-12</t>
+        </is>
+      </c>
+      <c r="B109" s="40" t="n">
+        <v>8534</v>
+      </c>
+      <c r="C109" s="30" t="n">
+        <v>107.0899963378906</v>
+      </c>
+      <c r="D109" s="30" t="n">
+        <v>283.1300048828125</v>
+      </c>
+      <c r="E109" s="53" t="n">
+        <v>1.337499260902405</v>
+      </c>
+      <c r="F109" s="13" t="n">
+        <v>0.2184600929181141</v>
+      </c>
+      <c r="G109" s="33" t="n">
+        <v>161.0678905421233</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="52" t="inlineStr">
+        <is>
+          <t>2025-10-19</t>
+        </is>
+      </c>
+      <c r="B110" s="40" t="n">
+        <v>9796</v>
+      </c>
+      <c r="C110" s="30" t="n">
+        <v>106.9199981689453</v>
+      </c>
+      <c r="D110" s="30" t="n">
+        <v>286.6700134277344</v>
+      </c>
+      <c r="E110" s="53" t="n">
+        <v>1.330700397491455</v>
+      </c>
+      <c r="F110" s="13" t="n">
+        <v>0.1911345951003985</v>
+      </c>
+      <c r="G110" s="33" t="n">
+        <v>181.6751278095344</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="52" t="inlineStr">
+        <is>
+          <t>2025-10-27</t>
+        </is>
+      </c>
+      <c r="B111" s="40" t="n">
+        <v>9486</v>
+      </c>
+      <c r="C111" s="30" t="n">
+        <v>105.3899993896484</v>
+      </c>
+      <c r="D111" s="30" t="n">
+        <v>266.7999877929688</v>
+      </c>
+      <c r="E111" s="53" t="n">
+        <v>1.315600752830505</v>
+      </c>
+      <c r="F111" s="13" t="n">
+        <v>0.1969656584269967</v>
+      </c>
+      <c r="G111" s="33" t="n">
+        <v>186.8831330686907</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="52" t="inlineStr">
+        <is>
+          <t>2025-11-03</t>
+        </is>
+      </c>
+      <c r="B112" s="40" t="n">
+        <v>9270</v>
+      </c>
+      <c r="C112" s="30" t="n">
+        <v>109.1100006103516</v>
+      </c>
+      <c r="D112" s="30" t="n">
+        <v>262.6000061035156</v>
+      </c>
+      <c r="E112" s="53" t="n">
+        <v>1.316000819206238</v>
+      </c>
+      <c r="F112" s="13" t="n">
+        <v>0.2087697645464585</v>
+      </c>
+      <c r="G112" s="33" t="n">
+        <v>185.6050720378119</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="52" t="inlineStr">
+        <is>
+          <t>2025-11-10</t>
+        </is>
+      </c>
+      <c r="B113" s="40" t="n">
+        <v>8764</v>
+      </c>
+      <c r="C113" s="30" t="n">
+        <v>109.5199966430664</v>
+      </c>
+      <c r="D113" s="30" t="n">
+        <v>273.9100036621094</v>
+      </c>
+      <c r="E113" s="53" t="n">
+        <v>1.315199375152588</v>
+      </c>
+      <c r="F113" s="13" t="n">
+        <v>0.2219623205129883</v>
+      </c>
+      <c r="G113" s="33" t="n">
+        <v>168.1259483713624</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="52" t="inlineStr">
+        <is>
+          <t>2025-11-17</t>
+        </is>
+      </c>
+      <c r="B114" s="40" t="n">
+        <v>8602</v>
+      </c>
+      <c r="C114" s="30" t="n">
+        <v>106.4599990844727</v>
+      </c>
+      <c r="D114" s="30" t="n">
+        <v>277.0199890136719</v>
+      </c>
+      <c r="E114" s="53" t="n">
+        <v>1.308099150657654</v>
+      </c>
+      <c r="F114" s="13" t="n">
+        <v>0.2211909133193269</v>
+      </c>
+      <c r="G114" s="33" t="n">
+        <v>162.2847356030948</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="52" t="inlineStr">
+        <is>
+          <t>2025-11-24</t>
+        </is>
+      </c>
+      <c r="B115" s="40" t="n">
+        <v>8908</v>
+      </c>
+      <c r="C115" s="30" t="n">
+        <v>108.8600006103516</v>
+      </c>
+      <c r="D115" s="30" t="n">
+        <v>277.2699890136719</v>
+      </c>
+      <c r="E115" s="53" t="n">
+        <v>1.325300216674805</v>
+      </c>
+      <c r="F115" s="13" t="n">
+        <v>0.2157427335470599</v>
+      </c>
+      <c r="G115" s="33" t="n">
+        <v>170.1140915358526</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="52" t="inlineStr">
+        <is>
+          <t>2025-12-01</t>
+        </is>
+      </c>
+      <c r="B116" s="40" t="n">
+        <v>8652</v>
+      </c>
+      <c r="C116" s="30" t="n">
+        <v>107.7699966430664</v>
+      </c>
+      <c r="D116" s="30" t="n">
+        <v>290.6300048828125</v>
+      </c>
+      <c r="E116" s="53" t="n">
+        <v>1.334600329399109</v>
+      </c>
+      <c r="F116" s="13" t="n">
+        <v>0.2185415997528903</v>
+      </c>
+      <c r="G116" s="33" t="n">
+        <v>158.7361955774925</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="52" t="inlineStr">
+        <is>
+          <t>2025-12-08</t>
+        </is>
+      </c>
+      <c r="B117" s="40" t="n">
+        <v>8464</v>
+      </c>
+      <c r="C117" s="30" t="n">
+        <v>107.1699981689453</v>
+      </c>
+      <c r="D117" s="30" t="n">
+        <v>292.4700012207031</v>
+      </c>
+      <c r="E117" s="53" t="n">
+        <v>1.337300658226013</v>
+      </c>
+      <c r="F117" s="13" t="n">
+        <v>0.2218780963880284</v>
+      </c>
+      <c r="G117" s="33" t="n">
+        <v>154.6222769113599</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="52" t="inlineStr">
+        <is>
+          <t>2025-12-15</t>
+        </is>
+      </c>
+      <c r="B118" s="40" t="n">
+        <v>8918</v>
+      </c>
+      <c r="C118" s="30" t="n">
+        <v>104.5199966430664</v>
+      </c>
+      <c r="D118" s="30" t="n">
+        <v>288.5400085449219</v>
+      </c>
+      <c r="E118" s="53" t="n">
+        <v>1.329599857330322</v>
+      </c>
+      <c r="F118" s="13" t="n">
+        <v>0.2067278955299122</v>
+      </c>
+      <c r="G118" s="33" t="n">
+        <v>164.1840882760104</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="52" t="inlineStr">
+        <is>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="B119" s="40" t="n">
+        <v>8874</v>
+      </c>
+      <c r="C119" s="30" t="n">
+        <v>107.8000030517578</v>
+      </c>
+      <c r="D119" s="30" t="n">
+        <v>292.1300048828125</v>
+      </c>
+      <c r="E119" s="53" t="n">
+        <v>1.351700305938721</v>
+      </c>
+      <c r="F119" s="13" t="n">
+        <v>0.2109354307886747</v>
+      </c>
+      <c r="G119" s="33" t="n">
+        <v>164.0485320720614</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="52" t="inlineStr">
+        <is>
+          <t>2025-12-29</t>
+        </is>
+      </c>
+      <c r="B120" s="40" t="n">
+        <v>8804</v>
+      </c>
+      <c r="C120" s="30" t="n">
+        <v>106.1999969482422</v>
+      </c>
+      <c r="D120" s="30" t="n">
+        <v>284.8999938964844</v>
+      </c>
+      <c r="E120" s="53" t="n">
+        <v>1.346799492835999</v>
+      </c>
+      <c r="F120" s="13" t="n">
+        <v>0.2103850460058603</v>
+      </c>
+      <c r="G120" s="33" t="n">
+        <v>166.2796938516103</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="52" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B121" s="40" t="n">
+        <v>8952</v>
+      </c>
+      <c r="C121" s="30" t="n">
+        <v>103.8600006103516</v>
+      </c>
+      <c r="D121" s="30" t="n">
+        <v>294.4500122070312</v>
+      </c>
+      <c r="E121" s="53" t="n">
+        <v>1.340800642967224</v>
+      </c>
+      <c r="F121" s="13" t="n">
+        <v>0.2034997756370419</v>
+      </c>
+      <c r="G121" s="33" t="n">
+        <v>162.8626077857975</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="52" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B122" s="40" t="n">
+        <v>9184</v>
+      </c>
+      <c r="C122" s="30" t="n">
+        <v>106.2600021362305</v>
+      </c>
+      <c r="D122" s="30" t="n">
+        <v>288.6000061035156</v>
+      </c>
+      <c r="E122" s="53" t="n">
+        <v>1.338700652122498</v>
+      </c>
+      <c r="F122" s="13" t="n">
+        <v>0.2035424932597611</v>
+      </c>
+      <c r="G122" s="33" t="n">
+        <v>170.2031886915294</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="52" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B123" s="40" t="n">
+        <v>8768</v>
+      </c>
+      <c r="C123" s="30" t="n">
+        <v>102.8000030517578</v>
+      </c>
+      <c r="D123" s="30" t="n">
+        <v>286.6799926757812</v>
+      </c>
+      <c r="E123" s="53" t="n">
+        <v>1.364600896835327</v>
+      </c>
+      <c r="F123" s="13" t="n">
+        <v>0.2026231714248906</v>
+      </c>
+      <c r="G123" s="33" t="n">
+        <v>166.7467918189795</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="52" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B124" s="40" t="n">
+        <v>8122</v>
+      </c>
+      <c r="C124" s="30" t="n">
+        <v>103.0699996948242</v>
+      </c>
+      <c r="D124" s="30" t="n">
+        <v>254.3600006103516</v>
+      </c>
+      <c r="E124" s="53" t="n">
+        <v>1.369300246238708</v>
+      </c>
+      <c r="F124" s="13" t="n">
+        <v>0.2188644207387715</v>
+      </c>
+      <c r="G124" s="33" t="n">
+        <v>174.6873803744348</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="52" t="inlineStr">
+        <is>
+          <t>2026-02-02</t>
+        </is>
+      </c>
+      <c r="B125" s="40" t="n">
+        <v>7502</v>
+      </c>
+      <c r="C125" s="30" t="n">
+        <v>112.129997253418</v>
+      </c>
+      <c r="D125" s="30" t="n">
+        <v>207.3200073242188</v>
+      </c>
+      <c r="E125" s="53" t="n">
+        <v>1.361700296401978</v>
+      </c>
+      <c r="F125" s="13" t="n">
+        <v>0.2595798692474712</v>
+      </c>
+      <c r="G125" s="33" t="n">
+        <v>196.8638863559729</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="52" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B126" s="40" t="n">
+        <v>7570</v>
+      </c>
+      <c r="C126" s="30" t="n">
+        <v>113.4100036621094</v>
+      </c>
+      <c r="D126" s="30" t="n">
+        <v>205.7899932861328</v>
+      </c>
+      <c r="E126" s="53" t="n">
+        <v>1.362199187278748</v>
+      </c>
+      <c r="F126" s="13" t="n">
+        <v>0.2604514158740433</v>
+      </c>
+      <c r="G126" s="33" t="n">
+        <v>200.1985471421863</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="52" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="B127" s="40" t="n">
+        <v>7904</v>
+      </c>
+      <c r="C127" s="30" t="n">
+        <v>119.4700012207031</v>
+      </c>
+      <c r="D127" s="30" t="n">
+        <v>195.0500030517578</v>
+      </c>
+      <c r="E127" s="53" t="n">
+        <v>1.348099589347839</v>
+      </c>
+      <c r="F127" s="13" t="n">
+        <v>0.2658928879261404</v>
+      </c>
+      <c r="G127" s="33" t="n">
+        <v>218.2587304209341</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="52" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="B128" s="40" t="n">
+        <v>8860</v>
+      </c>
+      <c r="C128" s="30" t="n">
+        <v>123.254997253418</v>
+      </c>
+      <c r="D128" s="30" t="n">
+        <v>216.8099975585938</v>
+      </c>
+      <c r="E128" s="53" t="n">
+        <v>1.34540069103241</v>
+      </c>
+      <c r="F128" s="13" t="n">
+        <v>0.2455509840735687</v>
+      </c>
+      <c r="G128" s="33" t="n">
+        <v>219.661903074769</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="52" t="inlineStr">
+        <is>
+          <t>2026-03-02</t>
+        </is>
+      </c>
+      <c r="B129" s="40" t="n">
+        <v>8792</v>
+      </c>
+      <c r="C129" s="30" t="n">
+        <v>124.5899963378906</v>
+      </c>
+      <c r="D129" s="30" t="n">
+        <v>225.8699951171875</v>
+      </c>
+      <c r="E129" s="53" t="n">
+        <v>1.340800642967224</v>
+      </c>
+      <c r="F129" s="13" t="n">
+        <v>0.2513392941560363</v>
+      </c>
+      <c r="G129" s="33" t="n">
+        <v>208.5172672542023</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="52" t="inlineStr">
+        <is>
+          <t>2026-03-09</t>
+        </is>
+      </c>
+      <c r="B130" s="40" t="n">
+        <v>8746</v>
+      </c>
+      <c r="C130" s="30" t="n">
+        <v>124.4199981689453</v>
+      </c>
+      <c r="D130" s="30" t="n">
+        <v>205.6499938964844</v>
+      </c>
+      <c r="E130" s="53" t="n">
+        <v>1.323800206184387</v>
+      </c>
+      <c r="F130" s="13" t="n">
+        <v>0.2559144594839002</v>
+      </c>
+      <c r="G130" s="33" t="n">
+        <v>224.9323365089381</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="52" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B131" s="40" t="n">
+        <v>8662</v>
+      </c>
+      <c r="C131" s="30" t="n">
+        <v>125.1500015258789</v>
+      </c>
+      <c r="D131" s="30" t="n">
+        <v>209.2700042724609</v>
+      </c>
+      <c r="E131" s="53" t="n">
+        <v>1.33400022983551</v>
+      </c>
+      <c r="F131" s="13" t="n">
+        <v>0.2582864494972917</v>
+      </c>
+      <c r="G131" s="33" t="n">
+        <v>220.6052170289857</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="52" t="inlineStr">
+        <is>
+          <t>2026-03-29</t>
+        </is>
+      </c>
+      <c r="B132" s="40" t="n">
+        <v>8920</v>
+      </c>
+      <c r="C132" s="30" t="n">
+        <v>116.5699996948242</v>
+      </c>
+      <c r="D132" s="30" t="n">
+        <v>198.3300018310547</v>
+      </c>
+      <c r="E132" s="53" t="n">
+        <v>1.322200417518616</v>
+      </c>
+      <c r="F132" s="13" t="n">
+        <v>0.2363205314878838</v>
+      </c>
+      <c r="G132" s="33" t="n">
+        <v>237.5868538256285</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="52" t="inlineStr">
+        <is>
+          <t>2026-04-05</t>
+        </is>
+      </c>
+      <c r="B133" s="40" t="n">
+        <v>8968</v>
+      </c>
+      <c r="C133" s="30" t="n">
+        <v>123.1999969482422</v>
+      </c>
+      <c r="D133" s="30" t="n">
+        <v>227.6799926757812</v>
+      </c>
+      <c r="E133" s="53" t="n">
+        <v>1.345599889755249</v>
+      </c>
+      <c r="F133" s="13" t="n">
+        <v>0.2444481178799553</v>
+      </c>
+      <c r="G133" s="33" t="n">
+        <v>211.7558181809361</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="52" t="inlineStr">
+        <is>
+          <t>2026-04-12</t>
+        </is>
+      </c>
+      <c r="B134" s="40" t="n">
+        <v>9456</v>
+      </c>
+      <c r="C134" s="30" t="n">
+        <v>121.4400024414062</v>
+      </c>
+      <c r="D134" s="30" t="n">
+        <v>211.6000061035156</v>
+      </c>
+      <c r="E134" s="53" t="n">
+        <v>1.352499127388</v>
+      </c>
+      <c r="F134" s="13" t="n">
+        <v>0.2276755806607057</v>
+      </c>
+      <c r="G134" s="33" t="n">
+        <v>241.477938340153</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="52" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B135" s="40" t="n">
+        <v>9992</v>
+      </c>
+      <c r="C135" s="30" t="n">
+        <v>118.3399963378906</v>
+      </c>
+      <c r="D135" s="30" t="n">
+        <v>232.7299957275391</v>
+      </c>
+      <c r="E135" s="53" t="n">
+        <v>1.349700689315796</v>
+      </c>
+      <c r="F135" s="13" t="n">
+        <v>0.210694530234947</v>
+      </c>
+      <c r="G135" s="33" t="n">
+        <v>231.5187727375953</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="52" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B136" s="40" t="n">
+        <v>9624</v>
+      </c>
+      <c r="C136" s="30" t="n">
+        <v>113.2900009155273</v>
+      </c>
+      <c r="D136" s="30" t="n">
+        <v>224.1199951171875</v>
+      </c>
+      <c r="E136" s="53" t="n">
+        <v>1.360399842262268</v>
+      </c>
+      <c r="F136" s="13" t="n">
+        <v>0.2080627454317005</v>
+      </c>
+      <c r="G136" s="33" t="n">
+        <v>233.3943083800185</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="52" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B137" s="40" t="n">
+        <v>9042</v>
+      </c>
+      <c r="C137" s="30" t="n">
+        <v>111.6800003051758</v>
+      </c>
+      <c r="D137" s="30" t="n">
+        <v>227.5800018310547</v>
+      </c>
+      <c r="E137" s="53" t="n">
+        <v>1.363499402999878</v>
+      </c>
+      <c r="F137" s="13" t="n">
+        <v>0.2181197934426317</v>
+      </c>
+      <c r="G137" s="33" t="n">
+        <v>216.4382612329804</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="52" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="B138" s="40" t="n">
+        <v>9132</v>
+      </c>
+      <c r="C138" s="30" t="n">
+        <v>108.8099975585938</v>
+      </c>
+      <c r="D138" s="30" t="n">
+        <v>223.6100006103516</v>
+      </c>
+      <c r="E138" s="53" t="n">
+        <v>1.332999229431152</v>
+      </c>
+      <c r="F138" s="13" t="n">
+        <v>0.2155396581357367</v>
+      </c>
+      <c r="G138" s="33" t="n">
+        <v>217.4969927432508</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="52" t="inlineStr">
+        <is>
+          <t>2026-05-17</t>
+        </is>
+      </c>
+      <c r="B139" s="40" t="n">
+        <v>9326</v>
+      </c>
+      <c r="C139" s="30" t="n">
+        <v>110.9400024414062</v>
+      </c>
+      <c r="D139" s="30" t="n">
+        <v>212.5800018310547</v>
+      </c>
+      <c r="E139" s="53" t="n">
+        <v>1.344100475311279</v>
+      </c>
+      <c r="F139" s="13" t="n">
+        <v>0.2137131040208542</v>
+      </c>
+      <c r="G139" s="33" t="n">
+        <v>235.5881367819547</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="52" t="inlineStr">
+        <is>
+          <t>2026-05-24</t>
+        </is>
+      </c>
+      <c r="B140" s="40" t="n">
+        <v>9022</v>
+      </c>
+      <c r="C140" s="30" t="n">
+        <v>106.1999969482422</v>
+      </c>
+      <c r="D140" s="30" t="n">
+        <v>232</v>
+      </c>
+      <c r="E140" s="53" t="n">
+        <v>1.34540069103241</v>
+      </c>
+      <c r="F140" s="13" t="n">
+        <v>0.2115714065289649</v>
+      </c>
+      <c r="G140" s="33" t="n">
+        <v>209.0331486684324</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="52" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="B141" s="40" t="n">
+        <v>9384</v>
+      </c>
+      <c r="C141" s="30" t="n">
+        <v>100.25</v>
+      </c>
+      <c r="D141" s="30" t="n">
+        <v>245.4700012207031</v>
+      </c>
+      <c r="E141" s="53" t="n">
+        <v>1.334400773048401</v>
+      </c>
+      <c r="F141" s="13" t="n">
+        <v>0.1938718363993848</v>
+      </c>
+      <c r="G141" s="33" t="n">
+        <v>203.8095534022724</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="52" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B142" s="40" t="n">
+        <v>9010</v>
+      </c>
+      <c r="C142" s="30" t="n">
+        <v>102.5299987792969</v>
+      </c>
+      <c r="D142" s="30" t="n">
+        <v>255.6199951171875</v>
+      </c>
+      <c r="E142" s="53" t="n">
+        <v>1.341000318527222</v>
+      </c>
+      <c r="F142" s="13" t="n">
+        <v>0.2057882032630078</v>
+      </c>
+      <c r="G142" s="33" t="n">
+        <v>188.8458858703845</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="52" t="inlineStr">
+        <is>
+          <t>2026-06-14</t>
+        </is>
+      </c>
+      <c r="B143" s="40" t="n">
+        <v>8460</v>
+      </c>
+      <c r="C143" s="30" t="n">
+        <v>101.1900024414062</v>
+      </c>
+      <c r="D143" s="30" t="n">
+        <v>241.1600036621094</v>
+      </c>
+      <c r="E143" s="53" t="n">
+        <v>1.327300310134888</v>
+      </c>
+      <c r="F143" s="13" t="n">
+        <v>0.2188470482231473</v>
+      </c>
+      <c r="G143" s="33" t="n">
+        <v>186.0299867904252</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="52" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B144" s="40" t="n">
+        <v>8062</v>
+      </c>
+      <c r="C144" s="30" t="n">
+        <v>99.48999786376953</v>
+      </c>
+      <c r="D144" s="30" t="n">
+        <v>221.2899932861328</v>
+      </c>
+      <c r="E144" s="53" t="n">
+        <v>1.320199966430664</v>
+      </c>
+      <c r="F144" s="13" t="n">
+        <v>0.2273316434710476</v>
+      </c>
+      <c r="G144" s="33" t="n">
+        <v>192.1628422485122</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="52" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B145" s="40" t="n">
+        <v>8670</v>
+      </c>
+      <c r="C145" s="30" t="n">
+        <v>93.51999664306641</v>
+      </c>
+      <c r="D145" s="30" t="n">
+        <v>231.7400054931641</v>
+      </c>
+      <c r="E145" s="53" t="n">
+        <v>1.339200854301453</v>
+      </c>
+      <c r="F145" s="13" t="n">
+        <v>0.196166060965063</v>
+      </c>
+      <c r="G145" s="33" t="n">
+        <v>200.1762182957983</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="52" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B146" s="40" t="n">
+        <v>8908</v>
+      </c>
+      <c r="C146" s="30" t="n">
+        <v>102.7900009155273</v>
+      </c>
+      <c r="D146" s="30" t="n">
+        <v>250.0899963378906</v>
+      </c>
+      <c r="E146" s="53" t="n">
+        <v>1.340299367904663</v>
+      </c>
+      <c r="F146" s="13" t="n">
+        <v>0.209978662747912</v>
+      </c>
+      <c r="G146" s="33" t="n">
+        <v>190.7367503152862</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="52" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B147" s="40" t="n">
+        <v>8978</v>
+      </c>
+      <c r="C147" s="30" t="n">
+        <v>97.86000061035156</v>
+      </c>
+      <c r="D147" s="30" t="n">
+        <v>247.1100006103516</v>
+      </c>
+      <c r="E147" s="53" t="n">
+        <v>1.344499826431274</v>
+      </c>
+      <c r="F147" s="13" t="n">
+        <v>0.1980132192552568</v>
+      </c>
+      <c r="G147" s="33" t="n">
+        <v>195.1635493787829</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="52" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="B148" s="40" t="n">
+        <v>8774</v>
+      </c>
+      <c r="C148" s="30" t="n">
+        <v>99.90000152587891</v>
+      </c>
+      <c r="D148" s="30" t="n">
+        <v>258.0899963378906</v>
+      </c>
+      <c r="E148" s="53" t="n">
+        <v>1.332100749015808</v>
+      </c>
+      <c r="F148" s="13" t="n">
+        <v>0.2090662908839105</v>
+      </c>
+      <c r="G148" s="33" t="n">
+        <v>180.9306774140697</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="52" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="B149" s="40" t="n">
+        <v>8398</v>
+      </c>
+      <c r="C149" s="30" t="n">
+        <v>99.83000183105469</v>
+      </c>
+      <c r="D149" s="30" t="n">
+        <v>254.3600006103516</v>
+      </c>
+      <c r="E149" s="53" t="n">
+        <v>1.34839940071106</v>
+      </c>
+      <c r="F149" s="13" t="n">
+        <v>0.215945758216057</v>
+      </c>
+      <c r="G149" s="33" t="n">
+        <v>177.8665502290039</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="52" t="inlineStr">
+        <is>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B150" s="40" t="n">
+        <v>8920</v>
+      </c>
+      <c r="C150" s="30" t="n">
+        <v>100.5</v>
+      </c>
+      <c r="D150" s="30" t="n">
+        <v>263.2000122070312</v>
+      </c>
+      <c r="E150" s="53" t="n">
+        <v>1.346799492835999</v>
+      </c>
+      <c r="F150" s="13" t="n">
+        <v>0.2052116351143182</v>
+      </c>
+      <c r="G150" s="33" t="n">
+        <v>182.3604148792122</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="52" t="inlineStr">
+        <is>
+          <t>2026-08-09</t>
+        </is>
+      </c>
+      <c r="B151" s="40" t="n">
+        <v>8536</v>
+      </c>
+      <c r="C151" s="30" t="n">
+        <v>102.620002746582</v>
+      </c>
+      <c r="D151" s="30" t="n">
+        <v>285.5700073242188</v>
+      </c>
+      <c r="E151" s="53" t="n">
+        <v>1.353000521659851</v>
+      </c>
+      <c r="F151" s="13" t="n">
+        <v>0.2182780019428615</v>
+      </c>
+      <c r="G151" s="33" t="n">
+        <v>161.580317023093</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="52" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B152" s="40" t="n">
+        <v>8602</v>
+      </c>
+      <c r="C152" s="30" t="n">
+        <v>106.2900009155273</v>
+      </c>
+      <c r="D152" s="30" t="n">
+        <v>283.489990234375</v>
+      </c>
+      <c r="E152" s="53" t="n">
+        <v>1.364200592041016</v>
+      </c>
+      <c r="F152" s="13" t="n">
+        <v>0.2228294370670036</v>
+      </c>
+      <c r="G152" s="33" t="n">
+        <v>165.3821452344408</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="52" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B153" s="40" t="n">
+        <v>9000</v>
+      </c>
+      <c r="C153" s="30" t="n">
+        <v>107.0400009155273</v>
+      </c>
+      <c r="D153" s="30" t="n">
+        <v>299.9100036621094</v>
+      </c>
+      <c r="E153" s="53" t="n">
+        <v>1.354899644851685</v>
+      </c>
+      <c r="F153" s="13" t="n">
+        <v>0.2162632393848498</v>
+      </c>
+      <c r="G153" s="33" t="n">
+        <v>162.4453799899936</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="52" t="inlineStr">
+        <is>
+          <t>2026-08-30</t>
+        </is>
+      </c>
+      <c r="B154" s="40" t="n">
+        <v>8830</v>
+      </c>
+      <c r="C154" s="30" t="n">
+        <v>108.870002746582</v>
+      </c>
+      <c r="D154" s="30" t="n">
+        <v>308.9800109863281</v>
+      </c>
+      <c r="E154" s="53" t="n">
+        <v>1.359099984169006</v>
+      </c>
+      <c r="F154" s="13" t="n">
+        <v>0.2238265938088625</v>
+      </c>
+      <c r="G154" s="33" t="n">
+        <v>155.1780909784675</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-06</t>
+        </is>
+      </c>
+      <c r="B155" s="40" t="n">
+        <v>8238</v>
+      </c>
+      <c r="C155" s="30" t="n">
+        <v>106.1999969482422</v>
+      </c>
+      <c r="D155" s="30" t="n">
+        <v>301.9599914550781</v>
+      </c>
+      <c r="E155" s="53" t="n">
+        <v>1.353599429130554</v>
+      </c>
+      <c r="F155" s="13" t="n">
+        <v>0.235319737222963</v>
+      </c>
+      <c r="G155" s="33" t="n">
+        <v>147.5404908095569</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="B156" s="40" t="n">
+        <v>8246</v>
+      </c>
+      <c r="C156" s="30" t="n">
+        <v>101.4400024414062</v>
+      </c>
+      <c r="D156" s="30" t="n">
+        <v>259.7099914550781</v>
+      </c>
+      <c r="E156" s="53" t="n">
+        <v>1.33899998664856</v>
+      </c>
+      <c r="F156" s="13" t="n">
+        <v>0.2273329053111093</v>
+      </c>
+      <c r="G156" s="33" t="n">
+        <v>169.8571853715746</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="B157" s="40" t="n">
+        <v>8200</v>
+      </c>
+      <c r="C157" s="30" t="n">
+        <v>103.9700012207031</v>
+      </c>
+      <c r="D157" s="30" t="n">
+        <v>283.8299865722656</v>
+      </c>
+      <c r="E157" s="53" t="n">
+        <v>1.325200080871582</v>
+      </c>
+      <c r="F157" s="13" t="n">
+        <v>0.2370946584185726</v>
+      </c>
+      <c r="G157" s="33" t="n">
+        <v>152.9627586987674</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="52" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="B158" s="40" t="n">
+        <v>8090</v>
+      </c>
+      <c r="C158" s="30" t="n">
+        <v>101.1900024414062</v>
+      </c>
+      <c r="D158" s="30" t="n">
+        <v>273.0799865722656</v>
+      </c>
+      <c r="E158" s="53" t="n">
+        <v>1.324399828910828</v>
+      </c>
+      <c r="F158" s="13" t="n">
+        <v>0.2343753799754173</v>
+      </c>
+      <c r="G158" s="33" t="n">
+        <v>156.7568193359698</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-04</t>
+        </is>
+      </c>
+      <c r="B159" s="40" t="n">
+        <v>8694</v>
+      </c>
+      <c r="C159" s="30" t="n">
+        <v>102.2200012207031</v>
+      </c>
+      <c r="D159" s="30" t="n">
+        <v>266</v>
+      </c>
+      <c r="E159" s="53" t="n">
+        <v>1.324299812316895</v>
+      </c>
+      <c r="F159" s="13" t="n">
+        <v>0.2206509828991645</v>
+      </c>
+      <c r="G159" s="33" t="n">
+        <v>172.9310565324599</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-11</t>
+        </is>
+      </c>
+      <c r="B160" s="40" t="n">
+        <v>8768</v>
+      </c>
+      <c r="C160" s="30" t="n">
+        <v>111.0800018310547</v>
+      </c>
+      <c r="D160" s="30" t="n">
+        <v>287.1799926757812</v>
+      </c>
+      <c r="E160" s="53" t="n">
+        <v>1.329799652099609</v>
+      </c>
+      <c r="F160" s="13" t="n">
+        <v>0.2371154781247387</v>
+      </c>
+      <c r="G160" s="33" t="n">
+        <v>162.2113557651295</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B161" s="40" t="n">
+        <v>9510</v>
+      </c>
+      <c r="C161" s="30" t="n">
+        <v>113.4899978637695</v>
+      </c>
+      <c r="D161" s="30" t="n">
+        <v>301.6700134277344</v>
+      </c>
+      <c r="E161" s="53" t="n">
+        <v>1.340392708778381</v>
+      </c>
+      <c r="F161" s="13" t="n">
+        <v>0.2219175094995671</v>
+      </c>
+      <c r="G161" s="33" t="n">
+        <v>168.8220265236977</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="52" t="inlineStr">
+        <is>
+          <t>2026-10-23</t>
+        </is>
+      </c>
+      <c r="B162" s="40" t="n">
+        <v>9510</v>
+      </c>
+      <c r="C162" s="30" t="n">
+        <v>122.5699996948242</v>
+      </c>
+      <c r="D162" s="30" t="n">
+        <v>331.3200073242188</v>
+      </c>
+      <c r="E162" s="53" t="n">
+        <v>1.337399005889893</v>
+      </c>
+      <c r="F162" s="13" t="n">
+        <v>0.24046059766849</v>
+      </c>
+      <c r="G162" s="33" t="n">
+        <v>153.3707455767087</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Tradeweb share count held at the latest 10-Q; LSEG share count interpolated between disclosed points. Prices: Yahoo Finance chart endpoint.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1828,7 +6342,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2231,7 +6745,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2297,13 +6811,13 @@
           <t>Revenue retention</t>
         </is>
       </c>
-      <c r="B5" s="51" t="n">
+      <c r="B5" s="54" t="n">
         <v>0.928</v>
       </c>
-      <c r="C5" s="51" t="n">
+      <c r="C5" s="54" t="n">
         <v>0.9131487262864029</v>
       </c>
-      <c r="D5" s="51" t="n">
+      <c r="D5" s="54" t="n">
         <v>-0.01485127371359712</v>
       </c>
       <c r="E5" t="inlineStr">
@@ -2318,13 +6832,13 @@
           <t>Markets volume growth, all drivers (shown on 2028 ADV growth)</t>
         </is>
       </c>
-      <c r="B6" s="51" t="n">
+      <c r="B6" s="54" t="n">
         <v>0.05</v>
       </c>
-      <c r="C6" s="51" t="n">
+      <c r="C6" s="54" t="n">
         <v>0.02734297461659459</v>
       </c>
-      <c r="D6" s="51" t="n">
+      <c r="D6" s="54" t="n">
         <v>-0.02265702538340542</v>
       </c>
       <c r="E6" t="inlineStr">
@@ -2339,13 +6853,13 @@
           <t>Divisional margin change per year</t>
         </is>
       </c>
-      <c r="B7" s="51" t="n">
+      <c r="B7" s="54" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="51" t="n">
+      <c r="C7" s="54" t="n">
         <v>-0.00319678945687564</v>
       </c>
-      <c r="D7" s="51" t="n">
+      <c r="D7" s="54" t="n">
         <v>-0.00319678945687564</v>
       </c>
       <c r="E7" t="inlineStr">
@@ -2360,13 +6874,13 @@
           <t>Terminal growth</t>
         </is>
       </c>
-      <c r="B8" s="51" t="n">
+      <c r="B8" s="54" t="n">
         <v>0.03</v>
       </c>
-      <c r="C8" s="51" t="n">
+      <c r="C8" s="54" t="n">
         <v>0.02831755048183757</v>
       </c>
-      <c r="D8" s="51" t="n">
+      <c r="D8" s="54" t="n">
         <v>-0.001682449518162425</v>
       </c>
       <c r="E8" t="inlineStr">
@@ -2388,25 +6902,25 @@
           <t>Retention (2027–2030)</t>
         </is>
       </c>
-      <c r="B12" s="51" t="n">
+      <c r="B12" s="54" t="n">
         <v>0.88</v>
       </c>
-      <c r="C12" s="51" t="n">
+      <c r="C12" s="54" t="n">
         <v>0.89</v>
       </c>
-      <c r="D12" s="51" t="n">
+      <c r="D12" s="54" t="n">
         <v>0.9</v>
       </c>
-      <c r="E12" s="51" t="n">
+      <c r="E12" s="54" t="n">
         <v>0.91</v>
       </c>
-      <c r="F12" s="51" t="n">
+      <c r="F12" s="54" t="n">
         <v>0.92</v>
       </c>
-      <c r="G12" s="51" t="n">
+      <c r="G12" s="54" t="n">
         <v>0.928</v>
       </c>
-      <c r="H12" s="51" t="n">
+      <c r="H12" s="54" t="n">
         <v>0.9350000000000001</v>
       </c>
     </row>
@@ -2443,7 +6957,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2688,7 +7202,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2703,14 +7217,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Trade expression: long LSEG / short FactSet</t>
+          <t>Trade expression: long LSEG / short FactSet (considered and rejected)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Isolates the 'market prices LSEG like FactSet' view and removes most market and sector beta.</t>
+          <t>Would isolate the AI-discount view and remove market beta. See the read below for why the outright long is preferred.</t>
         </is>
       </c>
     </row>
@@ -2800,14 +7314,14 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Read: LSEG trades only c.9% above FactSet although over half its income is exchange, index and risk-data revenue.</t>
+          <t>Read: the pair has already worked. Since Jan 2024 LSEG has beaten FactSet by c.53% in GBP (Trackers sheet), and FactSet ASV grew 7% with retention above 95%.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Risk: FactSet short interest is c.9% of float, a crowded short. Size small and set a stop on the price ratio.</t>
+          <t>Conclusion: prefer the outright long. FactSet short interest is c.9% of float, so the short leg carries squeeze risk with little valuation support left.</t>
         </is>
       </c>
     </row>
@@ -2816,7 +7330,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>